<commit_message>
Actualizacion automatica 01/06/2026 11:03 (Buenos Aires)
</commit_message>
<xml_diff>
--- a/Master UOPs.xlsx
+++ b/Master UOPs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365iebc-my.sharepoint.com/personal/mperez_iebc_com_ar/Documents/Seguimiento Obras/Reporte de Obras/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{06376EE1-B0DD-45EC-BF0E-FB21B357E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F137C80E-0B78-4223-BB7C-5BC7760D3CBF}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{06376EE1-B0DD-45EC-BF0E-FB21B357E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{988BB022-ABC9-4C4A-A239-9F0A36E77166}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{0B067436-489C-4F7D-A3D3-1998983265A1}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B067436-489C-4F7D-A3D3-1998983265A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="5" r:id="rId1"/>
@@ -260,7 +260,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2110" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2106" uniqueCount="368">
   <si>
     <t>UOP</t>
   </si>
@@ -9875,7 +9875,7 @@
         <v>29760318.289999999</v>
       </c>
       <c r="AJ66" s="94">
-        <f t="shared" ref="AJ66:AJ94" si="25">+AA66-AI66</f>
+        <f t="shared" ref="AJ66:AJ93" si="25">+AA66-AI66</f>
         <v>-7.429998368024826E-3</v>
       </c>
       <c r="AK66" s="90">
@@ -13039,7 +13039,7 @@
         <v>0</v>
       </c>
       <c r="AJ97" s="94">
-        <f t="shared" ref="AJ96:AJ108" si="35">+AA97-AI97</f>
+        <f t="shared" ref="AJ97:AJ108" si="35">+AA97-AI97</f>
         <v>0</v>
       </c>
       <c r="AK97" s="90" t="str">
@@ -21453,10 +21453,10 @@
       <c r="D186" s="89" t="s">
         <v>131</v>
       </c>
-      <c r="E186" s="89"/>
-      <c r="F186" s="89" t="s">
-        <v>273</v>
-      </c>
+      <c r="E186" s="89">
+        <v>0</v>
+      </c>
+      <c r="F186" s="89"/>
       <c r="G186" s="89" t="s">
         <v>273</v>
       </c>
@@ -21544,13 +21544,9 @@
       <c r="C187" s="10" t="s">
         <v>366</v>
       </c>
-      <c r="D187" s="89" t="s">
-        <v>131</v>
-      </c>
+      <c r="D187" s="89"/>
       <c r="E187" s="89"/>
-      <c r="F187" s="89" t="s">
-        <v>273</v>
-      </c>
+      <c r="F187" s="89"/>
       <c r="G187" s="89" t="s">
         <v>273</v>
       </c>
@@ -21634,8 +21630,8 @@
         <f>+AA187-AI187</f>
         <v>-100999999.99999905</v>
       </c>
-      <c r="AK187" s="90" t="s">
-        <v>45</v>
+      <c r="AK187" s="90">
+        <v>0</v>
       </c>
     </row>
     <row r="188" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -21738,7 +21734,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="189" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A189" s="14" t="s">
         <v>303</v>
       </c>
@@ -21758,9 +21754,7 @@
         <v>273</v>
       </c>
       <c r="I189" s="103"/>
-      <c r="J189" s="94">
-        <v>3390677291.5700002</v>
-      </c>
+      <c r="J189" s="94"/>
       <c r="K189" s="94">
         <v>3390677291.5700002</v>
       </c>
@@ -21786,7 +21780,7 @@
         <v>45</v>
       </c>
       <c r="S189" s="94">
-        <f t="shared" si="77"/>
+        <f>+K189</f>
         <v>3390677291.5700002</v>
       </c>
       <c r="T189" s="96">
@@ -21925,7 +21919,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="191" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A191" s="10" t="s">
         <v>303</v>
       </c>
@@ -34505,7 +34499,7 @@
       <c r="AI481" s="94"/>
       <c r="AJ481" s="94"/>
       <c r="AK481" s="90" t="str">
-        <f t="shared" ref="AK481:AK544" si="84">IF(Q481="ANULADA","N/A",IF(ABS(AJ481)&gt;10,"Pendiente",IF(MAX(AB481,AD481,AF481)=0,"Pendiente",MAX(0,MAX(AB481,AD481,AF481)-O481))))</f>
+        <f t="shared" ref="AK481:AK542" si="84">IF(Q481="ANULADA","N/A",IF(ABS(AJ481)&gt;10,"Pendiente",IF(MAX(AB481,AD481,AF481)=0,"Pendiente",MAX(0,MAX(AB481,AD481,AF481)-O481))))</f>
         <v>Pendiente</v>
       </c>
     </row>
@@ -36651,7 +36645,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="533" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="533" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A533" s="10" t="s">
         <v>303</v>
       </c>
@@ -36698,25 +36692,25 @@
       <c r="S533" s="94"/>
       <c r="T533" s="94"/>
       <c r="U533" s="94">
-        <f t="shared" ref="U533:U544" si="85">+S533*21%</f>
+        <f t="shared" ref="U533:U542" si="85">+S533*21%</f>
         <v>0</v>
       </c>
       <c r="V533" s="94">
-        <f t="shared" ref="V533:V544" si="86">+S533*3%</f>
+        <f t="shared" ref="V533:V542" si="86">+S533*3%</f>
         <v>0</v>
       </c>
       <c r="W533" s="94">
-        <f t="shared" ref="W533:W544" si="87">+S533*2.5%</f>
+        <f t="shared" ref="W533:W542" si="87">+S533*2.5%</f>
         <v>0</v>
       </c>
       <c r="X533" s="94">
-        <f t="shared" ref="X533:X544" si="88">IF(A533="00-175",S533*0.06,0)</f>
+        <f t="shared" ref="X533:X542" si="88">IF(A533="00-175",S533*0.06,0)</f>
         <v>0</v>
       </c>
       <c r="Y533" s="94"/>
       <c r="Z533" s="94"/>
       <c r="AA533" s="94">
-        <f t="shared" ref="AA533:AA544" si="89">+S533+T533+U533+W533+X533+V533+Y533</f>
+        <f t="shared" ref="AA533:AA542" si="89">+S533+T533+U533+W533+X533+V533+Y533</f>
         <v>0</v>
       </c>
       <c r="AB533" s="10"/>
@@ -36727,18 +36721,18 @@
       <c r="AG533" s="94"/>
       <c r="AH533" s="94"/>
       <c r="AI533" s="94">
-        <f t="shared" ref="AI533:AI544" si="90">+AC533+AE533+AG533+AH533</f>
+        <f t="shared" ref="AI533:AI542" si="90">+AC533+AE533+AG533+AH533</f>
         <v>0</v>
       </c>
       <c r="AJ533" s="94">
-        <f t="shared" ref="AJ533:AJ544" si="91">+AA533-AI533</f>
+        <f t="shared" ref="AJ533:AJ542" si="91">+AA533-AI533</f>
         <v>0</v>
       </c>
       <c r="AK533" s="90" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="534" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="534" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A534" s="10" t="s">
         <v>303</v>
       </c>
@@ -36825,7 +36819,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="535" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="535" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A535" s="10" t="s">
         <v>303</v>
       </c>
@@ -36912,7 +36906,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="536" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="536" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A536" s="10" t="s">
         <v>303</v>
       </c>
@@ -36999,7 +36993,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="537" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="537" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A537" s="10" t="s">
         <v>303</v>
       </c>
@@ -37085,7 +37079,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="538" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="538" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A538" s="10" t="s">
         <v>303</v>
       </c>
@@ -37171,7 +37165,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="539" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="539" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A539" s="10" t="s">
         <v>303</v>
       </c>
@@ -37258,7 +37252,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="540" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="540" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A540" s="10" t="s">
         <v>303</v>
       </c>
@@ -37345,7 +37339,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="541" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="541" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A541" s="10" t="s">
         <v>303</v>
       </c>
@@ -37433,7 +37427,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="542" spans="1:37" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="542" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A542" s="10" t="s">
         <v>303</v>
       </c>
@@ -37601,10 +37595,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AL542" xr:uid="{5A8C97C7-1B0D-4A6A-98DD-BAF1D96B2F33}">
-    <filterColumn colId="2">
+    <filterColumn colId="0">
       <filters>
-        <filter val="Edificios 5 al 8 - Puerto Nizuc"/>
-        <filter val="Edificios 7 a 8 - Puerto Nizuc"/>
+        <filter val="00-177"/>
+        <filter val="00-178"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -39183,21 +39177,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100EE506009F82FD740AE7A6453FF89BBF1" ma:contentTypeVersion="3" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="427c247a1fe2449ecb2d3d2841010e42">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1ef56690-0382-401c-bb03-84a4fbd81909" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="64db3c3f391b08d30a3ea0e014ceeeea" ns2:_="">
     <xsd:import namespace="1ef56690-0382-401c-bb03-84a4fbd81909"/>
@@ -39335,24 +39314,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C262C33D-CD57-41B0-B758-F02C54BD5F45}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{778BDEFC-2169-4411-86FE-3B90B0F4B579}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7072A91A-ED2E-4C03-B5DD-59EB3127F9D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -39368,4 +39345,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{778BDEFC-2169-4411-86FE-3B90B0F4B579}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C262C33D-CD57-41B0-B758-F02C54BD5F45}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica 01/06/2026 14:07 (Buenos Aires)
</commit_message>
<xml_diff>
--- a/Master UOPs.xlsx
+++ b/Master UOPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365iebc-my.sharepoint.com/personal/mperez_iebc_com_ar/Documents/Seguimiento Obras/Reporte de Obras/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{06376EE1-B0DD-45EC-BF0E-FB21B357E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{988BB022-ABC9-4C4A-A239-9F0A36E77166}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="8_{06376EE1-B0DD-45EC-BF0E-FB21B357E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43A94FB4-B8F2-45FF-9444-592618A601CE}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B067436-489C-4F7D-A3D3-1998983265A1}"/>
   </bookViews>
@@ -2986,7 +2986,7 @@
   <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AL544"/>
+  <dimension ref="A1:AL542"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" style="86" customWidth="1"/>
@@ -21581,20 +21581,19 @@
       <c r="R187" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="S187" s="94">
-        <f t="shared" si="77"/>
-        <v>0</v>
+      <c r="S187" s="96">
+        <v>4837006172.4499998</v>
       </c>
       <c r="T187" s="96">
         <v>507885648.11000001</v>
       </c>
       <c r="U187" s="96">
         <f t="shared" si="71"/>
-        <v>0</v>
+        <v>1015771296.2145</v>
       </c>
       <c r="V187" s="96">
         <f t="shared" si="70"/>
-        <v>0</v>
+        <v>145110185.1735</v>
       </c>
       <c r="W187" s="96">
         <v>145110185.16999999</v>
@@ -37515,84 +37514,6 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="543" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A543" s="10"/>
-      <c r="B543" s="14"/>
-      <c r="C543" s="10"/>
-      <c r="D543" s="89"/>
-      <c r="E543" s="89"/>
-      <c r="F543" s="89"/>
-      <c r="G543" s="89"/>
-      <c r="H543" s="92"/>
-      <c r="I543" s="103"/>
-      <c r="J543" s="94"/>
-      <c r="K543" s="94"/>
-      <c r="L543" s="89"/>
-      <c r="M543" s="10"/>
-      <c r="N543" s="33"/>
-      <c r="O543" s="12"/>
-      <c r="P543" s="10"/>
-      <c r="Q543" s="10"/>
-      <c r="R543" s="10"/>
-      <c r="S543" s="94"/>
-      <c r="T543" s="94"/>
-      <c r="U543" s="94"/>
-      <c r="V543" s="94"/>
-      <c r="W543" s="94"/>
-      <c r="X543" s="94"/>
-      <c r="Y543" s="94"/>
-      <c r="Z543" s="94"/>
-      <c r="AA543" s="94"/>
-      <c r="AB543" s="10"/>
-      <c r="AC543" s="94"/>
-      <c r="AD543" s="10"/>
-      <c r="AE543" s="94"/>
-      <c r="AF543" s="10"/>
-      <c r="AG543" s="94"/>
-      <c r="AH543" s="94"/>
-      <c r="AI543" s="94"/>
-      <c r="AJ543" s="94"/>
-      <c r="AK543" s="90"/>
-    </row>
-    <row r="544" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A544" s="27"/>
-      <c r="B544" s="27"/>
-      <c r="C544" s="10"/>
-      <c r="D544" s="89"/>
-      <c r="E544" s="89"/>
-      <c r="F544" s="89"/>
-      <c r="G544" s="89"/>
-      <c r="H544" s="92"/>
-      <c r="I544" s="103"/>
-      <c r="J544" s="94"/>
-      <c r="K544" s="94"/>
-      <c r="L544" s="89"/>
-      <c r="M544" s="27"/>
-      <c r="N544" s="33"/>
-      <c r="O544" s="12"/>
-      <c r="P544" s="10"/>
-      <c r="Q544" s="10"/>
-      <c r="R544" s="10"/>
-      <c r="S544" s="94"/>
-      <c r="T544" s="94"/>
-      <c r="U544" s="94"/>
-      <c r="V544" s="94"/>
-      <c r="W544" s="94"/>
-      <c r="X544" s="94"/>
-      <c r="Y544" s="94"/>
-      <c r="Z544" s="94"/>
-      <c r="AA544" s="94"/>
-      <c r="AB544" s="10"/>
-      <c r="AC544" s="94"/>
-      <c r="AD544" s="10"/>
-      <c r="AE544" s="94"/>
-      <c r="AF544" s="10"/>
-      <c r="AG544" s="94"/>
-      <c r="AH544" s="94"/>
-      <c r="AI544" s="94"/>
-      <c r="AJ544" s="94"/>
-      <c r="AK544" s="90"/>
-    </row>
   </sheetData>
   <autoFilter ref="A1:AL542" xr:uid="{5A8C97C7-1B0D-4A6A-98DD-BAF1D96B2F33}">
     <filterColumn colId="0">
@@ -37602,7 +37523,7 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AK544">
+  <conditionalFormatting sqref="A2:AK542">
     <cfRule type="expression" dxfId="6" priority="1" stopIfTrue="1">
       <formula>$Q2="ANULADA"</formula>
     </cfRule>
@@ -37626,7 +37547,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L544" xr:uid="{E756ABC1-A59D-4E79-9F2A-CB23C9909C50}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L542" xr:uid="{E756ABC1-A59D-4E79-9F2A-CB23C9909C50}">
       <formula1>"Validado,En Espera"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Actualizacion automatica 01/06/2026 14:12 (Buenos Aires)
</commit_message>
<xml_diff>
--- a/Master UOPs.xlsx
+++ b/Master UOPs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365iebc-my.sharepoint.com/personal/mperez_iebc_com_ar/Documents/Seguimiento Obras/Reporte de Obras/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{06376EE1-B0DD-45EC-BF0E-FB21B357E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43A94FB4-B8F2-45FF-9444-592618A601CE}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{06376EE1-B0DD-45EC-BF0E-FB21B357E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{94454E86-7D05-4F12-B026-ECE7D0806064}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B067436-489C-4F7D-A3D3-1998983265A1}"/>
   </bookViews>
@@ -260,7 +260,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2106" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2120" uniqueCount="368">
   <si>
     <t>UOP</t>
   </si>
@@ -2210,7 +2210,84 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{3BDA488D-6413-4408-9FA7-0A150A79E108}"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F4E79"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD6E4F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF4A0072"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE8D5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF595959"/>
@@ -2986,7 +3063,7 @@
   <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AL542"/>
+  <dimension ref="A1:AL544"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" style="86" customWidth="1"/>
@@ -37514,6 +37591,182 @@
         <v>Pendiente</v>
       </c>
     </row>
+    <row r="543" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A543" s="10" t="s">
+        <v>303</v>
+      </c>
+      <c r="B543" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C543" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="D543" s="89" t="s">
+        <v>307</v>
+      </c>
+      <c r="E543" s="89">
+        <v>6</v>
+      </c>
+      <c r="F543" s="89" t="s">
+        <v>316</v>
+      </c>
+      <c r="G543" s="89" t="s">
+        <v>47</v>
+      </c>
+      <c r="H543" s="92">
+        <v>46143</v>
+      </c>
+      <c r="I543" s="103">
+        <f>+J543-K543</f>
+        <v>424156102.47000003</v>
+      </c>
+      <c r="J543" s="116">
+        <v>792977332.10000002</v>
+      </c>
+      <c r="K543" s="116">
+        <v>368821229.63</v>
+      </c>
+      <c r="L543" s="89" t="s">
+        <v>233</v>
+      </c>
+      <c r="M543" s="10"/>
+      <c r="N543" s="33"/>
+      <c r="O543" s="12"/>
+      <c r="P543" s="10"/>
+      <c r="Q543" s="10"/>
+      <c r="R543" s="10"/>
+      <c r="S543" s="94"/>
+      <c r="T543" s="94"/>
+      <c r="U543" s="94">
+        <f t="shared" ref="U543:U544" si="93">+S543*21%</f>
+        <v>0</v>
+      </c>
+      <c r="V543" s="94">
+        <f t="shared" ref="V543:V544" si="94">+S543*3%</f>
+        <v>0</v>
+      </c>
+      <c r="W543" s="94">
+        <f t="shared" ref="W543:W544" si="95">+S543*2.5%</f>
+        <v>0</v>
+      </c>
+      <c r="X543" s="94">
+        <f t="shared" ref="X543:X544" si="96">IF(A543="00-175",S543*0.06,0)</f>
+        <v>0</v>
+      </c>
+      <c r="Y543" s="94"/>
+      <c r="Z543" s="94"/>
+      <c r="AA543" s="94">
+        <f t="shared" ref="AA543:AA544" si="97">+S543+T543+U543+W543+X543+V543+Y543</f>
+        <v>0</v>
+      </c>
+      <c r="AB543" s="10"/>
+      <c r="AC543" s="94"/>
+      <c r="AD543" s="10"/>
+      <c r="AE543" s="94"/>
+      <c r="AF543" s="10"/>
+      <c r="AG543" s="94"/>
+      <c r="AH543" s="94"/>
+      <c r="AI543" s="94">
+        <f t="shared" ref="AI543:AI544" si="98">+AC543+AE543+AG543+AH543</f>
+        <v>0</v>
+      </c>
+      <c r="AJ543" s="94">
+        <f t="shared" ref="AJ543:AJ544" si="99">+AA543-AI543</f>
+        <v>0</v>
+      </c>
+      <c r="AK543" s="90" t="str">
+        <f t="shared" ref="AK543:AK544" si="100">IF(Q543="ANULADA","N/A",IF(ABS(AJ543)&gt;10,"Pendiente",IF(MAX(AB543,AD543,AF543)=0,"Pendiente",MAX(0,MAX(AB543,AD543,AF543)-O543))))</f>
+        <v>Pendiente</v>
+      </c>
+    </row>
+    <row r="544" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A544" s="10" t="s">
+        <v>303</v>
+      </c>
+      <c r="B544" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="C544" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="D544" s="89" t="s">
+        <v>307</v>
+      </c>
+      <c r="E544" s="89">
+        <v>6</v>
+      </c>
+      <c r="F544" s="89" t="s">
+        <v>317</v>
+      </c>
+      <c r="G544" s="89" t="s">
+        <v>47</v>
+      </c>
+      <c r="H544" s="92">
+        <v>46143</v>
+      </c>
+      <c r="I544" s="103">
+        <f t="shared" ref="I544" si="101">+J544</f>
+        <v>56045106.539999999</v>
+      </c>
+      <c r="J544" s="116">
+        <v>56045106.539999999</v>
+      </c>
+      <c r="K544" s="116">
+        <v>0</v>
+      </c>
+      <c r="L544" s="89" t="s">
+        <v>233</v>
+      </c>
+      <c r="M544" s="10"/>
+      <c r="N544" s="33"/>
+      <c r="O544" s="12"/>
+      <c r="P544" s="10"/>
+      <c r="Q544" s="10"/>
+      <c r="R544" s="10"/>
+      <c r="S544" s="94"/>
+      <c r="T544" s="94"/>
+      <c r="U544" s="94">
+        <f t="shared" si="93"/>
+        <v>0</v>
+      </c>
+      <c r="V544" s="94">
+        <f t="shared" si="94"/>
+        <v>0</v>
+      </c>
+      <c r="W544" s="94">
+        <f t="shared" si="95"/>
+        <v>0</v>
+      </c>
+      <c r="X544" s="94">
+        <f t="shared" si="96"/>
+        <v>0</v>
+      </c>
+      <c r="Y544" s="94"/>
+      <c r="Z544" s="94"/>
+      <c r="AA544" s="94">
+        <f t="shared" si="97"/>
+        <v>0</v>
+      </c>
+      <c r="AB544" s="10"/>
+      <c r="AC544" s="94"/>
+      <c r="AD544" s="10"/>
+      <c r="AE544" s="94"/>
+      <c r="AF544" s="10"/>
+      <c r="AG544" s="94"/>
+      <c r="AH544" s="94"/>
+      <c r="AI544" s="94">
+        <f t="shared" si="98"/>
+        <v>0</v>
+      </c>
+      <c r="AJ544" s="94">
+        <f t="shared" si="99"/>
+        <v>0</v>
+      </c>
+      <c r="AK544" s="90" t="str">
+        <f t="shared" si="100"/>
+        <v>Pendiente</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AL542" xr:uid="{5A8C97C7-1B0D-4A6A-98DD-BAF1D96B2F33}">
     <filterColumn colId="0">
@@ -37524,30 +37777,53 @@
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="A2:AK542">
-    <cfRule type="expression" dxfId="6" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="8" stopIfTrue="1">
       <formula>$Q2="ANULADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="9" stopIfTrue="1">
       <formula>LEFT($M2,2)="NC"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="10" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,$AJ2&lt;-10)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="11" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,ABS($AJ2)&lt;=10)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="9" priority="12" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,$AJ2&gt;10)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="13" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;"ANULADA",$AA2&gt;0,OR($AI2=0,$AI2=""))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="14" stopIfTrue="1">
       <formula>$A2&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A543:AK544">
+    <cfRule type="expression" dxfId="6" priority="1" stopIfTrue="1">
+      <formula>$Q543="ANULADA"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="2" stopIfTrue="1">
+      <formula>LEFT($M543,2)="NC"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="3" stopIfTrue="1">
+      <formula>AND($Q543&lt;&gt;"ANULADA",$AI543&gt;0,$AJ543&lt;-10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
+      <formula>AND($Q543&lt;&gt;"ANULADA",$AI543&gt;0,ABS($AJ543)&lt;=10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
+      <formula>AND($Q543&lt;&gt;"ANULADA",$AI543&gt;0,$AJ543&gt;10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
+      <formula>AND($Q543&lt;&gt;"ANULADA",$AA543&gt;0,OR($AI543=0,$AI543=""))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="7" stopIfTrue="1">
+      <formula>$A543&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L542" xr:uid="{E756ABC1-A59D-4E79-9F2A-CB23C9909C50}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2:L544" xr:uid="{E756ABC1-A59D-4E79-9F2A-CB23C9909C50}">
       <formula1>"Validado,En Espera"</formula1>
     </dataValidation>
   </dataValidations>
@@ -39041,15 +39317,15 @@
       </c>
       <c r="I7" s="113">
         <f>SUMIFS(Master!I:I,Master!A:A,A7)</f>
-        <v>3541317286.6800003</v>
+        <v>4021518495.6900005</v>
       </c>
       <c r="J7" s="113">
         <f>H7-I7</f>
-        <v>1015.599871635437</v>
+        <v>-480200193.41012859</v>
       </c>
       <c r="K7" s="114">
         <f>IFERROR(I7/H7,0)</f>
-        <v>0.99999971321418046</v>
+        <v>1.1355992747392911</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Actualizacion automatica 02/06/2026 19:13 (Buenos Aires)
</commit_message>
<xml_diff>
--- a/Master UOPs.xlsx
+++ b/Master UOPs.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://365iebc-my.sharepoint.com/personal/mperez_iebc_com_ar/Documents/Seguimiento Obras/Reporte de Obras/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="8_{06376EE1-B0DD-45EC-BF0E-FB21B357E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0847FD7B-C0DC-4437-8632-371C7030A1BF}"/>
+  <xr:revisionPtr revIDLastSave="117" documentId="8_{06376EE1-B0DD-45EC-BF0E-FB21B357E1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42C45274-9C54-4D32-AB28-C9E46A6C8A4E}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B067436-489C-4F7D-A3D3-1998983265A1}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0B067436-489C-4F7D-A3D3-1998983265A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="5" r:id="rId1"/>
     <sheet name="530 con Mora - Calc de int" sheetId="4" r:id="rId2"/>
     <sheet name="Anticipos" sheetId="7" r:id="rId3"/>
+    <sheet name="Montos contractuales" sheetId="8" r:id="rId4"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Master!$A$1:$AL$542</definedName>
@@ -271,7 +272,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2106" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2124" uniqueCount="374">
   <si>
     <t>UOP</t>
   </si>
@@ -1385,18 +1386,37 @@
   <si>
     <t>0018-00002546</t>
   </si>
+  <si>
+    <t>Monto</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>contrato Ajuste alzado</t>
+  </si>
+  <si>
+    <t>Ampliacion</t>
+  </si>
+  <si>
+    <t>Carta Oferta</t>
+  </si>
+  <si>
+    <t>Contrato Coste y Costas</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="mm/yyyy"/>
+    <numFmt numFmtId="170" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
   </numFmts>
   <fonts count="41">
     <font>
@@ -1920,7 +1940,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2213,6 +2233,8 @@
     <xf numFmtId="0" fontId="37" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Hipervínculo 2" xfId="3" xr:uid="{AEDFE01B-1CF9-469C-A069-20D44665E288}"/>
@@ -2221,7 +2243,285 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{3BDA488D-6413-4408-9FA7-0A150A79E108}"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="31">
+    <dxf>
+      <numFmt numFmtId="22" formatCode="mmm\-yy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="170" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE4D6"/>
+          <bgColor rgb="FFFFD7D7"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F4E79"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD6E4F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF4A0072"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE8D5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F4E79"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD6E4F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF4A0072"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE8D5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF1F4E79"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD6E4F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF4A0072"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE8D5F5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF595959"/>
@@ -2670,6 +2970,19 @@
 </externalLink>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1EE128AB-CAF0-43E2-AA08-6794C04E04FA}" name="Tabla1" displayName="Tabla1" ref="A2:D9" totalsRowShown="0">
+  <autoFilter ref="A2:D9" xr:uid="{1EE128AB-CAF0-43E2-AA08-6794C04E04FA}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{64C72B70-DC43-4D40-855E-DAF5A7700583}" name="UOP" dataDxfId="2" dataCellStyle="Normal 2"/>
+    <tableColumn id="2" xr3:uid="{F87F7CA3-D4A1-4668-953D-123F5F6C107F}" name="Concepto"/>
+    <tableColumn id="3" xr3:uid="{E7E7C505-0FFB-4C70-8A2C-86DDE4FD4B32}" name="Monto" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{2FFACDB6-DBBC-4E53-B403-00E141A813FB}" name="Fecha" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -9075,7 +9388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:37" ht="15" customHeight="1">
+    <row r="59" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A59" s="10" t="s">
         <v>130</v>
       </c>
@@ -10840,7 +11153,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:37" ht="15" customHeight="1">
+    <row r="76" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A76" s="10" t="s">
         <v>130</v>
       </c>
@@ -10940,7 +11253,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="77" spans="1:37" ht="15" customHeight="1">
+    <row r="77" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A77" s="27" t="s">
         <v>130</v>
       </c>
@@ -11038,7 +11351,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="78" spans="1:37" ht="15" customHeight="1">
+    <row r="78" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A78" s="27" t="s">
         <v>130</v>
       </c>
@@ -12666,7 +12979,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="1:37" ht="15" customHeight="1">
+    <row r="94" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A94" s="10" t="s">
         <v>130</v>
       </c>
@@ -12764,7 +13077,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="95" spans="1:37" ht="15" customHeight="1">
+    <row r="95" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A95" s="27" t="s">
         <v>130</v>
       </c>
@@ -12860,7 +13173,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="96" spans="1:37" ht="15" customHeight="1">
+    <row r="96" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A96" s="10" t="s">
         <v>130</v>
       </c>
@@ -14185,7 +14498,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="109" spans="1:37" ht="15" customHeight="1">
+    <row r="109" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A109" s="10" t="s">
         <v>130</v>
       </c>
@@ -14281,7 +14594,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="110" spans="1:37">
+    <row r="110" spans="1:37" hidden="1">
       <c r="A110" s="27" t="s">
         <v>130</v>
       </c>
@@ -15701,7 +16014,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="124" spans="1:37" ht="15" customHeight="1">
+    <row r="124" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A124" s="10" t="s">
         <v>130</v>
       </c>
@@ -15807,7 +16120,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="125" spans="1:37" ht="15" customHeight="1">
+    <row r="125" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A125" s="27" t="s">
         <v>130</v>
       </c>
@@ -17181,7 +17494,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="141" spans="1:37" ht="15" customHeight="1">
+    <row r="141" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A141" s="10" t="s">
         <v>130</v>
       </c>
@@ -17266,7 +17579,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="142" spans="1:37" ht="15" customHeight="1">
+    <row r="142" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A142" s="27" t="s">
         <v>130</v>
       </c>
@@ -21451,7 +21764,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="186" spans="1:37" ht="15" customHeight="1">
+    <row r="186" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A186" s="14" t="s">
         <v>130</v>
       </c>
@@ -21545,7 +21858,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="187" spans="1:37" ht="15" customHeight="1">
+    <row r="187" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A187" s="14" t="s">
         <v>130</v>
       </c>
@@ -21744,7 +22057,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="189" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="189" spans="1:37" ht="15" customHeight="1">
       <c r="A189" s="14" t="s">
         <v>305</v>
       </c>
@@ -21837,7 +22150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:37" ht="15" customHeight="1">
+    <row r="190" spans="1:37" ht="15" hidden="1" customHeight="1">
       <c r="A190" s="7" t="s">
         <v>130</v>
       </c>
@@ -21929,7 +22242,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="191" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="191" spans="1:37" ht="15" customHeight="1">
       <c r="A191" s="10" t="s">
         <v>305</v>
       </c>
@@ -36655,7 +36968,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="533" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="533" spans="1:37" ht="15" customHeight="1">
       <c r="A533" s="10" t="s">
         <v>305</v>
       </c>
@@ -36742,7 +37055,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="534" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="534" spans="1:37" ht="15" customHeight="1">
       <c r="A534" s="10" t="s">
         <v>305</v>
       </c>
@@ -36829,7 +37142,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="535" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="535" spans="1:37" ht="15" customHeight="1">
       <c r="A535" s="10" t="s">
         <v>305</v>
       </c>
@@ -36916,7 +37229,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="536" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="536" spans="1:37" ht="15" customHeight="1">
       <c r="A536" s="10" t="s">
         <v>305</v>
       </c>
@@ -37003,7 +37316,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="537" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="537" spans="1:37" ht="15" customHeight="1">
       <c r="A537" s="10" t="s">
         <v>305</v>
       </c>
@@ -37089,7 +37402,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="538" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="538" spans="1:37" ht="15" customHeight="1">
       <c r="A538" s="10" t="s">
         <v>305</v>
       </c>
@@ -37175,7 +37488,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="539" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="539" spans="1:37" ht="15" customHeight="1">
       <c r="A539" s="10" t="s">
         <v>305</v>
       </c>
@@ -37262,7 +37575,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="540" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="540" spans="1:37" ht="15" customHeight="1">
       <c r="A540" s="10" t="s">
         <v>305</v>
       </c>
@@ -37349,7 +37662,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="541" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="541" spans="1:37" ht="15" customHeight="1">
       <c r="A541" s="10" t="s">
         <v>305</v>
       </c>
@@ -37437,7 +37750,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="542" spans="1:37" ht="15" hidden="1" customHeight="1">
+    <row r="542" spans="1:37" ht="15" customHeight="1">
       <c r="A542" s="10" t="s">
         <v>305</v>
       </c>
@@ -37529,30 +37842,30 @@
   <autoFilter ref="A1:AL542" xr:uid="{5A8C97C7-1B0D-4A6A-98DD-BAF1D96B2F33}">
     <filterColumn colId="0">
       <filters>
-        <filter val="00-177"/>
+        <filter val="00-178"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="A2:AK542">
-    <cfRule type="expression" dxfId="6" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="30" priority="1" stopIfTrue="1">
       <formula>$Q2="ANULADA"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="29" priority="2" stopIfTrue="1">
       <formula>LEFT($M2,2)="NC"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="28" priority="3" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,$AJ2&lt;-10)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="27" priority="4" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,ABS($AJ2)&lt;=10)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="26" priority="5" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,$AJ2&gt;10)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="25" priority="6" stopIfTrue="1">
       <formula>AND($Q2&lt;&gt;"ANULADA",$AA2&gt;0,OR($AI2=0,$AI2=""))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="24" priority="7" stopIfTrue="1">
       <formula>$A2&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
@@ -37653,7 +37966,7 @@
       </c>
       <c r="B7" s="46">
         <f ca="1">TODAY()</f>
-        <v>46174</v>
+        <v>46175</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="9.9499999999999993" customHeight="1"/>
@@ -37719,7 +38032,7 @@
       </c>
       <c r="G10" s="48">
         <f t="shared" ref="G10:G27" ca="1" si="2">IF(F10="",MAX(0,$B$7-E10),MAX(0,F10-E10))</f>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H10" s="52">
         <f>'[1]Facturas desde 2025'!P4</f>
@@ -37731,11 +38044,11 @@
       </c>
       <c r="J10" s="54">
         <f ca="1">H10*I10*(G10/365)</f>
-        <v>3109075.4085826031</v>
+        <v>3148430.7935013701</v>
       </c>
       <c r="K10" s="55">
         <f t="shared" ref="K10:K27" ca="1" si="3">H10+J10</f>
-        <v>53511585.918582603</v>
+        <v>53550941.303501368</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -37765,7 +38078,7 @@
       </c>
       <c r="G11" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H11" s="59">
         <f>'[1]Facturas desde 2025'!P5</f>
@@ -37777,11 +38090,11 @@
       </c>
       <c r="J11" s="60">
         <f t="shared" ref="J11:J27" ca="1" si="5">H11*I11*(G11/365)</f>
-        <v>41777.474464109589</v>
+        <v>42306.303254794519</v>
       </c>
       <c r="K11" s="61">
         <f t="shared" ca="1" si="3"/>
-        <v>719049.4344641096</v>
+        <v>719578.26325479452</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="18.600000000000001" customHeight="1">
@@ -37811,7 +38124,7 @@
       </c>
       <c r="G12" s="48">
         <f t="shared" ca="1" si="2"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H12" s="52">
         <f>'[1]Facturas desde 2025'!P6</f>
@@ -37823,11 +38136,11 @@
       </c>
       <c r="J12" s="54">
         <f t="shared" ca="1" si="5"/>
-        <v>1091812.5174821918</v>
+        <v>1105632.9290958904</v>
       </c>
       <c r="K12" s="55">
         <f t="shared" ca="1" si="3"/>
-        <v>18791637.91748219</v>
+        <v>18805458.329095889</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -37857,7 +38170,7 @@
       </c>
       <c r="G13" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H13" s="59">
         <f>'[1]Facturas desde 2025'!P7</f>
@@ -37869,11 +38182,11 @@
       </c>
       <c r="J13" s="60">
         <f t="shared" ca="1" si="5"/>
-        <v>62666.211696164391</v>
+        <v>63459.454882191785</v>
       </c>
       <c r="K13" s="61">
         <f t="shared" ca="1" si="3"/>
-        <v>1078574.1516961644</v>
+        <v>1079367.3948821917</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -37903,7 +38216,7 @@
       </c>
       <c r="G14" s="48">
         <f t="shared" ca="1" si="2"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H14" s="52">
         <f>'[1]Facturas desde 2025'!P8</f>
@@ -37915,11 +38228,11 @@
       </c>
       <c r="J14" s="54">
         <f t="shared" ca="1" si="5"/>
-        <v>1681153.42439137</v>
+        <v>1702433.8474849316</v>
       </c>
       <c r="K14" s="55">
         <f t="shared" ca="1" si="3"/>
-        <v>28935028.614391372</v>
+        <v>28956309.037484933</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -37949,7 +38262,7 @@
       </c>
       <c r="G15" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H15" s="59">
         <f>'[1]Facturas desde 2025'!P9</f>
@@ -37961,11 +38274,11 @@
       </c>
       <c r="J15" s="60">
         <f t="shared" ca="1" si="5"/>
-        <v>62666.211696164391</v>
+        <v>63459.454882191785</v>
       </c>
       <c r="K15" s="61">
         <f t="shared" ca="1" si="3"/>
-        <v>1078574.1516961644</v>
+        <v>1079367.3948821917</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -37995,7 +38308,7 @@
       </c>
       <c r="G16" s="48">
         <f t="shared" ca="1" si="2"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H16" s="52">
         <f>'[1]Facturas desde 2025'!P10</f>
@@ -38007,11 +38320,11 @@
       </c>
       <c r="J16" s="54">
         <f t="shared" ca="1" si="5"/>
-        <v>1765899.0312887675</v>
+        <v>1788252.1835835618</v>
       </c>
       <c r="K16" s="55">
         <f t="shared" ca="1" si="3"/>
-        <v>30393620.391288769</v>
+        <v>30415973.543583561</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -38041,7 +38354,7 @@
       </c>
       <c r="G17" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H17" s="59">
         <f>'[1]Facturas desde 2025'!P11</f>
@@ -38053,11 +38366,11 @@
       </c>
       <c r="J17" s="60">
         <f t="shared" ca="1" si="5"/>
-        <v>14705.71604630137</v>
+        <v>14891.864350684931</v>
       </c>
       <c r="K17" s="61">
         <f t="shared" ca="1" si="3"/>
-        <v>253106.17604630135</v>
+        <v>253292.32435068491</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -38087,7 +38400,7 @@
       </c>
       <c r="G18" s="48">
         <f t="shared" ca="1" si="2"/>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H18" s="52">
         <f>'[1]Facturas desde 2025'!P12</f>
@@ -38099,11 +38412,11 @@
       </c>
       <c r="J18" s="54">
         <f t="shared" ca="1" si="5"/>
-        <v>416892.34416328766</v>
+        <v>422169.46244383563</v>
       </c>
       <c r="K18" s="55">
         <f t="shared" ca="1" si="3"/>
-        <v>7175306.9841632871</v>
+        <v>7180584.1024438357</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -38133,7 +38446,7 @@
       </c>
       <c r="G19" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H19" s="59">
         <f>'[1]Facturas desde 2025'!P14</f>
@@ -38145,11 +38458,11 @@
       </c>
       <c r="J19" s="60">
         <f t="shared" ca="1" si="5"/>
-        <v>21863.199916849317</v>
+        <v>22210.234836164385</v>
       </c>
       <c r="K19" s="61">
         <f t="shared" ca="1" si="3"/>
-        <v>466311.4299168493</v>
+        <v>466658.46483616438</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -38179,7 +38492,7 @@
       </c>
       <c r="G20" s="48">
         <f t="shared" ca="1" si="2"/>
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H20" s="52">
         <f>'[1]Facturas desde 2025'!P16</f>
@@ -38191,11 +38504,11 @@
       </c>
       <c r="J20" s="54">
         <f t="shared" ca="1" si="5"/>
-        <v>631234.31210383575</v>
+        <v>641253.90435945219</v>
       </c>
       <c r="K20" s="55">
         <f t="shared" ca="1" si="3"/>
-        <v>13463343.692103837</v>
+        <v>13473363.284359453</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -38225,7 +38538,7 @@
       </c>
       <c r="G21" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H21" s="59">
         <f>'[1]Facturas desde 2025'!P17</f>
@@ -38237,11 +38550,11 @@
       </c>
       <c r="J21" s="60">
         <f t="shared" ca="1" si="5"/>
-        <v>8335.4789383561656</v>
+        <v>8479.1940924657556</v>
       </c>
       <c r="K21" s="61">
         <f t="shared" ca="1" si="3"/>
-        <v>192391.72893835616</v>
+        <v>192535.44409246577</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -38271,7 +38584,7 @@
       </c>
       <c r="G22" s="48">
         <f t="shared" ca="1" si="2"/>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H22" s="52">
         <f>'[1]Facturas desde 2025'!P18</f>
@@ -38283,11 +38596,11 @@
       </c>
       <c r="J22" s="54">
         <f t="shared" ca="1" si="5"/>
-        <v>245727.13526958911</v>
+        <v>249963.8100156165</v>
       </c>
       <c r="K22" s="55">
         <f t="shared" ca="1" si="3"/>
-        <v>5671643.9152695891</v>
+        <v>5675880.5900156172</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -38317,7 +38630,7 @@
       </c>
       <c r="G23" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H23" s="59">
         <f>'[1]Facturas desde 2025'!P19</f>
@@ -38363,7 +38676,7 @@
       </c>
       <c r="G24" s="48">
         <f t="shared" ca="1" si="2"/>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H24" s="52">
         <f>'[1]Facturas desde 2025'!P20</f>
@@ -38409,7 +38722,7 @@
       </c>
       <c r="G25" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H25" s="59">
         <f>'[1]Facturas desde 2025'!P21</f>
@@ -38421,11 +38734,11 @@
       </c>
       <c r="J25" s="60">
         <f t="shared" ca="1" si="5"/>
-        <v>2538.3782202739726</v>
+        <v>2697.026859041096</v>
       </c>
       <c r="K25" s="61">
         <f t="shared" ca="1" si="3"/>
-        <v>205719.96822027396</v>
+        <v>205878.6168590411</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -38455,7 +38768,7 @@
       </c>
       <c r="G26" s="48">
         <f t="shared" ca="1" si="2"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H26" s="52">
         <f>'[1]Facturas desde 2025'!P22</f>
@@ -38501,7 +38814,7 @@
       </c>
       <c r="G27" s="56">
         <f t="shared" ca="1" si="2"/>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H27" s="59">
         <f>'[1]Facturas desde 2025'!P23</f>
@@ -38513,11 +38826,11 @@
       </c>
       <c r="J27" s="60">
         <f t="shared" ca="1" si="5"/>
-        <v>78285.275815890418</v>
+        <v>83178.105554383568</v>
       </c>
       <c r="K27" s="61">
         <f t="shared" ca="1" si="3"/>
-        <v>6344540.9058158901</v>
+        <v>6349433.7355543831</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -38715,7 +39028,7 @@
       <c r="F32" s="77"/>
       <c r="G32" s="78">
         <f ca="1">IF(COUNTA(F10:F31)&gt;0,AVERAGE(G10:G31),AVERAGE(G10:G31))</f>
-        <v>50.636363636363633</v>
+        <v>51.454545454545453</v>
       </c>
       <c r="H32" s="79">
         <f>SUBTOTAL(109,H10:H31)</f>
@@ -38724,11 +39037,11 @@
       <c r="I32" s="77"/>
       <c r="J32" s="79">
         <f ca="1">SUBTOTAL(109,J10:J31)</f>
-        <v>9234632.1200757548</v>
+        <v>9358818.5691965744</v>
       </c>
       <c r="K32" s="79">
         <f ca="1">SUBTOTAL(109,K10:K31)</f>
-        <v>320304946.82007575</v>
+        <v>320429133.26919657</v>
       </c>
     </row>
     <row r="34" spans="1:2">
@@ -38751,7 +39064,7 @@
       </c>
       <c r="B36" s="81">
         <f ca="1">J32</f>
-        <v>9234632.1200757548</v>
+        <v>9358818.5691965744</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="15.6">
@@ -38760,7 +39073,7 @@
       </c>
       <c r="B37" s="83">
         <f ca="1">B35+B36</f>
-        <v>320304946.82007575</v>
+        <v>320429133.26919657</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -38778,7 +39091,7 @@
       </c>
       <c r="B39" s="85">
         <f ca="1">G32</f>
-        <v>50.636363636363633</v>
+        <v>51.454545454545453</v>
       </c>
     </row>
   </sheetData>
@@ -39107,19 +39420,218 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFD968D-F146-4A4A-BB9D-AE16639B2D38}">
+  <dimension ref="A2:D9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s">
+        <v>370</v>
+      </c>
+      <c r="C3" s="118">
+        <v>1759695739.95</v>
+      </c>
+      <c r="D3" s="119">
+        <v>44256</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>371</v>
+      </c>
+      <c r="C4" s="118">
+        <v>351934615.48000002</v>
+      </c>
+      <c r="D4" s="119">
+        <v>46042</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
+        <v>372</v>
+      </c>
+      <c r="C5" s="118">
+        <v>2337056186.5799999</v>
+      </c>
+      <c r="D5" s="119">
+        <v>45870</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" t="s">
+        <v>372</v>
+      </c>
+      <c r="C6" s="118">
+        <v>5000000000</v>
+      </c>
+      <c r="D6" s="119">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" t="s">
+        <v>373</v>
+      </c>
+      <c r="C7" s="118">
+        <v>30896493733.389999</v>
+      </c>
+      <c r="D7" s="119">
+        <v>45870</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="10" t="s">
+        <v>305</v>
+      </c>
+      <c r="B8" t="s">
+        <v>373</v>
+      </c>
+      <c r="C8" s="118">
+        <v>33906772915.32</v>
+      </c>
+      <c r="D8" s="119">
+        <v>45870</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" t="s">
+        <v>372</v>
+      </c>
+      <c r="C9" s="118">
+        <v>1500000000</v>
+      </c>
+      <c r="D9" s="119">
+        <v>45839</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A3:A4 A9">
+    <cfRule type="expression" dxfId="23" priority="8" stopIfTrue="1">
+      <formula>$Q3="ANULADA"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="9" stopIfTrue="1">
+      <formula>LEFT($M3,2)="NC"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="21" priority="10" stopIfTrue="1">
+      <formula>AND($Q3&lt;&gt;"ANULADA",$AI3&gt;0,$AJ3&lt;-10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="20" priority="11" stopIfTrue="1">
+      <formula>AND($Q3&lt;&gt;"ANULADA",$AI3&gt;0,ABS($AJ3)&lt;=10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="12" stopIfTrue="1">
+      <formula>AND($Q3&lt;&gt;"ANULADA",$AI3&gt;0,$AJ3&gt;10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="13" stopIfTrue="1">
+      <formula>AND($Q3&lt;&gt;"ANULADA",$AA3&gt;0,OR($AI3=0,$AI3=""))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="17" priority="14" stopIfTrue="1">
+      <formula>$A3&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:A6">
+    <cfRule type="expression" dxfId="16" priority="1" stopIfTrue="1">
+      <formula>$Q2="ANULADA"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="2" stopIfTrue="1">
+      <formula>LEFT($M2,2)="NC"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="3" stopIfTrue="1">
+      <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,$AJ2&lt;-10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="4" stopIfTrue="1">
+      <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,ABS($AJ2)&lt;=10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="5" stopIfTrue="1">
+      <formula>AND($Q2&lt;&gt;"ANULADA",$AI2&gt;0,$AJ2&gt;10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="6" stopIfTrue="1">
+      <formula>AND($Q2&lt;&gt;"ANULADA",$AA2&gt;0,OR($AI2=0,$AI2=""))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="7" stopIfTrue="1">
+      <formula>$A5&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A7:A8">
+    <cfRule type="expression" dxfId="9" priority="29" stopIfTrue="1">
+      <formula>$Q5="ANULADA"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="30" stopIfTrue="1">
+      <formula>LEFT($M5,2)="NC"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="31" stopIfTrue="1">
+      <formula>AND($Q5&lt;&gt;"ANULADA",$AI5&gt;0,$AJ5&lt;-10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="32" stopIfTrue="1">
+      <formula>AND($Q5&lt;&gt;"ANULADA",$AI5&gt;0,ABS($AJ5)&lt;=10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="33" stopIfTrue="1">
+      <formula>AND($Q5&lt;&gt;"ANULADA",$AI5&gt;0,$AJ5&gt;10)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="34" stopIfTrue="1">
+      <formula>AND($Q5&lt;&gt;"ANULADA",$AA5&gt;0,OR($AI5=0,$AI5=""))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="35" stopIfTrue="1">
+      <formula>$A7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -39261,11 +39773,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{778BDEFC-2169-4411-86FE-3B90B0F4B579}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C262C33D-CD57-41B0-B758-F02C54BD5F45}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C262C33D-CD57-41B0-B758-F02C54BD5F45}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{778BDEFC-2169-4411-86FE-3B90B0F4B579}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Actualizacion automatica 12/06/2026 13:34 (Buenos Aires)
</commit_message>
<xml_diff>
--- a/Master UOPs.xlsx
+++ b/Master UOPs.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
     <author>Matias Perez de la Torre</author>
   </authors>
@@ -44,27 +44,6 @@
 </t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="J189" authorId="0">
       <text>
@@ -78,27 +57,6 @@
 Acumula lo anterior</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="J190" authorId="0">
       <text>
@@ -113,27 +71,6 @@
 </t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="AB75" authorId="0">
       <text>
@@ -147,27 +84,6 @@
 ODP 0000-00004421 - Transferencia 21/05/2026</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="AB76" authorId="0">
       <text>
@@ -181,27 +97,6 @@
 ODP 0000-00004421 - Transferencia 21/05/2026</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="AB77" authorId="0">
       <text>
@@ -215,27 +110,6 @@
 ODP 0000-00004421 - Transferencia 21/05/2026</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="AB142" authorId="0">
       <text>
@@ -249,27 +123,6 @@
 ODP 0000-00004421 - Transferencia 21/05/2026</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="AB143" authorId="0">
       <text>
@@ -283,27 +136,6 @@
 ODP 0000-00004421 - Transferencia 21/05/2026</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="AB144" authorId="0">
       <text>
@@ -317,27 +149,6 @@
 ODP 0000-00004421 - Transferencia 21/05/2026</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="AB145" authorId="0">
       <text>
@@ -351,27 +162,6 @@
 ODP 0000-00004421 - Transferencia 21/05/2026</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
     <comment ref="AB146" authorId="0">
       <text>
@@ -385,27 +175,6 @@
 ODP 0000-00004421 - Transferencia 21/05/2026</t>
         </r>
       </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>5</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>2</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-257</xdr:colOff>
-                <xdr:row>2</xdr:row>
-                <xdr:rowOff>19</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
@@ -1591,21 +1360,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="14">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_-&quot;$ &quot;* #,##0.00_-;&quot;-$ &quot;* #,##0.00_-;_-&quot;$ &quot;* \-??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="168" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="#,##0"/>
-    <numFmt numFmtId="170" formatCode="mm/yyyy"/>
-    <numFmt numFmtId="171" formatCode="#,##0.00"/>
-    <numFmt numFmtId="172" formatCode="0.00%"/>
-    <numFmt numFmtId="173" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="174" formatCode="0.0%"/>
-    <numFmt numFmtId="175" formatCode="0.0"/>
-    <numFmt numFmtId="176" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* \-??_ ;_-@_ "/>
-    <numFmt numFmtId="177" formatCode="mmm\-yy"/>
+    <numFmt numFmtId="168" formatCode="#,##0"/>
+    <numFmt numFmtId="169" formatCode="mm/yyyy"/>
+    <numFmt numFmtId="170" formatCode="#,##0.00"/>
+    <numFmt numFmtId="171" formatCode="0.00%"/>
+    <numFmt numFmtId="172" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="173" formatCode="0.0%"/>
+    <numFmt numFmtId="174" formatCode="0.0"/>
+    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* \-??_ ;_-@_ "/>
+    <numFmt numFmtId="176" formatCode="mmm\-yy"/>
   </numFmts>
   <fonts count="34">
     <font>
@@ -2047,10 +1815,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2071,339 +1836,339 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="5" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="6" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="8" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="5" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="11" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="10" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="12" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="13" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="13" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="13" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="9" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="14" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="15" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="16" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="16" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="16" fillId="16" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="16" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="16" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="15" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="17" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="17" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="17" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="10" fillId="17" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="18" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="18" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="19" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="20" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="22" fillId="21" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="22" fillId="21" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="19" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="26" fillId="22" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="26" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="26" fillId="22" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="26" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="27" fillId="22" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="27" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="27" fillId="23" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="27" fillId="23" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="22" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="26" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="26" fillId="22" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="26" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="28" fillId="22" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="28" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="29" fillId="22" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="29" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="26" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="26" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="26" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="26" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="27" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="27" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="26" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="28" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="28" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="29" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="29" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="26" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="26" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="19" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="30" fillId="19" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="30" fillId="19" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="31" fillId="0" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="24" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="32" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="31" fillId="24" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="31" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="5" borderId="0" xfId="22" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2411,11 +2176,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2435,15 +2200,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="33" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2451,15 +2216,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2808,9 +2573,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>210240</xdr:colOff>
+      <xdr:colOff>209880</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>38160</xdr:rowOff>
+      <xdr:rowOff>37800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2825,7 +2590,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10472040" y="10696680"/>
-          <a:ext cx="4845600" cy="2047680"/>
+          <a:ext cx="4845240" cy="2047320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2847,9 +2612,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1495080</xdr:colOff>
+      <xdr:colOff>1494720</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>25200</xdr:rowOff>
+      <xdr:rowOff>24840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2864,7 +2629,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4453560" y="6731280"/>
-          <a:ext cx="6011640" cy="6000120"/>
+          <a:ext cx="6011280" cy="5999760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3069,7 +2834,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:AL552"/>
+  <dimension ref="A1:AK552"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -3689,15 +3454,15 @@
       <c r="T6" s="24"/>
       <c r="U6" s="24" t="n">
         <f aca="false">+S6*21%</f>
-        <v>32344385.2880632</v>
+        <v>32344385.2880633</v>
       </c>
       <c r="V6" s="24" t="n">
         <f aca="false">+S6*3%</f>
-        <v>4620626.46972332</v>
+        <v>4620626.46972333</v>
       </c>
       <c r="W6" s="24" t="n">
         <f aca="false">+S6*2.5%</f>
-        <v>3850522.05810277</v>
+        <v>3850522.05810278</v>
       </c>
       <c r="X6" s="24" t="n">
         <f aca="false">IF(A6="00-175",S6*0.06,0)</f>
@@ -3873,15 +3638,15 @@
       <c r="T8" s="24"/>
       <c r="U8" s="24" t="n">
         <f aca="false">+S8*21%</f>
-        <v>22083915.8931225</v>
+        <v>22083915.8931224</v>
       </c>
       <c r="V8" s="24" t="n">
         <f aca="false">+S8*3%</f>
-        <v>3154845.12758893</v>
+        <v>3154845.12758892</v>
       </c>
       <c r="W8" s="24" t="n">
         <f aca="false">+S8*2.5%</f>
-        <v>2629037.60632411</v>
+        <v>2629037.6063241</v>
       </c>
       <c r="X8" s="24" t="n">
         <f aca="false">IF(A8="00-175",S8*0.06,0)</f>
@@ -3891,7 +3656,7 @@
       <c r="Z8" s="24"/>
       <c r="AA8" s="24" t="n">
         <f aca="false">+S8+T8+U8+W8+X8+V8+Y8</f>
-        <v>133029302.88</v>
+        <v>133029302.879999</v>
       </c>
       <c r="AB8" s="27"/>
       <c r="AC8" s="24"/>
@@ -3906,7 +3671,7 @@
       </c>
       <c r="AJ8" s="13" t="n">
         <f aca="false">+AA8-AI8</f>
-        <v>133029302.88</v>
+        <v>133029302.879999</v>
       </c>
       <c r="AK8" s="19" t="str">
         <f aca="false">IF(Q8="ANULADA","N/A",IF(ABS(AJ8)&gt;10,"Pendiente",IF(MAX(AB8,AD8,AF8)=0,"Pendiente",MAX(0,MAX(AB8,AD8,AF8)-O8))))</f>
@@ -3965,15 +3730,15 @@
       <c r="T9" s="24"/>
       <c r="U9" s="24" t="n">
         <f aca="false">+S9*21%</f>
-        <v>22070146.9501186</v>
+        <v>22070146.9501187</v>
       </c>
       <c r="V9" s="24" t="n">
         <f aca="false">+S9*3%</f>
-        <v>3152878.13573123</v>
+        <v>3152878.13573124</v>
       </c>
       <c r="W9" s="24" t="n">
         <f aca="false">+S9*2.5%</f>
-        <v>2627398.44644269</v>
+        <v>2627398.4464427</v>
       </c>
       <c r="X9" s="24" t="n">
         <f aca="false">IF(A9="00-175",S9*0.06,0)</f>
@@ -3983,7 +3748,7 @@
       <c r="Z9" s="24"/>
       <c r="AA9" s="24" t="n">
         <f aca="false">+S9+T9+U9+W9+X9+V9+Y9</f>
-        <v>132946361.39</v>
+        <v>132946361.390001</v>
       </c>
       <c r="AB9" s="27"/>
       <c r="AC9" s="24"/>
@@ -3998,7 +3763,7 @@
       </c>
       <c r="AJ9" s="13" t="n">
         <f aca="false">+AA9-AI9</f>
-        <v>132946361.39</v>
+        <v>132946361.390001</v>
       </c>
       <c r="AK9" s="19" t="str">
         <f aca="false">IF(Q9="ANULADA","N/A",IF(ABS(AJ9)&gt;10,"Pendiente",IF(MAX(AB9,AD9,AF9)=0,"Pendiente",MAX(0,MAX(AB9,AD9,AF9)-O9))))</f>
@@ -4057,15 +3822,15 @@
       <c r="T10" s="24"/>
       <c r="U10" s="24" t="n">
         <f aca="false">+S10*21%</f>
-        <v>22583360.30917</v>
+        <v>22583360.3091699</v>
       </c>
       <c r="V10" s="24" t="n">
         <f aca="false">+S10*3%</f>
-        <v>3226194.32988142</v>
+        <v>3226194.32988141</v>
       </c>
       <c r="W10" s="24" t="n">
         <f aca="false">+S10*2.5%</f>
-        <v>2688495.27490119</v>
+        <v>2688495.27490118</v>
       </c>
       <c r="X10" s="24" t="n">
         <f aca="false">IF(A10="00-175",S10*0.06,0)</f>
@@ -4075,7 +3840,7 @@
       <c r="Z10" s="24"/>
       <c r="AA10" s="24" t="n">
         <f aca="false">+S10+T10+U10+W10+X10+V10+Y10</f>
-        <v>136037860.91</v>
+        <v>136037860.909999</v>
       </c>
       <c r="AB10" s="27"/>
       <c r="AC10" s="24"/>
@@ -4090,7 +3855,7 @@
       </c>
       <c r="AJ10" s="13" t="n">
         <f aca="false">+AA10-AI10</f>
-        <v>136037860.91</v>
+        <v>136037860.909999</v>
       </c>
       <c r="AK10" s="19" t="str">
         <f aca="false">IF(Q10="ANULADA","N/A",IF(ABS(AJ10)&gt;10,"Pendiente",IF(MAX(AB10,AD10,AF10)=0,"Pendiente",MAX(0,MAX(AB10,AD10,AF10)-O10))))</f>
@@ -4153,11 +3918,11 @@
       </c>
       <c r="V11" s="24" t="n">
         <f aca="false">+S11*3%</f>
-        <v>3101317.53557312</v>
+        <v>3101317.53557313</v>
       </c>
       <c r="W11" s="24" t="n">
         <f aca="false">+S11*2.5%</f>
-        <v>2584431.27964427</v>
+        <v>2584431.27964428</v>
       </c>
       <c r="X11" s="24" t="n">
         <f aca="false">IF(A11="00-175",S11*0.06,0)</f>
@@ -4333,15 +4098,15 @@
       <c r="T13" s="24"/>
       <c r="U13" s="24" t="n">
         <f aca="false">+S13*21%</f>
-        <v>3704858.2913834</v>
+        <v>3704858.29138341</v>
       </c>
       <c r="V13" s="24" t="n">
         <f aca="false">+S13*3%</f>
-        <v>529265.470197629</v>
+        <v>529265.47019763</v>
       </c>
       <c r="W13" s="24" t="n">
         <f aca="false">+S13*2.5%</f>
-        <v>441054.558498024</v>
+        <v>441054.558498025</v>
       </c>
       <c r="X13" s="24" t="n">
         <f aca="false">IF(A13="00-175",S13*0.06,0)</f>
@@ -4351,7 +4116,7 @@
       <c r="Z13" s="24"/>
       <c r="AA13" s="24" t="n">
         <f aca="false">+S13+T13+U13+W13+X13+V13+Y13</f>
-        <v>22317360.66</v>
+        <v>22317360.6600001</v>
       </c>
       <c r="AB13" s="27"/>
       <c r="AC13" s="24"/>
@@ -4366,7 +4131,7 @@
       </c>
       <c r="AJ13" s="13" t="n">
         <f aca="false">+AA13-AI13</f>
-        <v>22317360.66</v>
+        <v>22317360.6600001</v>
       </c>
       <c r="AK13" s="19" t="str">
         <f aca="false">IF(Q13="ANULADA","N/A",IF(ABS(AJ13)&gt;10,"Pendiente",IF(MAX(AB13,AD13,AF13)=0,"Pendiente",MAX(0,MAX(AB13,AD13,AF13)-O13))))</f>
@@ -4429,11 +4194,11 @@
       </c>
       <c r="V14" s="24" t="n">
         <f aca="false">+S14*3%</f>
-        <v>872506.024031621</v>
+        <v>872506.024031622</v>
       </c>
       <c r="W14" s="24" t="n">
         <f aca="false">+S14*2.5%</f>
-        <v>727088.353359684</v>
+        <v>727088.353359685</v>
       </c>
       <c r="X14" s="24" t="n">
         <f aca="false">IF(A14="00-175",S14*0.06,0)</f>
@@ -4443,7 +4208,7 @@
       <c r="Z14" s="24"/>
       <c r="AA14" s="24" t="n">
         <f aca="false">+S14+T14+U14+W14+X14+V14+Y14</f>
-        <v>36790670.68</v>
+        <v>36790670.6800001</v>
       </c>
       <c r="AB14" s="27"/>
       <c r="AC14" s="24"/>
@@ -4458,7 +4223,7 @@
       </c>
       <c r="AJ14" s="13" t="n">
         <f aca="false">+AA14-AI14</f>
-        <v>36790670.68</v>
+        <v>36790670.6800001</v>
       </c>
       <c r="AK14" s="19" t="str">
         <f aca="false">IF(Q14="ANULADA","N/A",IF(ABS(AJ14)&gt;10,"Pendiente",IF(MAX(AB14,AD14,AF14)=0,"Pendiente",MAX(0,MAX(AB14,AD14,AF14)-O14))))</f>
@@ -4517,15 +4282,15 @@
       <c r="T15" s="24"/>
       <c r="U15" s="24" t="n">
         <f aca="false">+S15*21%</f>
-        <v>3555224.45312253</v>
+        <v>3555224.45312252</v>
       </c>
       <c r="V15" s="24" t="n">
         <f aca="false">+S15*3%</f>
-        <v>507889.207588933</v>
+        <v>507889.207588932</v>
       </c>
       <c r="W15" s="24" t="n">
         <f aca="false">+S15*2.5%</f>
-        <v>423241.006324111</v>
+        <v>423241.00632411</v>
       </c>
       <c r="X15" s="24" t="n">
         <f aca="false">IF(A15="00-175",S15*0.06,0)</f>
@@ -4701,15 +4466,15 @@
       <c r="T17" s="24"/>
       <c r="U17" s="24" t="n">
         <f aca="false">+S17*21%</f>
-        <v>6160959.39177866</v>
+        <v>6160959.39177867</v>
       </c>
       <c r="V17" s="24" t="n">
         <f aca="false">+S17*3%</f>
-        <v>880137.055968379</v>
+        <v>880137.055968381</v>
       </c>
       <c r="W17" s="24" t="n">
         <f aca="false">+S17*2.5%</f>
-        <v>733447.546640316</v>
+        <v>733447.546640318</v>
       </c>
       <c r="X17" s="24" t="n">
         <f aca="false">IF(A17="00-175",S17*0.06,0)</f>
@@ -4719,7 +4484,7 @@
       <c r="Z17" s="24"/>
       <c r="AA17" s="24" t="n">
         <f aca="false">+S17+T17+U17+W17+X17+V17+Y17</f>
-        <v>37112445.86</v>
+        <v>37112445.8600001</v>
       </c>
       <c r="AB17" s="27"/>
       <c r="AC17" s="24"/>
@@ -4734,7 +4499,7 @@
       </c>
       <c r="AJ17" s="13" t="n">
         <f aca="false">+AA17-AI17</f>
-        <v>37112445.86</v>
+        <v>37112445.8600001</v>
       </c>
       <c r="AK17" s="19" t="str">
         <f aca="false">IF(Q17="ANULADA","N/A",IF(ABS(AJ17)&gt;10,"Pendiente",IF(MAX(AB17,AD17,AF17)=0,"Pendiente",MAX(0,MAX(AB17,AD17,AF17)-O17))))</f>
@@ -4793,15 +4558,15 @@
       <c r="T18" s="24"/>
       <c r="U18" s="24" t="n">
         <f aca="false">+S18*21%</f>
-        <v>6831568.34347826</v>
+        <v>6831568.34347827</v>
       </c>
       <c r="V18" s="24" t="n">
         <f aca="false">+S18*3%</f>
-        <v>975938.334782609</v>
+        <v>975938.33478261</v>
       </c>
       <c r="W18" s="24" t="n">
         <f aca="false">+S18*2.5%</f>
-        <v>813281.945652174</v>
+        <v>813281.945652175</v>
       </c>
       <c r="X18" s="24" t="n">
         <f aca="false">IF(A18="00-175",S18*0.06,0)</f>
@@ -4811,7 +4576,7 @@
       <c r="Z18" s="24"/>
       <c r="AA18" s="24" t="n">
         <f aca="false">+S18+T18+U18+W18+X18+V18+Y18</f>
-        <v>41152066.45</v>
+        <v>41152066.4500001</v>
       </c>
       <c r="AB18" s="27"/>
       <c r="AC18" s="24"/>
@@ -4826,7 +4591,7 @@
       </c>
       <c r="AJ18" s="13" t="n">
         <f aca="false">+AA18-AI18</f>
-        <v>41152066.45</v>
+        <v>41152066.4500001</v>
       </c>
       <c r="AK18" s="19" t="str">
         <f aca="false">IF(Q18="ANULADA","N/A",IF(ABS(AJ18)&gt;10,"Pendiente",IF(MAX(AB18,AD18,AF18)=0,"Pendiente",MAX(0,MAX(AB18,AD18,AF18)-O18))))</f>
@@ -4885,15 +4650,15 @@
       <c r="T19" s="24"/>
       <c r="U19" s="24" t="n">
         <f aca="false">+S19*21%</f>
-        <v>2488551.57533597</v>
+        <v>2488551.57533596</v>
       </c>
       <c r="V19" s="24" t="n">
         <f aca="false">+S19*3%</f>
-        <v>355507.367905138</v>
+        <v>355507.367905137</v>
       </c>
       <c r="W19" s="24" t="n">
         <f aca="false">+S19*2.5%</f>
-        <v>296256.139920949</v>
+        <v>296256.139920948</v>
       </c>
       <c r="X19" s="24" t="n">
         <f aca="false">IF(A19="00-175",S19*0.06,0)</f>
@@ -4903,7 +4668,7 @@
       <c r="Z19" s="24"/>
       <c r="AA19" s="24" t="n">
         <f aca="false">+S19+T19+U19+W19+X19+V19+Y19</f>
-        <v>14990560.68</v>
+        <v>14990560.6799999</v>
       </c>
       <c r="AB19" s="27"/>
       <c r="AC19" s="24"/>
@@ -4918,7 +4683,7 @@
       </c>
       <c r="AJ19" s="13" t="n">
         <f aca="false">+AA19-AI19</f>
-        <v>14990560.68</v>
+        <v>14990560.6799999</v>
       </c>
       <c r="AK19" s="19" t="str">
         <f aca="false">IF(Q19="ANULADA","N/A",IF(ABS(AJ19)&gt;10,"Pendiente",IF(MAX(AB19,AD19,AF19)=0,"Pendiente",MAX(0,MAX(AB19,AD19,AF19)-O19))))</f>
@@ -4981,7 +4746,7 @@
       </c>
       <c r="V20" s="24" t="n">
         <f aca="false">+S20*3%</f>
-        <v>1667862.68134387</v>
+        <v>1667862.68134388</v>
       </c>
       <c r="W20" s="24" t="n">
         <f aca="false">+S20*2.5%</f>
@@ -4995,7 +4760,7 @@
       <c r="Z20" s="24"/>
       <c r="AA20" s="24" t="n">
         <f aca="false">+S20+T20+U20+W20+X20+V20+Y20</f>
-        <v>70328209.73</v>
+        <v>70328209.7300001</v>
       </c>
       <c r="AB20" s="27"/>
       <c r="AC20" s="24"/>
@@ -5010,7 +4775,7 @@
       </c>
       <c r="AJ20" s="13" t="n">
         <f aca="false">+AA20-AI20</f>
-        <v>70328209.73</v>
+        <v>70328209.7300001</v>
       </c>
       <c r="AK20" s="19" t="str">
         <f aca="false">IF(Q20="ANULADA","N/A",IF(ABS(AJ20)&gt;10,"Pendiente",IF(MAX(AB20,AD20,AF20)=0,"Pendiente",MAX(0,MAX(AB20,AD20,AF20)-O20))))</f>
@@ -5077,7 +4842,7 @@
       </c>
       <c r="W21" s="24" t="n">
         <f aca="false">+S21*2.5%</f>
-        <v>1872334.83517787</v>
+        <v>1872334.83517786</v>
       </c>
       <c r="X21" s="24" t="n">
         <f aca="false">IF(A21="00-175",S21*0.06,0)</f>
@@ -5165,11 +4930,11 @@
       </c>
       <c r="V22" s="24" t="n">
         <f aca="false">+S22*3%</f>
-        <v>5964546.69557312</v>
+        <v>5964546.69557313</v>
       </c>
       <c r="W22" s="24" t="n">
         <f aca="false">+S22*2.5%</f>
-        <v>4970455.57964427</v>
+        <v>4970455.57964428</v>
       </c>
       <c r="X22" s="24" t="n">
         <f aca="false">IF(A22="00-175",S22*0.06,0)</f>
@@ -5253,15 +5018,15 @@
       <c r="T23" s="24"/>
       <c r="U23" s="24" t="n">
         <f aca="false">+S23*21%</f>
-        <v>40435927.5052174</v>
+        <v>40435927.5052175</v>
       </c>
       <c r="V23" s="24" t="n">
         <f aca="false">+S23*3%</f>
-        <v>5776561.07217392</v>
+        <v>5776561.07217393</v>
       </c>
       <c r="W23" s="24" t="n">
         <f aca="false">+S23*2.5%</f>
-        <v>4813800.89347826</v>
+        <v>4813800.89347828</v>
       </c>
       <c r="X23" s="24" t="n">
         <f aca="false">IF(A23="00-175",S23*0.06,0)</f>
@@ -5271,7 +5036,7 @@
       <c r="Z23" s="24"/>
       <c r="AA23" s="24" t="n">
         <f aca="false">+S23+T23+U23+W23+X23+V23+Y23</f>
-        <v>243578325.21</v>
+        <v>243578325.210001</v>
       </c>
       <c r="AB23" s="27"/>
       <c r="AC23" s="24"/>
@@ -5286,7 +5051,7 @@
       </c>
       <c r="AJ23" s="13" t="n">
         <f aca="false">+AA23-AI23</f>
-        <v>243578325.21</v>
+        <v>243578325.210001</v>
       </c>
       <c r="AK23" s="19" t="str">
         <f aca="false">IF(Q23="ANULADA","N/A",IF(ABS(AJ23)&gt;10,"Pendiente",IF(MAX(AB23,AD23,AF23)=0,"Pendiente",MAX(0,MAX(AB23,AD23,AF23)-O23))))</f>
@@ -5561,7 +5326,7 @@
       <c r="T26" s="13"/>
       <c r="U26" s="13" t="n">
         <f aca="false">+S26*21%</f>
-        <v>883270.512893323</v>
+        <v>883270.512893324</v>
       </c>
       <c r="V26" s="13" t="n">
         <f aca="false">+S26*3%</f>
@@ -6085,15 +5850,15 @@
       </c>
       <c r="V31" s="13" t="n">
         <f aca="false">+S31*3%</f>
-        <v>3906628.93699156</v>
+        <v>3906628.93699155</v>
       </c>
       <c r="W31" s="13" t="n">
         <f aca="false">+S31*0.3%</f>
-        <v>390662.893699156</v>
+        <v>390662.893699155</v>
       </c>
       <c r="X31" s="13" t="n">
         <f aca="false">IF(A31="00-175",S31*0.06,0)</f>
-        <v>7813257.87398312</v>
+        <v>7813257.8739831</v>
       </c>
       <c r="Y31" s="13"/>
       <c r="Z31" s="13"/>
@@ -6185,19 +5950,19 @@
       <c r="T32" s="13"/>
       <c r="U32" s="13" t="n">
         <f aca="false">+S32*21%</f>
-        <v>2149758.48465081</v>
+        <v>2149758.4846508</v>
       </c>
       <c r="V32" s="13" t="n">
         <f aca="false">+S32*3%</f>
-        <v>307108.354950115</v>
+        <v>307108.354950114</v>
       </c>
       <c r="W32" s="13" t="n">
         <f aca="false">+S32*0.3%</f>
-        <v>30710.8354950115</v>
+        <v>30710.8354950114</v>
       </c>
       <c r="X32" s="13" t="n">
         <f aca="false">IF(A32="00-175",S32*0.06,0)</f>
-        <v>614216.70990023</v>
+        <v>614216.709900228</v>
       </c>
       <c r="Y32" s="13"/>
       <c r="Z32" s="13"/>
@@ -6301,7 +6066,7 @@
       </c>
       <c r="X33" s="13" t="n">
         <f aca="false">IF(A33="00-175",S33*0.06,0)</f>
-        <v>667874.764696853</v>
+        <v>667874.764696854</v>
       </c>
       <c r="Y33" s="13"/>
       <c r="Z33" s="13"/>
@@ -6411,7 +6176,7 @@
       <c r="Z34" s="13"/>
       <c r="AA34" s="13" t="n">
         <f aca="false">+S34+T34+U34+W34+X34+V34+Y34</f>
-        <v>855594.31</v>
+        <v>855594.310000001</v>
       </c>
       <c r="AB34" s="29" t="n">
         <v>45917</v>
@@ -6501,15 +6266,15 @@
       </c>
       <c r="V35" s="13" t="n">
         <f aca="false">+S35*3%</f>
-        <v>3945378.96469685</v>
+        <v>3945378.96469686</v>
       </c>
       <c r="W35" s="13" t="n">
         <f aca="false">+S35*0.3%</f>
-        <v>394537.896469685</v>
+        <v>394537.896469686</v>
       </c>
       <c r="X35" s="13" t="n">
         <f aca="false">IF(A35="00-175",S35*0.06,0)</f>
-        <v>7890757.92939371</v>
+        <v>7890757.92939372</v>
       </c>
       <c r="Y35" s="13"/>
       <c r="Z35" s="13"/>
@@ -6609,15 +6374,15 @@
       </c>
       <c r="V36" s="13" t="n">
         <f aca="false">+S36*3%</f>
-        <v>439958.704834996</v>
+        <v>439958.704834995</v>
       </c>
       <c r="W36" s="13" t="n">
         <f aca="false">+S36*0.3%</f>
-        <v>43995.8704834996</v>
+        <v>43995.8704834995</v>
       </c>
       <c r="X36" s="13" t="n">
         <f aca="false">IF(A36="00-175",S36*0.06,0)</f>
-        <v>879917.409669992</v>
+        <v>879917.40966999</v>
       </c>
       <c r="Y36" s="13"/>
       <c r="Z36" s="13"/>
@@ -7021,7 +6786,7 @@
       <c r="T40" s="13"/>
       <c r="U40" s="13" t="n">
         <f aca="false">+S40*21%</f>
-        <v>79758.515732924</v>
+        <v>79758.5157329241</v>
       </c>
       <c r="V40" s="13" t="n">
         <f aca="false">+S40*3%</f>
@@ -7129,11 +6894,11 @@
       </c>
       <c r="V41" s="13" t="n">
         <f aca="false">+S41*3%</f>
-        <v>5467254.33131236</v>
+        <v>5467254.33131235</v>
       </c>
       <c r="W41" s="13" t="n">
         <f aca="false">+S41*0.3%</f>
-        <v>546725.433131236</v>
+        <v>546725.433131235</v>
       </c>
       <c r="X41" s="13" t="n">
         <f aca="false">IF(A41="00-175",S41*0.06,0)</f>
@@ -7229,15 +6994,15 @@
       <c r="T42" s="13"/>
       <c r="U42" s="13" t="n">
         <f aca="false">+S42*21%</f>
-        <v>4604456.77505756</v>
+        <v>4604456.77505755</v>
       </c>
       <c r="V42" s="13" t="n">
         <f aca="false">+S42*3%</f>
-        <v>657779.539293937</v>
+        <v>657779.539293936</v>
       </c>
       <c r="W42" s="13" t="n">
         <f aca="false">+S42*0.3%</f>
-        <v>65777.9539293937</v>
+        <v>65777.9539293936</v>
       </c>
       <c r="X42" s="13" t="n">
         <f aca="false">IF(A42="00-175",S42*0.06,0)</f>
@@ -7349,7 +7114,7 @@
       </c>
       <c r="X43" s="13" t="n">
         <f aca="false">IF(A43="00-175",S43*0.06,0)</f>
-        <v>2912509.59324636</v>
+        <v>2912509.59324635</v>
       </c>
       <c r="Y43" s="13"/>
       <c r="Z43" s="13"/>
@@ -7445,11 +7210,11 @@
       </c>
       <c r="V44" s="13" t="n">
         <f aca="false">+S44*3%</f>
-        <v>97860.3223330775</v>
+        <v>97860.3223330776</v>
       </c>
       <c r="W44" s="13" t="n">
         <f aca="false">+S44*0.3%</f>
-        <v>9786.03223330775</v>
+        <v>9786.03223330776</v>
       </c>
       <c r="X44" s="13" t="n">
         <f aca="false">IF(A44="00-175",S44*0.06,0)</f>
@@ -14129,7 +13894,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="20" t="s">
         <v>186</v>
       </c>
@@ -14217,7 +13982,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="20" t="s">
         <v>186</v>
       </c>
@@ -18408,7 +18173,6 @@
         <f aca="false">IF(Q154="ANULADA","N/A",IF(ABS(AJ154)&gt;10,"Pendiente",IF(MAX(AB154,AD154,AF154)=0,"Pendiente",MAX(0,MAX(AB154,AD154,AF154)-O154))))</f>
         <v>Pendiente</v>
       </c>
-      <c r="AL154" s="41"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="20" t="s">
@@ -19216,7 +18980,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="20" t="s">
         <v>263</v>
       </c>
@@ -19316,7 +19080,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="36" t="s">
         <v>263</v>
       </c>
@@ -19349,7 +19113,7 @@
       <c r="N164" s="36" t="n">
         <v>2007</v>
       </c>
-      <c r="O164" s="42" t="n">
+      <c r="O164" s="41" t="n">
         <v>46041</v>
       </c>
       <c r="P164" s="36" t="s">
@@ -19408,7 +19172,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="20" t="s">
         <v>263</v>
       </c>
@@ -19510,7 +19274,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="36" t="s">
         <v>263</v>
       </c>
@@ -19543,7 +19307,7 @@
       <c r="N166" s="36" t="n">
         <v>2009</v>
       </c>
-      <c r="O166" s="42" t="n">
+      <c r="O166" s="41" t="n">
         <v>46051</v>
       </c>
       <c r="P166" s="36" t="s">
@@ -19602,7 +19366,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="20" t="s">
         <v>263</v>
       </c>
@@ -19702,7 +19466,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="20" t="s">
         <v>263</v>
       </c>
@@ -19804,7 +19568,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="20" t="s">
         <v>263</v>
       </c>
@@ -19904,7 +19668,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="20" t="s">
         <v>263</v>
       </c>
@@ -19996,7 +19760,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="20" t="s">
         <v>263</v>
       </c>
@@ -20088,7 +19852,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="20" t="s">
         <v>263</v>
       </c>
@@ -20187,7 +19951,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="20" t="s">
         <v>263</v>
       </c>
@@ -20279,7 +20043,7 @@
         <v>N/A</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="20" t="s">
         <v>263</v>
       </c>
@@ -21932,19 +21696,18 @@
         <f aca="false">IF(Q190="ANULADA","N/A",IF(ABS(AJ190)&gt;10,"Pendiente",IF(MAX(AB190,AD190,AF190)=0,"Pendiente",MAX(0,MAX(AB190,AD190,AF190)-O190))))</f>
         <v>21</v>
       </c>
-      <c r="AL190" s="41"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A191" s="43" t="s">
+      <c r="A191" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B191" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C191" s="43" t="s">
+      <c r="C191" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D191" s="43" t="s">
+      <c r="D191" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E191" s="11" t="n">
@@ -21969,7 +21732,7 @@
       <c r="L191" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M191" s="43" t="s">
+      <c r="M191" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N191" s="35" t="n">
@@ -21978,7 +21741,7 @@
       <c r="O191" s="15" t="n">
         <v>46367</v>
       </c>
-      <c r="P191" s="43" t="s">
+      <c r="P191" s="42" t="s">
         <v>303</v>
       </c>
       <c r="Q191" s="16" t="s">
@@ -22022,7 +21785,7 @@
       </c>
       <c r="AD191" s="18"/>
       <c r="AE191" s="13"/>
-      <c r="AF191" s="43"/>
+      <c r="AF191" s="42"/>
       <c r="AG191" s="13"/>
       <c r="AH191" s="13"/>
       <c r="AI191" s="13" t="n">
@@ -22039,16 +21802,16 @@
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A192" s="43" t="s">
+      <c r="A192" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B192" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C192" s="43" t="s">
+      <c r="C192" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D192" s="43" t="s">
+      <c r="D192" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E192" s="11" t="n">
@@ -22073,7 +21836,7 @@
       <c r="L192" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M192" s="43" t="s">
+      <c r="M192" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N192" s="35" t="n">
@@ -22082,7 +21845,7 @@
       <c r="O192" s="15" t="n">
         <v>46367</v>
       </c>
-      <c r="P192" s="43" t="s">
+      <c r="P192" s="42" t="s">
         <v>304</v>
       </c>
       <c r="Q192" s="16" t="s">
@@ -22126,7 +21889,7 @@
       </c>
       <c r="AD192" s="18"/>
       <c r="AE192" s="13"/>
-      <c r="AF192" s="43"/>
+      <c r="AF192" s="42"/>
       <c r="AG192" s="13"/>
       <c r="AH192" s="13"/>
       <c r="AI192" s="13" t="n">
@@ -22143,16 +21906,16 @@
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A193" s="43" t="s">
+      <c r="A193" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B193" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C193" s="43" t="s">
+      <c r="C193" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D193" s="43" t="s">
+      <c r="D193" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E193" s="11" t="n">
@@ -22177,7 +21940,7 @@
       <c r="L193" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M193" s="43" t="s">
+      <c r="M193" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N193" s="35" t="n">
@@ -22186,7 +21949,7 @@
       <c r="O193" s="15" t="n">
         <v>46053</v>
       </c>
-      <c r="P193" s="43" t="s">
+      <c r="P193" s="42" t="s">
         <v>305</v>
       </c>
       <c r="Q193" s="16" t="s">
@@ -22230,7 +21993,7 @@
       </c>
       <c r="AD193" s="18"/>
       <c r="AE193" s="13"/>
-      <c r="AF193" s="43"/>
+      <c r="AF193" s="42"/>
       <c r="AG193" s="13"/>
       <c r="AH193" s="13"/>
       <c r="AI193" s="13" t="n">
@@ -22247,16 +22010,16 @@
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A194" s="43" t="s">
+      <c r="A194" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B194" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C194" s="43" t="s">
+      <c r="C194" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D194" s="43" t="s">
+      <c r="D194" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E194" s="11" t="n">
@@ -22281,7 +22044,7 @@
       <c r="L194" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M194" s="43" t="s">
+      <c r="M194" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N194" s="35" t="n">
@@ -22290,7 +22053,7 @@
       <c r="O194" s="15" t="n">
         <v>46053</v>
       </c>
-      <c r="P194" s="43" t="s">
+      <c r="P194" s="42" t="s">
         <v>306</v>
       </c>
       <c r="Q194" s="16" t="s">
@@ -22334,7 +22097,7 @@
       </c>
       <c r="AD194" s="18"/>
       <c r="AE194" s="13"/>
-      <c r="AF194" s="43"/>
+      <c r="AF194" s="42"/>
       <c r="AG194" s="13"/>
       <c r="AH194" s="13"/>
       <c r="AI194" s="13" t="n">
@@ -22351,16 +22114,16 @@
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A195" s="43" t="s">
+      <c r="A195" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B195" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C195" s="43" t="s">
+      <c r="C195" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D195" s="43" t="s">
+      <c r="D195" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E195" s="11" t="n">
@@ -22385,7 +22148,7 @@
       <c r="L195" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M195" s="43" t="s">
+      <c r="M195" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N195" s="35" t="n">
@@ -22394,7 +22157,7 @@
       <c r="O195" s="15" t="n">
         <v>46108</v>
       </c>
-      <c r="P195" s="43" t="s">
+      <c r="P195" s="42" t="s">
         <v>307</v>
       </c>
       <c r="Q195" s="16" t="s">
@@ -22438,7 +22201,7 @@
       </c>
       <c r="AD195" s="18"/>
       <c r="AE195" s="13"/>
-      <c r="AF195" s="43"/>
+      <c r="AF195" s="42"/>
       <c r="AG195" s="13"/>
       <c r="AH195" s="13"/>
       <c r="AI195" s="13" t="n">
@@ -22455,16 +22218,16 @@
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A196" s="43" t="s">
+      <c r="A196" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B196" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C196" s="43" t="s">
+      <c r="C196" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D196" s="43" t="s">
+      <c r="D196" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E196" s="11" t="n">
@@ -22489,7 +22252,7 @@
       <c r="L196" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M196" s="43" t="s">
+      <c r="M196" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N196" s="35" t="n">
@@ -22498,7 +22261,7 @@
       <c r="O196" s="15" t="n">
         <v>46108</v>
       </c>
-      <c r="P196" s="43" t="s">
+      <c r="P196" s="42" t="s">
         <v>308</v>
       </c>
       <c r="Q196" s="16" t="s">
@@ -22542,7 +22305,7 @@
       </c>
       <c r="AD196" s="18"/>
       <c r="AE196" s="13"/>
-      <c r="AF196" s="43"/>
+      <c r="AF196" s="42"/>
       <c r="AG196" s="13"/>
       <c r="AH196" s="13"/>
       <c r="AI196" s="13" t="n">
@@ -22559,16 +22322,16 @@
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A197" s="43" t="s">
+      <c r="A197" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B197" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C197" s="43" t="s">
+      <c r="C197" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D197" s="43" t="s">
+      <c r="D197" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E197" s="11" t="n">
@@ -22593,7 +22356,7 @@
       <c r="L197" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M197" s="43" t="s">
+      <c r="M197" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N197" s="35" t="n">
@@ -22602,7 +22365,7 @@
       <c r="O197" s="15" t="n">
         <v>46108</v>
       </c>
-      <c r="P197" s="43" t="s">
+      <c r="P197" s="42" t="s">
         <v>309</v>
       </c>
       <c r="Q197" s="16" t="s">
@@ -22650,7 +22413,7 @@
       <c r="AE197" s="13" t="n">
         <v>129995926.5</v>
       </c>
-      <c r="AF197" s="43"/>
+      <c r="AF197" s="42"/>
       <c r="AG197" s="13"/>
       <c r="AH197" s="13"/>
       <c r="AI197" s="13" t="n">
@@ -22667,16 +22430,16 @@
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A198" s="43" t="s">
+      <c r="A198" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B198" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C198" s="43" t="s">
+      <c r="C198" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D198" s="43" t="s">
+      <c r="D198" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E198" s="11"/>
@@ -22695,7 +22458,7 @@
         <v>0</v>
       </c>
       <c r="L198" s="11"/>
-      <c r="M198" s="43" t="s">
+      <c r="M198" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N198" s="35" t="n">
@@ -22704,7 +22467,7 @@
       <c r="O198" s="15" t="n">
         <v>46108</v>
       </c>
-      <c r="P198" s="43" t="s">
+      <c r="P198" s="42" t="s">
         <v>310</v>
       </c>
       <c r="Q198" s="16" t="s">
@@ -22744,7 +22507,7 @@
       <c r="AC198" s="13"/>
       <c r="AD198" s="18"/>
       <c r="AE198" s="13"/>
-      <c r="AF198" s="43"/>
+      <c r="AF198" s="42"/>
       <c r="AG198" s="13"/>
       <c r="AH198" s="13"/>
       <c r="AI198" s="13" t="n">
@@ -22761,16 +22524,16 @@
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A199" s="43" t="s">
+      <c r="A199" s="42" t="s">
         <v>301</v>
       </c>
       <c r="B199" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="C199" s="43" t="s">
+      <c r="C199" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="D199" s="43" t="s">
+      <c r="D199" s="42" t="s">
         <v>302</v>
       </c>
       <c r="E199" s="11" t="n">
@@ -22795,7 +22558,7 @@
       <c r="L199" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M199" s="43" t="s">
+      <c r="M199" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N199" s="35" t="n">
@@ -22804,7 +22567,7 @@
       <c r="O199" s="15" t="n">
         <v>46108</v>
       </c>
-      <c r="P199" s="43" t="s">
+      <c r="P199" s="42" t="s">
         <v>310</v>
       </c>
       <c r="Q199" s="16" t="s">
@@ -22899,7 +22662,7 @@
       <c r="L200" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M200" s="43" t="s">
+      <c r="M200" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N200" s="22" t="n">
@@ -22999,7 +22762,7 @@
       <c r="L201" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M201" s="43" t="s">
+      <c r="M201" s="42" t="s">
         <v>41</v>
       </c>
       <c r="N201" s="22" t="n">
@@ -23863,13 +23626,13 @@
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A210" s="44" t="s">
+      <c r="A210" s="43" t="s">
         <v>324</v>
       </c>
       <c r="B210" s="20" t="s">
         <v>315</v>
       </c>
-      <c r="C210" s="44" t="s">
+      <c r="C210" s="43" t="s">
         <v>315</v>
       </c>
       <c r="D210" s="20" t="s">
@@ -23895,22 +23658,22 @@
       <c r="L210" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M210" s="44" t="s">
+      <c r="M210" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="N210" s="45" t="n">
+      <c r="N210" s="44" t="n">
         <v>2489</v>
       </c>
       <c r="O210" s="15" t="n">
         <v>45869</v>
       </c>
-      <c r="P210" s="44" t="s">
+      <c r="P210" s="43" t="s">
         <v>331</v>
       </c>
-      <c r="Q210" s="46" t="s">
+      <c r="Q210" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="R210" s="46" t="s">
+      <c r="R210" s="45" t="s">
         <v>44</v>
       </c>
       <c r="S210" s="13" t="n">
@@ -23941,7 +23704,7 @@
         <f aca="false">+S210+T210+U210+W210+X210+V210+Y210</f>
         <v>16996040.408</v>
       </c>
-      <c r="AB210" s="47" t="n">
+      <c r="AB210" s="46" t="n">
         <v>45877</v>
       </c>
       <c r="AC210" s="13" t="n">
@@ -23950,7 +23713,7 @@
       </c>
       <c r="AD210" s="18"/>
       <c r="AE210" s="13"/>
-      <c r="AF210" s="44"/>
+      <c r="AF210" s="43"/>
       <c r="AG210" s="13"/>
       <c r="AH210" s="13"/>
       <c r="AI210" s="13" t="n">
@@ -37898,7 +37661,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="535" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="535" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A535" s="20"/>
       <c r="B535" s="20"/>
       <c r="C535" s="20"/>
@@ -37940,7 +37703,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="536" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="536" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A536" s="20"/>
       <c r="B536" s="20"/>
       <c r="C536" s="20"/>
@@ -38490,15 +38253,15 @@
       <c r="A549" s="20"/>
       <c r="B549" s="20"/>
       <c r="C549" s="20"/>
-      <c r="D549" s="11"/>
-      <c r="E549" s="11"/>
-      <c r="F549" s="11"/>
-      <c r="G549" s="11"/>
+      <c r="D549" s="47"/>
+      <c r="E549" s="47"/>
+      <c r="F549" s="47"/>
+      <c r="G549" s="47"/>
       <c r="H549" s="21"/>
       <c r="I549" s="12"/>
       <c r="J549" s="13"/>
       <c r="K549" s="13"/>
-      <c r="L549" s="11"/>
+      <c r="L549" s="47"/>
       <c r="M549" s="20"/>
       <c r="N549" s="22"/>
       <c r="O549" s="15"/>
@@ -38532,15 +38295,15 @@
       <c r="A550" s="20"/>
       <c r="B550" s="20"/>
       <c r="C550" s="20"/>
-      <c r="D550" s="11"/>
-      <c r="E550" s="11"/>
-      <c r="F550" s="11"/>
-      <c r="G550" s="11"/>
+      <c r="D550" s="47"/>
+      <c r="E550" s="47"/>
+      <c r="F550" s="47"/>
+      <c r="G550" s="47"/>
       <c r="H550" s="21"/>
       <c r="I550" s="12"/>
       <c r="J550" s="13"/>
       <c r="K550" s="13"/>
-      <c r="L550" s="11"/>
+      <c r="L550" s="47"/>
       <c r="M550" s="20"/>
       <c r="N550" s="22"/>
       <c r="O550" s="15"/>
@@ -38574,15 +38337,15 @@
       <c r="A551" s="20"/>
       <c r="B551" s="20"/>
       <c r="C551" s="20"/>
-      <c r="D551" s="11"/>
-      <c r="E551" s="11"/>
-      <c r="F551" s="11"/>
-      <c r="G551" s="11"/>
+      <c r="D551" s="47"/>
+      <c r="E551" s="47"/>
+      <c r="F551" s="47"/>
+      <c r="G551" s="47"/>
       <c r="H551" s="21"/>
       <c r="I551" s="12"/>
       <c r="J551" s="13"/>
       <c r="K551" s="13"/>
-      <c r="L551" s="11"/>
+      <c r="L551" s="47"/>
       <c r="M551" s="20"/>
       <c r="N551" s="22"/>
       <c r="O551" s="15"/>
@@ -38616,15 +38379,15 @@
       <c r="A552" s="20"/>
       <c r="B552" s="23"/>
       <c r="C552" s="20"/>
-      <c r="D552" s="11"/>
-      <c r="E552" s="11"/>
-      <c r="F552" s="11"/>
-      <c r="G552" s="11"/>
+      <c r="D552" s="47"/>
+      <c r="E552" s="47"/>
+      <c r="F552" s="47"/>
+      <c r="G552" s="47"/>
       <c r="H552" s="21"/>
       <c r="I552" s="12"/>
       <c r="J552" s="37"/>
       <c r="K552" s="37"/>
-      <c r="L552" s="11"/>
+      <c r="L552" s="47"/>
       <c r="M552" s="20"/>
       <c r="N552" s="35"/>
       <c r="O552" s="15"/>
@@ -38829,18 +38592,18 @@
         <v>337</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="53" t="s">
         <v>338</v>
       </c>
       <c r="B5" s="54" t="n">
-        <v>0.2527</v>
+        <v>0.237</v>
       </c>
       <c r="C5" s="55" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="53" t="s">
         <v>340</v>
       </c>
@@ -38851,13 +38614,13 @@
         <v>341</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="57" t="s">
         <v>342</v>
       </c>
       <c r="B7" s="58" t="n">
         <f aca="true">TODAY()</f>
-        <v>46184</v>
+        <v>46185</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -38896,7 +38659,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="60" t="n">
         <v>1998</v>
       </c>
@@ -38920,25 +38683,25 @@
       </c>
       <c r="G10" s="60" t="n">
         <f aca="false">IF(F10="",MAX(0,$B$7-E10),MAX(0,F10-E10))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H10" s="64" t="n">
         <v>50402510.51</v>
       </c>
       <c r="I10" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J10" s="66" t="n">
         <f aca="false">H10*I10*(G10/365)</f>
-        <v>3474362.42516371</v>
+        <v>3318280.34946658</v>
       </c>
       <c r="K10" s="67" t="n">
         <f aca="false">H10+J10</f>
-        <v>53876872.9351637</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>53720790.8594666</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="68" t="n">
         <v>1999</v>
       </c>
@@ -38962,22 +38725,22 @@
       </c>
       <c r="G11" s="68" t="n">
         <f aca="false">IF(F11="",MAX(0,$B$7-E11),MAX(0,F11-E11))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H11" s="71" t="n">
         <v>677271.96</v>
       </c>
       <c r="I11" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J11" s="72" t="n">
         <f aca="false">H11*I11*(G11/365)</f>
-        <v>46685.933411474</v>
+        <v>44588.6169830137</v>
       </c>
       <c r="K11" s="73" t="n">
         <f aca="false">H11+J11</f>
-        <v>723957.893411474</v>
+        <v>721860.576983014</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -39004,25 +38767,25 @@
       </c>
       <c r="G12" s="60" t="n">
         <f aca="false">IF(F12="",MAX(0,$B$7-E12),MAX(0,F12-E12))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H12" s="64" t="n">
         <v>17699825.4</v>
       </c>
       <c r="I12" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J12" s="66" t="n">
         <f aca="false">H12*I12*(G12/365)</f>
-        <v>1220090.18359348</v>
+        <v>1165278.91606027</v>
       </c>
       <c r="K12" s="67" t="n">
         <f aca="false">H12+J12</f>
-        <v>18919915.5835935</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>18865104.3160603</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="68" t="n">
         <v>2001</v>
       </c>
@@ -39046,25 +38809,25 @@
       </c>
       <c r="G13" s="68" t="n">
         <f aca="false">IF(F13="",MAX(0,$B$7-E13),MAX(0,F13-E13))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H13" s="71" t="n">
         <v>1015907.94</v>
       </c>
       <c r="I13" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J13" s="72" t="n">
         <f aca="false">H13*I13*(G13/365)</f>
-        <v>70028.9001172109</v>
+        <v>66882.9254745205</v>
       </c>
       <c r="K13" s="73" t="n">
         <f aca="false">H13+J13</f>
-        <v>1085936.84011721</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1082790.86547452</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="60" t="n">
         <v>2002</v>
       </c>
@@ -39088,25 +38851,25 @@
       </c>
       <c r="G14" s="60" t="n">
         <f aca="false">IF(F14="",MAX(0,$B$7-E14),MAX(0,F14-E14))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H14" s="64" t="n">
         <v>27253875.19</v>
       </c>
       <c r="I14" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J14" s="66" t="n">
         <f aca="false">H14*I14*(G14/365)</f>
-        <v>1878673.08477522</v>
+        <v>1794275.67346767</v>
       </c>
       <c r="K14" s="67" t="n">
         <f aca="false">H14+J14</f>
-        <v>29132548.2747752</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>29048150.8634677</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="68" t="n">
         <v>2003</v>
       </c>
@@ -39130,25 +38893,25 @@
       </c>
       <c r="G15" s="68" t="n">
         <f aca="false">IF(F15="",MAX(0,$B$7-E15),MAX(0,F15-E15))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H15" s="71" t="n">
         <v>1015907.94</v>
       </c>
       <c r="I15" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J15" s="72" t="n">
         <f aca="false">H15*I15*(G15/365)</f>
-        <v>70028.9001172109</v>
+        <v>66882.9254745205</v>
       </c>
       <c r="K15" s="73" t="n">
         <f aca="false">H15+J15</f>
-        <v>1085936.84011721</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1082790.86547452</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="60" t="n">
         <v>2004</v>
       </c>
@@ -39172,25 +38935,25 @@
       </c>
       <c r="G16" s="60" t="n">
         <f aca="false">IF(F16="",MAX(0,$B$7-E16),MAX(0,F16-E16))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H16" s="64" t="n">
         <v>28627721.36</v>
       </c>
       <c r="I16" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J16" s="66" t="n">
         <f aca="false">H16*I16*(G16/365)</f>
-        <v>1973375.50064112</v>
+        <v>1884723.6829611</v>
       </c>
       <c r="K16" s="67" t="n">
         <f aca="false">H16+J16</f>
-        <v>30601096.8606411</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>30512445.0429611</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="68" t="n">
         <v>2005</v>
       </c>
@@ -39214,25 +38977,25 @@
       </c>
       <c r="G17" s="68" t="n">
         <f aca="false">IF(F17="",MAX(0,$B$7-E17),MAX(0,F17-E17))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H17" s="71" t="n">
         <v>238400.46</v>
       </c>
       <c r="I17" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J17" s="72" t="n">
         <f aca="false">H17*I17*(G17/365)</f>
-        <v>16433.4988869534</v>
+        <v>15695.2412432877</v>
       </c>
       <c r="K17" s="73" t="n">
         <f aca="false">H17+J17</f>
-        <v>254833.958886953</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>254095.701243288</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="60" t="n">
         <v>2006</v>
       </c>
@@ -39256,25 +39019,25 @@
       </c>
       <c r="G18" s="60" t="n">
         <f aca="false">IF(F18="",MAX(0,$B$7-E18),MAX(0,F18-E18))</f>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H18" s="64" t="n">
         <v>6758414.64</v>
       </c>
       <c r="I18" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J18" s="66" t="n">
         <f aca="false">H18*I18*(G18/365)</f>
-        <v>465873.259909019</v>
+        <v>444944.393970411</v>
       </c>
       <c r="K18" s="67" t="n">
         <f aca="false">H18+J18</f>
-        <v>7224287.89990902</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>7203359.03397041</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="68" t="n">
         <v>2008</v>
       </c>
@@ -39298,25 +39061,25 @@
       </c>
       <c r="G19" s="68" t="n">
         <f aca="false">IF(F19="",MAX(0,$B$7-E19),MAX(0,F19-E19))</f>
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H19" s="71" t="n">
         <v>444448.23</v>
       </c>
       <c r="I19" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J19" s="72" t="n">
         <f aca="false">H19*I19*(G19/365)</f>
-        <v>25129.1029242</v>
+        <v>24058.652406411</v>
       </c>
       <c r="K19" s="73" t="n">
         <f aca="false">H19+J19</f>
-        <v>469577.3329242</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>468506.882406411</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="60" t="n">
         <v>2010</v>
       </c>
@@ -39340,25 +39103,25 @@
       </c>
       <c r="G20" s="60" t="n">
         <f aca="false">IF(F20="",MAX(0,$B$7-E20),MAX(0,F20-E20))</f>
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H20" s="64" t="n">
         <v>12832109.38</v>
       </c>
       <c r="I20" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J20" s="66" t="n">
         <f aca="false">H20*I20*(G20/365)</f>
-        <v>725527.4643452</v>
+        <v>694621.41679463</v>
       </c>
       <c r="K20" s="67" t="n">
         <f aca="false">H20+J20</f>
-        <v>13557636.8443452</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>13526730.7967946</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="68" t="n">
         <v>2011</v>
       </c>
@@ -39382,25 +39145,25 @@
       </c>
       <c r="G21" s="68" t="n">
         <f aca="false">IF(F21="",MAX(0,$B$7-E21),MAX(0,F21-E21))</f>
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H21" s="71" t="n">
         <v>184056.25</v>
       </c>
       <c r="I21" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J21" s="72" t="n">
         <f aca="false">H21*I21*(G21/365)</f>
-        <v>9693.7636369863</v>
+        <v>9290.05011986301</v>
       </c>
       <c r="K21" s="73" t="n">
         <f aca="false">H21+J21</f>
-        <v>193750.013636986</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>193346.300119863</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="60" t="n">
         <v>2012</v>
       </c>
@@ -39424,25 +39187,25 @@
       </c>
       <c r="G22" s="60" t="n">
         <f aca="false">IF(F22="",MAX(0,$B$7-E22),MAX(0,F22-E22))</f>
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H22" s="64" t="n">
         <v>5425916.78</v>
       </c>
       <c r="I22" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J22" s="66" t="n">
         <f aca="false">H22*I22*(G22/365)</f>
-        <v>285768.914553447</v>
+        <v>273867.574898466</v>
       </c>
       <c r="K22" s="67" t="n">
         <f aca="false">H22+J22</f>
-        <v>5711685.69455345</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5699784.35489847</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="68" t="n">
         <v>2013</v>
       </c>
@@ -39466,14 +39229,14 @@
       </c>
       <c r="G23" s="68" t="n">
         <f aca="false">IF(F23="",MAX(0,$B$7-E23),MAX(0,F23-E23))</f>
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H23" s="71" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J23" s="72" t="n">
         <f aca="false">H23*I23*(G23/365)</f>
@@ -39484,7 +39247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="60" t="n">
         <v>2014</v>
       </c>
@@ -39508,14 +39271,14 @@
       </c>
       <c r="G24" s="60" t="n">
         <f aca="false">IF(F24="",MAX(0,$B$7-E24),MAX(0,F24-E24))</f>
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H24" s="64" t="n">
         <v>0</v>
       </c>
       <c r="I24" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J24" s="66" t="n">
         <f aca="false">H24*I24*(G24/365)</f>
@@ -39526,7 +39289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="68" t="n">
         <v>2015</v>
       </c>
@@ -39550,25 +39313,25 @@
       </c>
       <c r="G25" s="68" t="n">
         <f aca="false">IF(F25="",MAX(0,$B$7-E25),MAX(0,F25-E25))</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H25" s="71" t="n">
         <v>203181.59</v>
       </c>
       <c r="I25" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J25" s="72" t="n">
         <f aca="false">H25*I25*(G25/365)</f>
-        <v>4091.57622689863</v>
+        <v>4012.9755679726</v>
       </c>
       <c r="K25" s="73" t="n">
         <f aca="false">H25+J25</f>
-        <v>207273.166226899</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>207194.565567973</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="60" t="n">
         <v>2016</v>
       </c>
@@ -39592,14 +39355,14 @@
       </c>
       <c r="G26" s="60" t="n">
         <f aca="false">IF(F26="",MAX(0,$B$7-E26),MAX(0,F26-E26))</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H26" s="64" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J26" s="66" t="n">
         <f aca="false">H26*I26*(G26/365)</f>
@@ -39610,7 +39373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="68" t="n">
         <v>2017</v>
       </c>
@@ -39634,25 +39397,25 @@
       </c>
       <c r="G27" s="68" t="n">
         <f aca="false">IF(F27="",MAX(0,$B$7-E27),MAX(0,F27-E27))</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H27" s="71" t="n">
         <v>6266255.63</v>
       </c>
       <c r="I27" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J27" s="72" t="n">
         <f aca="false">H27*I27*(G27/365)</f>
-        <v>126186.937346921</v>
+        <v>123762.840648411</v>
       </c>
       <c r="K27" s="73" t="n">
         <f aca="false">H27+J27</f>
-        <v>6392442.56734692</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>6390018.47064841</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="60" t="n">
         <v>2018</v>
       </c>
@@ -39676,25 +39439,25 @@
       </c>
       <c r="G28" s="60" t="n">
         <f aca="false">IF(F28="",MAX(0,$B$7-E28),MAX(0,F28-E28))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H28" s="64" t="n">
         <v>633024.04</v>
       </c>
       <c r="I28" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J28" s="66" t="n">
         <f aca="false">H28*I28*(G28/365)</f>
-        <v>980.580252646575</v>
+        <v>1389.18426312329</v>
       </c>
       <c r="K28" s="67" t="n">
         <f aca="false">H28+J28</f>
-        <v>634004.620252647</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>634413.224263123</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="68" t="n">
         <v>2019</v>
       </c>
@@ -39718,25 +39481,25 @@
       </c>
       <c r="G29" s="68" t="n">
         <f aca="false">IF(F29="",MAX(0,$B$7-E29),MAX(0,F29-E29))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H29" s="71" t="n">
         <v>19702240.1</v>
       </c>
       <c r="I29" s="74" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J29" s="72" t="n">
         <f aca="false">H29*I29*(G29/365)</f>
-        <v>30519.579596</v>
+        <v>43236.97074</v>
       </c>
       <c r="K29" s="73" t="n">
         <f aca="false">H29+J29</f>
-        <v>19732759.679596</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19745477.07074</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="60" t="n">
         <v>2021</v>
       </c>
@@ -39760,25 +39523,25 @@
       </c>
       <c r="G30" s="60" t="n">
         <f aca="false">IF(F30="",MAX(0,$B$7-E30),MAX(0,F30-E30))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30" s="64" t="n">
         <v>95946.87</v>
       </c>
       <c r="I30" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J30" s="66" t="n">
         <f aca="false">H30*I30*(G30/365)</f>
-        <v>148.625644652055</v>
+        <v>210.557377726027</v>
       </c>
       <c r="K30" s="67" t="n">
         <f aca="false">H30+J30</f>
-        <v>96095.4956446521</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>96157.427377726</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="60" t="n">
         <v>2024</v>
       </c>
@@ -39809,7 +39572,7 @@
       </c>
       <c r="I31" s="65" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2827</v>
+        <v>0.267</v>
       </c>
       <c r="J31" s="66" t="n">
         <f aca="false">H31*I31*(G31/365)</f>
@@ -39820,7 +39583,7 @@
         <v>131593300.43</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="75" t="s">
         <v>354</v>
       </c>
@@ -39831,7 +39594,7 @@
       <c r="F32" s="75"/>
       <c r="G32" s="76" t="n">
         <f aca="false">IF(COUNTA(F10:F31)&gt;0,AVERAGE(G10:G31),AVERAGE(G10:G31))</f>
-        <v>59.0909090909091</v>
+        <v>60.0454545454546</v>
       </c>
       <c r="H32" s="77" t="n">
         <f aca="false">SUBTOTAL(109,H10:H31)</f>
@@ -39840,14 +39603,14 @@
       <c r="I32" s="75"/>
       <c r="J32" s="77" t="n">
         <f aca="false">SUBTOTAL(109,J10:J31)</f>
-        <v>10423598.2311423</v>
+        <v>9976002.94791797</v>
       </c>
       <c r="K32" s="77" t="n">
         <f aca="false">SUBTOTAL(109,K10:K31)</f>
-        <v>321493912.931142</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>321046317.647918</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="78" t="s">
         <v>355</v>
       </c>
@@ -39867,7 +39630,7 @@
       </c>
       <c r="B36" s="79" t="n">
         <f aca="false">J32</f>
-        <v>10423598.2311423</v>
+        <v>9976002.94791797</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -39876,10 +39639,10 @@
       </c>
       <c r="B37" s="81" t="n">
         <f aca="false">B35+B36</f>
-        <v>321493912.931142</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>321046317.647918</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="57" t="s">
         <v>359</v>
       </c>
@@ -39888,13 +39651,13 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="57" t="s">
         <v>360</v>
       </c>
       <c r="B39" s="83" t="n">
         <f aca="false">G32</f>
-        <v>59.0909090909091</v>
+        <v>60.0454545454546</v>
       </c>
     </row>
   </sheetData>
@@ -39920,19 +39683,19 @@
   <dimension ref="A1:K8"/>
   <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="48" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="48" width="50.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="48" width="32.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="48" width="16.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="48" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="48" width="21.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="48" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="48" width="23.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="48" width="25.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="84" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="85" t="s">
         <v>0</v>
       </c>
@@ -39967,7 +39730,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="88" t="s">
         <v>203</v>
       </c>
@@ -40003,7 +39766,7 @@
         <v>0.689429355685356</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="88" t="s">
         <v>203</v>
       </c>
@@ -40039,7 +39802,7 @@
         <v>0.856724348497189</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="88" t="s">
         <v>203</v>
       </c>
@@ -40075,7 +39838,7 @@
         <v>0.928022136016653</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="88" t="s">
         <v>203</v>
       </c>
@@ -40111,7 +39874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="88" t="s">
         <v>263</v>
       </c>
@@ -40147,7 +39910,7 @@
         <v>0.327006348146499</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="88" t="s">
         <v>186</v>
       </c>
@@ -40186,7 +39949,7 @@
         <v>1.0047634017279</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="88" t="s">
         <v>149</v>
       </c>
@@ -40244,12 +40007,12 @@
   <dimension ref="A2:D9"/>
   <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="48" width="22.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="48" width="19.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="48" width="11.45"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="96" t="s">
         <v>0</v>
       </c>
@@ -40263,11 +40026,11 @@
         <v>383</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
         <v>263</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="48" t="s">
         <v>384</v>
       </c>
       <c r="C3" s="97" t="n">
@@ -40277,11 +40040,11 @@
         <v>44256</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
         <v>263</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="48" t="s">
         <v>385</v>
       </c>
       <c r="C4" s="97" t="n">
@@ -40291,11 +40054,11 @@
         <v>46042</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="48" t="s">
         <v>386</v>
       </c>
       <c r="C5" s="97" t="n">
@@ -40305,11 +40068,11 @@
         <v>45870</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="48" t="s">
         <v>386</v>
       </c>
       <c r="C6" s="97" t="n">
@@ -40319,11 +40082,11 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="48" t="s">
         <v>387</v>
       </c>
       <c r="C7" s="97" t="n">
@@ -40333,11 +40096,11 @@
         <v>45870</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
         <v>186</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="48" t="s">
         <v>387</v>
       </c>
       <c r="C8" s="97" t="n">
@@ -40347,11 +40110,11 @@
         <v>45870</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
         <v>301</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="48" t="s">
         <v>386</v>
       </c>
       <c r="C9" s="97" t="n">

</xml_diff>

<commit_message>
Actualizacion automatica 18/06/2026 14:49 (Buenos Aires)
</commit_message>
<xml_diff>
--- a/Master UOPs.xlsx
+++ b/Master UOPs.xlsx
@@ -2074,16 +2074,16 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="102">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2091,7 +2091,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2119,7 +2119,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2167,7 +2167,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2195,7 +2195,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2275,11 +2275,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2291,27 +2299,27 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2335,7 +2343,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="26" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2343,11 +2351,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="28" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="28" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="29" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="29" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2363,15 +2371,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="26" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="28" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="28" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="29" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="29" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2379,7 +2387,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2387,35 +2395,35 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="32" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="31" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="31" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="175" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2463,15 +2471,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2828,9 +2836,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>209520</xdr:colOff>
+      <xdr:colOff>209160</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>37440</xdr:rowOff>
+      <xdr:rowOff>37080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2845,7 +2853,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10472040" y="10696680"/>
-          <a:ext cx="4844880" cy="2046960"/>
+          <a:ext cx="4844520" cy="2046600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2867,9 +2875,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1494360</xdr:colOff>
+      <xdr:colOff>1494000</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>24480</xdr:rowOff>
+      <xdr:rowOff>24120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2884,7 +2892,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4453560" y="6731280"/>
-          <a:ext cx="6010920" cy="5999400"/>
+          <a:ext cx="6010560" cy="5999040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -38795,13 +38803,13 @@
       <c r="D554" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="E554" s="13" t="n">
+      <c r="E554" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F554" s="13" t="s">
+      <c r="F554" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="G554" s="13" t="s">
+      <c r="G554" s="50" t="s">
         <v>79</v>
       </c>
       <c r="H554" s="30" t="n">
@@ -38881,10 +38889,10 @@
       <c r="D555" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="E555" s="13" t="n">
+      <c r="E555" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F555" s="13" t="s">
+      <c r="F555" s="50" t="s">
         <v>126</v>
       </c>
       <c r="G555" s="13" t="s">
@@ -38967,10 +38975,10 @@
       <c r="D556" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="E556" s="13" t="n">
+      <c r="E556" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F556" s="13" t="s">
+      <c r="F556" s="50" t="s">
         <v>126</v>
       </c>
       <c r="G556" s="13" t="s">
@@ -39723,1124 +39731,1124 @@
   <dimension ref="A1:K39"/>
   <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="18.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="22.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="51" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="51" width="18.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="51" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="51" width="18.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="51" width="12.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="51" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="51" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="51" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="51" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="51" width="22.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>338</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="53" t="s">
         <v>339</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="54" t="s">
         <v>340</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="B4" s="55" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="56" t="s">
         <v>342</v>
       </c>
-      <c r="B5" s="55" t="n">
-        <v>0.2557</v>
-      </c>
-      <c r="C5" s="56" t="s">
+      <c r="B5" s="57" t="n">
+        <v>0.2362</v>
+      </c>
+      <c r="C5" s="58" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="54" t="s">
+      <c r="A6" s="56" t="s">
         <v>344</v>
       </c>
-      <c r="B6" s="57" t="n">
+      <c r="B6" s="59" t="n">
         <v>60</v>
       </c>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="58" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="60" t="s">
         <v>346</v>
       </c>
-      <c r="B7" s="59" t="n">
+      <c r="B7" s="61" t="n">
         <f aca="true">TODAY()</f>
-        <v>46190</v>
+        <v>46191</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="60" t="s">
+      <c r="A9" s="62" t="s">
         <v>347</v>
       </c>
-      <c r="B9" s="60" t="s">
+      <c r="B9" s="62" t="s">
         <v>348</v>
       </c>
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="62" t="s">
         <v>349</v>
       </c>
-      <c r="D9" s="60" t="s">
+      <c r="D9" s="62" t="s">
         <v>350</v>
       </c>
-      <c r="E9" s="60" t="s">
+      <c r="E9" s="62" t="s">
         <v>351</v>
       </c>
-      <c r="F9" s="60" t="s">
+      <c r="F9" s="62" t="s">
         <v>352</v>
       </c>
-      <c r="G9" s="60" t="s">
+      <c r="G9" s="62" t="s">
         <v>353</v>
       </c>
-      <c r="H9" s="60" t="s">
+      <c r="H9" s="62" t="s">
         <v>354</v>
       </c>
-      <c r="I9" s="60" t="s">
+      <c r="I9" s="62" t="s">
         <v>355</v>
       </c>
-      <c r="J9" s="60" t="s">
+      <c r="J9" s="62" t="s">
         <v>356</v>
       </c>
-      <c r="K9" s="60" t="s">
+      <c r="K9" s="62" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="61" t="n">
+      <c r="A10" s="63" t="n">
         <v>1998</v>
       </c>
-      <c r="B10" s="62" t="n">
+      <c r="B10" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C10" s="63" t="n">
+      <c r="C10" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D10" s="61" t="n">
+      <c r="D10" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E10" s="62" t="n">
+      <c r="E10" s="64" t="n">
         <f aca="false">C10+D10</f>
         <v>46095</v>
       </c>
-      <c r="F10" s="64" t="str">
+      <c r="F10" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G10" s="61" t="n">
+      <c r="G10" s="63" t="n">
         <f aca="false">IF(F10="",MAX(0,$B$7-E10),MAX(0,F10-E10))</f>
-        <v>95</v>
-      </c>
-      <c r="H10" s="65" t="n">
+        <v>96</v>
+      </c>
+      <c r="H10" s="67" t="n">
         <v>50402510.51</v>
       </c>
-      <c r="I10" s="66" t="n">
+      <c r="I10" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J10" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J10" s="69" t="n">
         <f aca="false">H10*I10*(G10/365)</f>
-        <v>3747944.49043059</v>
-      </c>
-      <c r="K10" s="68" t="n">
+        <v>3528893.79886343</v>
+      </c>
+      <c r="K10" s="70" t="n">
         <f aca="false">H10+J10</f>
-        <v>54150455.0004306</v>
+        <v>53931404.3088634</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="69" t="n">
+      <c r="A11" s="71" t="n">
         <v>1999</v>
       </c>
-      <c r="B11" s="70" t="n">
+      <c r="B11" s="72" t="n">
         <v>46035</v>
       </c>
-      <c r="C11" s="71" t="n">
+      <c r="C11" s="73" t="n">
         <v>46035</v>
       </c>
-      <c r="D11" s="69" t="n">
+      <c r="D11" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E11" s="70" t="n">
+      <c r="E11" s="72" t="n">
         <f aca="false">C11+D11</f>
         <v>46095</v>
       </c>
-      <c r="F11" s="64" t="str">
+      <c r="F11" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G11" s="69" t="n">
+      <c r="G11" s="71" t="n">
         <f aca="false">IF(F11="",MAX(0,$B$7-E11),MAX(0,F11-E11))</f>
-        <v>95</v>
-      </c>
-      <c r="H11" s="72" t="n">
+        <v>96</v>
+      </c>
+      <c r="H11" s="74" t="n">
         <v>677271.96</v>
       </c>
-      <c r="I11" s="66" t="n">
+      <c r="I11" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J11" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J11" s="75" t="n">
         <f aca="false">H11*I11*(G11/365)</f>
-        <v>50362.1284995616</v>
-      </c>
-      <c r="K11" s="74" t="n">
+        <v>47418.6860060055</v>
+      </c>
+      <c r="K11" s="76" t="n">
         <f aca="false">H11+J11</f>
-        <v>727634.088499562</v>
+        <v>724690.646006006</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="61" t="n">
+      <c r="A12" s="63" t="n">
         <v>2000</v>
       </c>
-      <c r="B12" s="62" t="n">
+      <c r="B12" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C12" s="63" t="n">
+      <c r="C12" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D12" s="61" t="n">
+      <c r="D12" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E12" s="62" t="n">
+      <c r="E12" s="64" t="n">
         <f aca="false">C12+D12</f>
         <v>46095</v>
       </c>
-      <c r="F12" s="64" t="str">
+      <c r="F12" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G12" s="61" t="n">
+      <c r="G12" s="63" t="n">
         <f aca="false">IF(F12="",MAX(0,$B$7-E12),MAX(0,F12-E12))</f>
-        <v>95</v>
-      </c>
-      <c r="H12" s="65" t="n">
+        <v>96</v>
+      </c>
+      <c r="H12" s="67" t="n">
         <v>17699825.4</v>
       </c>
-      <c r="I12" s="66" t="n">
+      <c r="I12" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J12" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J12" s="69" t="n">
         <f aca="false">H12*I12*(G12/365)</f>
-        <v>1316163.86601123</v>
-      </c>
-      <c r="K12" s="68" t="n">
+        <v>1239239.93989611</v>
+      </c>
+      <c r="K12" s="70" t="n">
         <f aca="false">H12+J12</f>
-        <v>19015989.2660112</v>
+        <v>18939065.3398961</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="69" t="n">
+      <c r="A13" s="71" t="n">
         <v>2001</v>
       </c>
-      <c r="B13" s="70" t="n">
+      <c r="B13" s="72" t="n">
         <v>46035</v>
       </c>
-      <c r="C13" s="71" t="n">
+      <c r="C13" s="73" t="n">
         <v>46035</v>
       </c>
-      <c r="D13" s="69" t="n">
+      <c r="D13" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E13" s="70" t="n">
+      <c r="E13" s="72" t="n">
         <f aca="false">C13+D13</f>
         <v>46095</v>
       </c>
-      <c r="F13" s="64" t="str">
+      <c r="F13" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G13" s="69" t="n">
+      <c r="G13" s="71" t="n">
         <f aca="false">IF(F13="",MAX(0,$B$7-E13),MAX(0,F13-E13))</f>
-        <v>95</v>
-      </c>
-      <c r="H13" s="72" t="n">
+        <v>96</v>
+      </c>
+      <c r="H13" s="74" t="n">
         <v>1015907.94</v>
       </c>
-      <c r="I13" s="66" t="n">
+      <c r="I13" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J13" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J13" s="75" t="n">
         <f aca="false">H13*I13*(G13/365)</f>
-        <v>75543.1927493424</v>
-      </c>
-      <c r="K13" s="74" t="n">
+        <v>71128.0290090082</v>
+      </c>
+      <c r="K13" s="76" t="n">
         <f aca="false">H13+J13</f>
-        <v>1091451.13274934</v>
+        <v>1087035.96900901</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="61" t="n">
+      <c r="A14" s="63" t="n">
         <v>2002</v>
       </c>
-      <c r="B14" s="62" t="n">
+      <c r="B14" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C14" s="63" t="n">
+      <c r="C14" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D14" s="61" t="n">
+      <c r="D14" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E14" s="62" t="n">
+      <c r="E14" s="64" t="n">
         <f aca="false">C14+D14</f>
         <v>46095</v>
       </c>
-      <c r="F14" s="64" t="str">
+      <c r="F14" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G14" s="61" t="n">
+      <c r="G14" s="63" t="n">
         <f aca="false">IF(F14="",MAX(0,$B$7-E14),MAX(0,F14-E14))</f>
-        <v>95</v>
-      </c>
-      <c r="H14" s="65" t="n">
+        <v>96</v>
+      </c>
+      <c r="H14" s="67" t="n">
         <v>27253875.19</v>
       </c>
-      <c r="I14" s="66" t="n">
+      <c r="I14" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J14" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J14" s="69" t="n">
         <f aca="false">H14*I14*(G14/365)</f>
-        <v>2026605.62594352</v>
-      </c>
-      <c r="K14" s="68" t="n">
+        <v>1908159.53768627</v>
+      </c>
+      <c r="K14" s="70" t="n">
         <f aca="false">H14+J14</f>
-        <v>29280480.8159435</v>
+        <v>29162034.7276863</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="69" t="n">
+      <c r="A15" s="71" t="n">
         <v>2003</v>
       </c>
-      <c r="B15" s="70" t="n">
+      <c r="B15" s="72" t="n">
         <v>46035</v>
       </c>
-      <c r="C15" s="71" t="n">
+      <c r="C15" s="73" t="n">
         <v>46035</v>
       </c>
-      <c r="D15" s="69" t="n">
+      <c r="D15" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E15" s="70" t="n">
+      <c r="E15" s="72" t="n">
         <f aca="false">C15+D15</f>
         <v>46095</v>
       </c>
-      <c r="F15" s="64" t="str">
+      <c r="F15" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G15" s="69" t="n">
+      <c r="G15" s="71" t="n">
         <f aca="false">IF(F15="",MAX(0,$B$7-E15),MAX(0,F15-E15))</f>
-        <v>95</v>
-      </c>
-      <c r="H15" s="72" t="n">
+        <v>96</v>
+      </c>
+      <c r="H15" s="74" t="n">
         <v>1015907.94</v>
       </c>
-      <c r="I15" s="66" t="n">
+      <c r="I15" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J15" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J15" s="75" t="n">
         <f aca="false">H15*I15*(G15/365)</f>
-        <v>75543.1927493424</v>
-      </c>
-      <c r="K15" s="74" t="n">
+        <v>71128.0290090082</v>
+      </c>
+      <c r="K15" s="76" t="n">
         <f aca="false">H15+J15</f>
-        <v>1091451.13274934</v>
+        <v>1087035.96900901</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="61" t="n">
+      <c r="A16" s="63" t="n">
         <v>2004</v>
       </c>
-      <c r="B16" s="62" t="n">
+      <c r="B16" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C16" s="63" t="n">
+      <c r="C16" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D16" s="61" t="n">
+      <c r="D16" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E16" s="62" t="n">
+      <c r="E16" s="64" t="n">
         <f aca="false">C16+D16</f>
         <v>46095</v>
       </c>
-      <c r="F16" s="64" t="str">
+      <c r="F16" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G16" s="61" t="n">
+      <c r="G16" s="63" t="n">
         <f aca="false">IF(F16="",MAX(0,$B$7-E16),MAX(0,F16-E16))</f>
-        <v>95</v>
-      </c>
-      <c r="H16" s="65" t="n">
+        <v>96</v>
+      </c>
+      <c r="H16" s="67" t="n">
         <v>28627721.36</v>
       </c>
-      <c r="I16" s="66" t="n">
+      <c r="I16" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J16" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J16" s="69" t="n">
         <f aca="false">H16*I16*(G16/365)</f>
-        <v>2128765.20354093</v>
-      </c>
-      <c r="K16" s="68" t="n">
+        <v>2004348.34218924</v>
+      </c>
+      <c r="K16" s="70" t="n">
         <f aca="false">H16+J16</f>
-        <v>30756486.5635409</v>
+        <v>30632069.7021892</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="69" t="n">
+      <c r="A17" s="71" t="n">
         <v>2005</v>
       </c>
-      <c r="B17" s="70" t="n">
+      <c r="B17" s="72" t="n">
         <v>46035</v>
       </c>
-      <c r="C17" s="71" t="n">
+      <c r="C17" s="73" t="n">
         <v>46035</v>
       </c>
-      <c r="D17" s="69" t="n">
+      <c r="D17" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E17" s="70" t="n">
+      <c r="E17" s="72" t="n">
         <f aca="false">C17+D17</f>
         <v>46095</v>
       </c>
-      <c r="F17" s="64" t="str">
+      <c r="F17" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G17" s="69" t="n">
+      <c r="G17" s="71" t="n">
         <f aca="false">IF(F17="",MAX(0,$B$7-E17),MAX(0,F17-E17))</f>
-        <v>95</v>
-      </c>
-      <c r="H17" s="72" t="n">
+        <v>96</v>
+      </c>
+      <c r="H17" s="74" t="n">
         <v>238400.46</v>
       </c>
-      <c r="I17" s="66" t="n">
+      <c r="I17" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J17" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J17" s="75" t="n">
         <f aca="false">H17*I17*(G17/365)</f>
-        <v>17727.5235207945</v>
-      </c>
-      <c r="K17" s="74" t="n">
+        <v>16691.4285901151</v>
+      </c>
+      <c r="K17" s="76" t="n">
         <f aca="false">H17+J17</f>
-        <v>256127.983520795</v>
+        <v>255091.888590115</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="61" t="n">
+      <c r="A18" s="63" t="n">
         <v>2006</v>
       </c>
-      <c r="B18" s="62" t="n">
+      <c r="B18" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C18" s="63" t="n">
+      <c r="C18" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D18" s="61" t="n">
+      <c r="D18" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E18" s="62" t="n">
+      <c r="E18" s="64" t="n">
         <f aca="false">C18+D18</f>
         <v>46095</v>
       </c>
-      <c r="F18" s="64" t="str">
+      <c r="F18" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G18" s="61" t="n">
+      <c r="G18" s="63" t="n">
         <f aca="false">IF(F18="",MAX(0,$B$7-E18),MAX(0,F18-E18))</f>
-        <v>95</v>
-      </c>
-      <c r="H18" s="65" t="n">
+        <v>96</v>
+      </c>
+      <c r="H18" s="67" t="n">
         <v>6758414.64</v>
       </c>
-      <c r="I18" s="66" t="n">
+      <c r="I18" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J18" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J18" s="69" t="n">
         <f aca="false">H18*I18*(G18/365)</f>
-        <v>502557.564250849</v>
-      </c>
-      <c r="K18" s="68" t="n">
+        <v>473185.309063364</v>
+      </c>
+      <c r="K18" s="70" t="n">
         <f aca="false">H18+J18</f>
-        <v>7260972.20425085</v>
+        <v>7231599.94906336</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="69" t="n">
+      <c r="A19" s="71" t="n">
         <v>2008</v>
       </c>
-      <c r="B19" s="70" t="n">
+      <c r="B19" s="72" t="n">
         <v>46051</v>
       </c>
-      <c r="C19" s="71" t="n">
+      <c r="C19" s="73" t="n">
         <v>46051</v>
       </c>
-      <c r="D19" s="69" t="n">
+      <c r="D19" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E19" s="70" t="n">
+      <c r="E19" s="72" t="n">
         <f aca="false">C19+D19</f>
         <v>46111</v>
       </c>
-      <c r="F19" s="64" t="str">
+      <c r="F19" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G19" s="69" t="n">
+      <c r="G19" s="71" t="n">
         <f aca="false">IF(F19="",MAX(0,$B$7-E19),MAX(0,F19-E19))</f>
-        <v>79</v>
-      </c>
-      <c r="H19" s="72" t="n">
+        <v>80</v>
+      </c>
+      <c r="H19" s="74" t="n">
         <v>444448.23</v>
       </c>
-      <c r="I19" s="66" t="n">
+      <c r="I19" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J19" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J19" s="75" t="n">
         <f aca="false">H19*I19*(G19/365)</f>
-        <v>27483.0955769014</v>
-      </c>
-      <c r="K19" s="74" t="n">
+        <v>25931.4233043288</v>
+      </c>
+      <c r="K19" s="76" t="n">
         <f aca="false">H19+J19</f>
-        <v>471931.325576901</v>
+        <v>470379.653304329</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="61" t="n">
+      <c r="A20" s="63" t="n">
         <v>2010</v>
       </c>
-      <c r="B20" s="62" t="n">
+      <c r="B20" s="64" t="n">
         <v>46051</v>
       </c>
-      <c r="C20" s="63" t="n">
+      <c r="C20" s="65" t="n">
         <v>46051</v>
       </c>
-      <c r="D20" s="61" t="n">
+      <c r="D20" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E20" s="62" t="n">
+      <c r="E20" s="64" t="n">
         <f aca="false">C20+D20</f>
         <v>46111</v>
       </c>
-      <c r="F20" s="64" t="str">
+      <c r="F20" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G20" s="61" t="n">
+      <c r="G20" s="63" t="n">
         <f aca="false">IF(F20="",MAX(0,$B$7-E20),MAX(0,F20-E20))</f>
-        <v>79</v>
-      </c>
-      <c r="H20" s="65" t="n">
+        <v>80</v>
+      </c>
+      <c r="H20" s="67" t="n">
         <v>12832109.38</v>
       </c>
-      <c r="I20" s="66" t="n">
+      <c r="I20" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J20" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J20" s="69" t="n">
         <f aca="false">H20*I20*(G20/365)</f>
-        <v>793491.940655929</v>
-      </c>
-      <c r="K20" s="68" t="n">
+        <v>748692.058510904</v>
+      </c>
+      <c r="K20" s="70" t="n">
         <f aca="false">H20+J20</f>
-        <v>13625601.3206559</v>
+        <v>13580801.4385109</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="69" t="n">
+      <c r="A21" s="71" t="n">
         <v>2011</v>
       </c>
-      <c r="B21" s="70" t="n">
+      <c r="B21" s="72" t="n">
         <v>46056</v>
       </c>
-      <c r="C21" s="71" t="n">
+      <c r="C21" s="73" t="n">
         <v>46056</v>
       </c>
-      <c r="D21" s="69" t="n">
+      <c r="D21" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E21" s="70" t="n">
+      <c r="E21" s="72" t="n">
         <f aca="false">C21+D21</f>
         <v>46116</v>
       </c>
-      <c r="F21" s="64" t="str">
+      <c r="F21" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G21" s="69" t="n">
+      <c r="G21" s="71" t="n">
         <f aca="false">IF(F21="",MAX(0,$B$7-E21),MAX(0,F21-E21))</f>
-        <v>74</v>
-      </c>
-      <c r="H21" s="72" t="n">
+        <v>75</v>
+      </c>
+      <c r="H21" s="74" t="n">
         <v>184056.25</v>
       </c>
-      <c r="I21" s="66" t="n">
+      <c r="I21" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J21" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J21" s="75" t="n">
         <f aca="false">H21*I21*(G21/365)</f>
-        <v>10661.0422636986</v>
-      </c>
-      <c r="K21" s="74" t="n">
+        <v>10067.6247431507</v>
+      </c>
+      <c r="K21" s="76" t="n">
         <f aca="false">H21+J21</f>
-        <v>194717.292263699</v>
+        <v>194123.874743151</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="61" t="n">
+      <c r="A22" s="63" t="n">
         <v>2012</v>
       </c>
-      <c r="B22" s="62" t="n">
+      <c r="B22" s="64" t="n">
         <v>46056</v>
       </c>
-      <c r="C22" s="63" t="n">
+      <c r="C22" s="65" t="n">
         <v>46056</v>
       </c>
-      <c r="D22" s="61" t="n">
+      <c r="D22" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E22" s="62" t="n">
+      <c r="E22" s="64" t="n">
         <f aca="false">C22+D22</f>
         <v>46116</v>
       </c>
-      <c r="F22" s="64" t="str">
+      <c r="F22" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G22" s="61" t="n">
+      <c r="G22" s="63" t="n">
         <f aca="false">IF(F22="",MAX(0,$B$7-E22),MAX(0,F22-E22))</f>
-        <v>74</v>
-      </c>
-      <c r="H22" s="65" t="n">
+        <v>75</v>
+      </c>
+      <c r="H22" s="67" t="n">
         <v>5425916.78</v>
       </c>
-      <c r="I22" s="66" t="n">
+      <c r="I22" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J22" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J22" s="69" t="n">
         <f aca="false">H22*I22*(G22/365)</f>
-        <v>314283.965423025</v>
-      </c>
-      <c r="K22" s="68" t="n">
+        <v>296790.215103288</v>
+      </c>
+      <c r="K22" s="70" t="n">
         <f aca="false">H22+J22</f>
-        <v>5740200.74542302</v>
+        <v>5722706.99510329</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="69" t="n">
+      <c r="A23" s="71" t="n">
         <v>2013</v>
       </c>
-      <c r="B23" s="70" t="n">
+      <c r="B23" s="72" t="n">
         <v>46056</v>
       </c>
-      <c r="C23" s="71" t="n">
+      <c r="C23" s="73" t="n">
         <v>46056</v>
       </c>
-      <c r="D23" s="69" t="n">
+      <c r="D23" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E23" s="70" t="n">
+      <c r="E23" s="72" t="n">
         <f aca="false">C23+D23</f>
         <v>46116</v>
       </c>
-      <c r="F23" s="64" t="str">
+      <c r="F23" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G23" s="69" t="n">
+      <c r="G23" s="71" t="n">
         <f aca="false">IF(F23="",MAX(0,$B$7-E23),MAX(0,F23-E23))</f>
-        <v>74</v>
-      </c>
-      <c r="H23" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="66" t="n">
+        <v>75</v>
+      </c>
+      <c r="H23" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J23" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J23" s="75" t="n">
         <f aca="false">H23*I23*(G23/365)</f>
         <v>0</v>
       </c>
-      <c r="K23" s="74" t="n">
+      <c r="K23" s="76" t="n">
         <f aca="false">H23+J23</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="61" t="n">
+      <c r="A24" s="63" t="n">
         <v>2014</v>
       </c>
-      <c r="B24" s="62" t="n">
+      <c r="B24" s="64" t="n">
         <v>46059</v>
       </c>
-      <c r="C24" s="63" t="n">
+      <c r="C24" s="65" t="n">
         <v>46059</v>
       </c>
-      <c r="D24" s="61" t="n">
+      <c r="D24" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E24" s="62" t="n">
+      <c r="E24" s="64" t="n">
         <f aca="false">C24+D24</f>
         <v>46119</v>
       </c>
-      <c r="F24" s="64" t="str">
+      <c r="F24" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G24" s="61" t="n">
+      <c r="G24" s="63" t="n">
         <f aca="false">IF(F24="",MAX(0,$B$7-E24),MAX(0,F24-E24))</f>
-        <v>71</v>
-      </c>
-      <c r="H24" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="66" t="n">
+        <v>72</v>
+      </c>
+      <c r="H24" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J24" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J24" s="69" t="n">
         <f aca="false">H24*I24*(G24/365)</f>
         <v>0</v>
       </c>
-      <c r="K24" s="68" t="n">
+      <c r="K24" s="70" t="n">
         <f aca="false">H24+J24</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="69" t="n">
+      <c r="A25" s="71" t="n">
         <v>2015</v>
       </c>
-      <c r="B25" s="70" t="n">
+      <c r="B25" s="72" t="n">
         <v>46098</v>
       </c>
-      <c r="C25" s="71" t="n">
+      <c r="C25" s="73" t="n">
         <v>46098</v>
       </c>
-      <c r="D25" s="69" t="n">
+      <c r="D25" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E25" s="70" t="n">
+      <c r="E25" s="72" t="n">
         <f aca="false">C25+D25</f>
         <v>46158</v>
       </c>
-      <c r="F25" s="64" t="str">
+      <c r="F25" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G25" s="69" t="n">
+      <c r="G25" s="71" t="n">
         <f aca="false">IF(F25="",MAX(0,$B$7-E25),MAX(0,F25-E25))</f>
-        <v>32</v>
-      </c>
-      <c r="H25" s="72" t="n">
+        <v>33</v>
+      </c>
+      <c r="H25" s="74" t="n">
         <v>203181.59</v>
       </c>
-      <c r="I25" s="66" t="n">
+      <c r="I25" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J25" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J25" s="75" t="n">
         <f aca="false">H25*I25*(G25/365)</f>
-        <v>5089.22566689315</v>
-      </c>
-      <c r="K25" s="74" t="n">
+        <v>4890.05204250411</v>
+      </c>
+      <c r="K25" s="76" t="n">
         <f aca="false">H25+J25</f>
-        <v>208270.815666893</v>
+        <v>208071.642042504</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="61" t="n">
+      <c r="A26" s="63" t="n">
         <v>2016</v>
       </c>
-      <c r="B26" s="62" t="n">
+      <c r="B26" s="64" t="n">
         <v>46098</v>
       </c>
-      <c r="C26" s="63" t="n">
+      <c r="C26" s="65" t="n">
         <v>46098</v>
       </c>
-      <c r="D26" s="61" t="n">
+      <c r="D26" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E26" s="62" t="n">
+      <c r="E26" s="64" t="n">
         <f aca="false">C26+D26</f>
         <v>46158</v>
       </c>
-      <c r="F26" s="64" t="str">
+      <c r="F26" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G26" s="61" t="n">
+      <c r="G26" s="63" t="n">
         <f aca="false">IF(F26="",MAX(0,$B$7-E26),MAX(0,F26-E26))</f>
-        <v>32</v>
-      </c>
-      <c r="H26" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="66" t="n">
+        <v>33</v>
+      </c>
+      <c r="H26" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J26" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J26" s="69" t="n">
         <f aca="false">H26*I26*(G26/365)</f>
         <v>0</v>
       </c>
-      <c r="K26" s="68" t="n">
+      <c r="K26" s="70" t="n">
         <f aca="false">H26+J26</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="69" t="n">
+      <c r="A27" s="71" t="n">
         <v>2017</v>
       </c>
-      <c r="B27" s="70" t="n">
+      <c r="B27" s="72" t="n">
         <v>46098</v>
       </c>
-      <c r="C27" s="71" t="n">
+      <c r="C27" s="73" t="n">
         <v>46098</v>
       </c>
-      <c r="D27" s="69" t="n">
+      <c r="D27" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E27" s="70" t="n">
+      <c r="E27" s="72" t="n">
         <f aca="false">C27+D27</f>
         <v>46158</v>
       </c>
-      <c r="F27" s="64" t="str">
+      <c r="F27" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G27" s="69" t="n">
+      <c r="G27" s="71" t="n">
         <f aca="false">IF(F27="",MAX(0,$B$7-E27),MAX(0,F27-E27))</f>
-        <v>32</v>
-      </c>
-      <c r="H27" s="72" t="n">
+        <v>33</v>
+      </c>
+      <c r="H27" s="74" t="n">
         <v>6266255.63</v>
       </c>
-      <c r="I27" s="66" t="n">
+      <c r="I27" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J27" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J27" s="75" t="n">
         <f aca="false">H27*I27*(G27/365)</f>
-        <v>156955.110881403</v>
-      </c>
-      <c r="K27" s="74" t="n">
+        <v>150812.463581638</v>
+      </c>
+      <c r="K27" s="76" t="n">
         <f aca="false">H27+J27</f>
-        <v>6423210.7408814</v>
+        <v>6417068.09358164</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="61" t="n">
+      <c r="A28" s="63" t="n">
         <v>2018</v>
       </c>
-      <c r="B28" s="62" t="n">
+      <c r="B28" s="64" t="n">
         <v>46122</v>
       </c>
-      <c r="C28" s="63" t="n">
+      <c r="C28" s="65" t="n">
         <v>46122</v>
       </c>
-      <c r="D28" s="61" t="n">
+      <c r="D28" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E28" s="62" t="n">
+      <c r="E28" s="64" t="n">
         <f aca="false">C28+D28</f>
         <v>46182</v>
       </c>
-      <c r="F28" s="64" t="str">
+      <c r="F28" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G28" s="61" t="n">
+      <c r="G28" s="63" t="n">
         <f aca="false">IF(F28="",MAX(0,$B$7-E28),MAX(0,F28-E28))</f>
-        <v>8</v>
-      </c>
-      <c r="H28" s="65" t="n">
+        <v>9</v>
+      </c>
+      <c r="H28" s="67" t="n">
         <v>633024.04</v>
       </c>
-      <c r="I28" s="66" t="n">
+      <c r="I28" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J28" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J28" s="69" t="n">
         <f aca="false">H28*I28*(G28/365)</f>
-        <v>3963.94450910685</v>
-      </c>
-      <c r="K28" s="68" t="n">
+        <v>4155.0657398137</v>
+      </c>
+      <c r="K28" s="70" t="n">
         <f aca="false">H28+J28</f>
-        <v>636987.984509107</v>
+        <v>637179.105739814</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="69" t="n">
+      <c r="A29" s="71" t="n">
         <v>2019</v>
       </c>
-      <c r="B29" s="70" t="n">
+      <c r="B29" s="72" t="n">
         <v>46122</v>
       </c>
-      <c r="C29" s="71" t="n">
+      <c r="C29" s="73" t="n">
         <v>46122</v>
       </c>
-      <c r="D29" s="69" t="n">
+      <c r="D29" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E29" s="70" t="n">
+      <c r="E29" s="72" t="n">
         <f aca="false">C29+D29</f>
         <v>46182</v>
       </c>
-      <c r="F29" s="64" t="str">
+      <c r="F29" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G29" s="69" t="n">
+      <c r="G29" s="71" t="n">
         <f aca="false">IF(F29="",MAX(0,$B$7-E29),MAX(0,F29-E29))</f>
-        <v>8</v>
-      </c>
-      <c r="H29" s="72" t="n">
+        <v>9</v>
+      </c>
+      <c r="H29" s="74" t="n">
         <v>19702240.1</v>
       </c>
-      <c r="I29" s="75" t="n">
+      <c r="I29" s="77" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J29" s="73" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J29" s="75" t="n">
         <f aca="false">H29*I29*(G29/365)</f>
-        <v>123373.808144</v>
-      </c>
-      <c r="K29" s="74" t="n">
+        <v>129322.265292</v>
+      </c>
+      <c r="K29" s="76" t="n">
         <f aca="false">H29+J29</f>
-        <v>19825613.908144</v>
+        <v>19831562.365292</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="61" t="n">
+      <c r="A30" s="63" t="n">
         <v>2021</v>
       </c>
-      <c r="B30" s="62" t="n">
+      <c r="B30" s="64" t="n">
         <v>46122</v>
       </c>
-      <c r="C30" s="63" t="n">
+      <c r="C30" s="65" t="n">
         <v>46122</v>
       </c>
-      <c r="D30" s="61" t="n">
+      <c r="D30" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E30" s="62" t="n">
+      <c r="E30" s="64" t="n">
         <f aca="false">C30+D30</f>
         <v>46182</v>
       </c>
-      <c r="F30" s="64" t="str">
+      <c r="F30" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G30" s="61" t="n">
+      <c r="G30" s="63" t="n">
         <f aca="false">IF(F30="",MAX(0,$B$7-E30),MAX(0,F30-E30))</f>
-        <v>8</v>
-      </c>
-      <c r="H30" s="65" t="n">
+        <v>9</v>
+      </c>
+      <c r="H30" s="67" t="n">
         <v>95946.87</v>
       </c>
-      <c r="I30" s="66" t="n">
+      <c r="I30" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J30" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J30" s="69" t="n">
         <f aca="false">H30*I30*(G30/365)</f>
-        <v>600.81141389589</v>
-      </c>
-      <c r="K30" s="68" t="n">
+        <v>629.779482591781</v>
+      </c>
+      <c r="K30" s="70" t="n">
         <f aca="false">H30+J30</f>
-        <v>96547.6814138959</v>
+        <v>96576.6494825918</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="61" t="n">
+      <c r="A31" s="63" t="n">
         <v>2024</v>
       </c>
-      <c r="B31" s="62" t="n">
+      <c r="B31" s="64" t="n">
         <v>46142</v>
       </c>
-      <c r="C31" s="63" t="n">
+      <c r="C31" s="65" t="n">
         <v>46142</v>
       </c>
-      <c r="D31" s="61" t="n">
+      <c r="D31" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E31" s="62" t="n">
+      <c r="E31" s="64" t="n">
         <f aca="false">C31+D31</f>
         <v>46202</v>
       </c>
-      <c r="F31" s="64" t="str">
+      <c r="F31" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G31" s="61" t="n">
+      <c r="G31" s="63" t="n">
         <f aca="false">IF(F31="",MAX(0,$B$7-E31),MAX(0,F31-E31))</f>
         <v>0</v>
       </c>
-      <c r="H31" s="65" t="n">
+      <c r="H31" s="67" t="n">
         <v>131593300.43</v>
       </c>
-      <c r="I31" s="66" t="n">
+      <c r="I31" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.2857</v>
-      </c>
-      <c r="J31" s="67" t="n">
+        <v>0.2662</v>
+      </c>
+      <c r="J31" s="69" t="n">
         <f aca="false">H31*I31*(G31/365)</f>
         <v>0</v>
       </c>
-      <c r="K31" s="68" t="n">
+      <c r="K31" s="70" t="n">
         <f aca="false">H31+J31</f>
         <v>131593300.43</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="76" t="s">
+      <c r="A32" s="78" t="s">
         <v>358</v>
       </c>
-      <c r="B32" s="76"/>
-      <c r="C32" s="76"/>
-      <c r="D32" s="76"/>
-      <c r="E32" s="76"/>
-      <c r="F32" s="76"/>
-      <c r="G32" s="77" t="n">
+      <c r="B32" s="78"/>
+      <c r="C32" s="78"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="79" t="n">
         <f aca="false">IF(COUNTA(F10:F31)&gt;0,AVERAGE(G10:G31),AVERAGE(G10:G31))</f>
-        <v>64.8181818181818</v>
-      </c>
-      <c r="H32" s="78" t="n">
+        <v>65.7727272727273</v>
+      </c>
+      <c r="H32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,H10:H31)</f>
         <v>311070314.7</v>
       </c>
-      <c r="I32" s="76"/>
-      <c r="J32" s="78" t="n">
+      <c r="I32" s="78"/>
+      <c r="J32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,J10:J31)</f>
-        <v>11377115.732231</v>
-      </c>
-      <c r="K32" s="78" t="n">
+        <v>10731484.0481128</v>
+      </c>
+      <c r="K32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,K10:K31)</f>
-        <v>322447430.432231</v>
+        <v>321801798.748113</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="79" t="s">
+      <c r="A34" s="81" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="54" t="s">
+      <c r="A35" s="56" t="s">
         <v>360</v>
       </c>
-      <c r="B35" s="80" t="n">
+      <c r="B35" s="82" t="n">
         <f aca="false">H32</f>
         <v>311070314.7</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="54" t="s">
+      <c r="A36" s="56" t="s">
         <v>361</v>
       </c>
-      <c r="B36" s="80" t="n">
+      <c r="B36" s="82" t="n">
         <f aca="false">J32</f>
-        <v>11377115.732231</v>
+        <v>10731484.0481128</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="81" t="s">
+      <c r="A37" s="83" t="s">
         <v>362</v>
       </c>
-      <c r="B37" s="82" t="n">
+      <c r="B37" s="84" t="n">
         <f aca="false">B35+B36</f>
-        <v>322447430.432231</v>
+        <v>321801798.748113</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="58" t="s">
+      <c r="A38" s="60" t="s">
         <v>363</v>
       </c>
-      <c r="B38" s="83" t="n">
+      <c r="B38" s="85" t="n">
         <f aca="false">COUNTIF(G10:G31,"&gt;"&amp;0)</f>
         <v>21</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="58" t="s">
+      <c r="A39" s="60" t="s">
         <v>364</v>
       </c>
-      <c r="B39" s="84" t="n">
+      <c r="B39" s="86" t="n">
         <f aca="false">G32</f>
-        <v>64.8181818181818</v>
+        <v>65.7727272727273</v>
       </c>
     </row>
   </sheetData>
@@ -40866,307 +40874,307 @@
   <dimension ref="A1:K8"/>
   <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="85" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="51" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="51" width="50.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="51" width="32.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="16.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="51" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="51" width="21.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="51" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="51" width="23.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="51" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="87" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="86" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="86" t="s">
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="86" t="s">
+      <c r="C1" s="88" t="s">
         <v>365</v>
       </c>
-      <c r="D1" s="86" t="s">
+      <c r="D1" s="88" t="s">
         <v>366</v>
       </c>
-      <c r="E1" s="86" t="s">
+      <c r="E1" s="88" t="s">
         <v>367</v>
       </c>
-      <c r="F1" s="86" t="s">
+      <c r="F1" s="88" t="s">
         <v>368</v>
       </c>
-      <c r="G1" s="87" t="s">
+      <c r="G1" s="89" t="s">
         <v>369</v>
       </c>
-      <c r="H1" s="87" t="s">
+      <c r="H1" s="89" t="s">
         <v>370</v>
       </c>
-      <c r="I1" s="87" t="s">
+      <c r="I1" s="89" t="s">
         <v>371</v>
       </c>
-      <c r="J1" s="87" t="s">
+      <c r="J1" s="89" t="s">
         <v>372</v>
       </c>
-      <c r="K1" s="88" t="s">
+      <c r="K1" s="90" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="89" t="s">
+      <c r="A2" s="91" t="s">
         <v>207</v>
       </c>
-      <c r="B2" s="90" t="s">
+      <c r="B2" s="92" t="s">
         <v>208</v>
       </c>
-      <c r="C2" s="91" t="s">
+      <c r="C2" s="93" t="s">
         <v>374</v>
       </c>
-      <c r="D2" s="89" t="n">
+      <c r="D2" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="89" t="s">
+      <c r="E2" s="91" t="s">
         <v>375</v>
       </c>
-      <c r="F2" s="92" t="n">
+      <c r="F2" s="94" t="n">
         <v>45938</v>
       </c>
-      <c r="G2" s="93" t="n">
+      <c r="G2" s="95" t="n">
         <v>21615296.4</v>
       </c>
-      <c r="H2" s="93"/>
-      <c r="I2" s="94" t="n">
+      <c r="H2" s="95"/>
+      <c r="I2" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!D:D,"Provision Tableros electricos")</f>
         <v>14902219.87</v>
       </c>
-      <c r="J2" s="94" t="n">
+      <c r="J2" s="96" t="n">
         <f aca="false">G2-I2</f>
         <v>6713076.53</v>
       </c>
-      <c r="K2" s="95" t="n">
+      <c r="K2" s="97" t="n">
         <f aca="false">IFERROR(I2/G2,0)</f>
         <v>0.689429355685356</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>207</v>
       </c>
-      <c r="B3" s="90" t="s">
+      <c r="B3" s="92" t="s">
         <v>208</v>
       </c>
-      <c r="C3" s="91" t="s">
+      <c r="C3" s="93" t="s">
         <v>376</v>
       </c>
-      <c r="D3" s="89" t="n">
+      <c r="D3" s="91" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="89" t="s">
+      <c r="E3" s="91" t="s">
         <v>377</v>
       </c>
-      <c r="F3" s="92" t="n">
+      <c r="F3" s="94" t="n">
         <v>46078</v>
       </c>
-      <c r="G3" s="93" t="n">
+      <c r="G3" s="95" t="n">
         <v>48893832.04</v>
       </c>
-      <c r="H3" s="93"/>
-      <c r="I3" s="94" t="n">
+      <c r="H3" s="95"/>
+      <c r="I3" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!D:D,"Conexión y Cableado")</f>
         <v>41888536.4</v>
       </c>
-      <c r="J3" s="94" t="n">
+      <c r="J3" s="96" t="n">
         <f aca="false">G3-I3</f>
         <v>7005295.64</v>
       </c>
-      <c r="K3" s="95" t="n">
+      <c r="K3" s="97" t="n">
         <f aca="false">IFERROR(I3/G3,0)</f>
         <v>0.856724348497189</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="91" t="s">
         <v>207</v>
       </c>
-      <c r="B4" s="90" t="s">
+      <c r="B4" s="92" t="s">
         <v>208</v>
       </c>
-      <c r="C4" s="91" t="s">
+      <c r="C4" s="93" t="s">
         <v>378</v>
       </c>
-      <c r="D4" s="89" t="n">
+      <c r="D4" s="91" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="89" t="s">
+      <c r="E4" s="91" t="s">
         <v>379</v>
       </c>
-      <c r="F4" s="92" t="n">
+      <c r="F4" s="94" t="n">
         <v>45904</v>
       </c>
-      <c r="G4" s="93" t="n">
+      <c r="G4" s="95" t="n">
         <v>81685880</v>
       </c>
-      <c r="H4" s="93"/>
-      <c r="I4" s="94" t="n">
+      <c r="H4" s="95"/>
+      <c r="I4" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!D:D,"Manifold y Tableros")</f>
         <v>75806304.84</v>
       </c>
-      <c r="J4" s="94" t="n">
+      <c r="J4" s="96" t="n">
         <f aca="false">G4-I4</f>
         <v>5879575.16</v>
       </c>
-      <c r="K4" s="95" t="n">
+      <c r="K4" s="97" t="n">
         <f aca="false">IFERROR(I4/G4,0)</f>
         <v>0.928022136016653</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="89" t="s">
+      <c r="A5" s="91" t="s">
         <v>207</v>
       </c>
-      <c r="B5" s="90" t="s">
+      <c r="B5" s="92" t="s">
         <v>208</v>
       </c>
-      <c r="C5" s="91" t="s">
+      <c r="C5" s="93" t="s">
         <v>380</v>
       </c>
-      <c r="D5" s="89" t="n">
+      <c r="D5" s="91" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="89" t="s">
+      <c r="E5" s="91" t="s">
         <v>381</v>
       </c>
-      <c r="F5" s="92" t="n">
+      <c r="F5" s="94" t="n">
         <v>45916</v>
       </c>
-      <c r="G5" s="93" t="n">
+      <c r="G5" s="95" t="n">
         <v>12601653.25</v>
       </c>
-      <c r="H5" s="93"/>
-      <c r="I5" s="94" t="n">
+      <c r="H5" s="95"/>
+      <c r="I5" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!D:D,"Oficina Tecnica")</f>
         <v>0</v>
       </c>
-      <c r="J5" s="94" t="n">
+      <c r="J5" s="96" t="n">
         <f aca="false">G5-I5</f>
         <v>12601653.25</v>
       </c>
-      <c r="K5" s="95" t="n">
+      <c r="K5" s="97" t="n">
         <f aca="false">IFERROR(I5/G5,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="89" t="s">
+      <c r="A6" s="91" t="s">
         <v>267</v>
       </c>
-      <c r="B6" s="90" t="s">
+      <c r="B6" s="92" t="s">
         <v>269</v>
       </c>
-      <c r="C6" s="91" t="s">
+      <c r="C6" s="93" t="s">
         <v>382</v>
       </c>
-      <c r="D6" s="89" t="n">
+      <c r="D6" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="89" t="s">
+      <c r="E6" s="91" t="s">
         <v>383</v>
       </c>
-      <c r="F6" s="92" t="n">
+      <c r="F6" s="94" t="n">
         <v>44308</v>
       </c>
-      <c r="G6" s="93" t="n">
+      <c r="G6" s="95" t="n">
         <v>175969573.995</v>
       </c>
-      <c r="H6" s="93"/>
-      <c r="I6" s="94" t="n">
+      <c r="H6" s="95"/>
+      <c r="I6" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!A:A,A6)</f>
         <v>57543167.777</v>
       </c>
-      <c r="J6" s="94" t="n">
+      <c r="J6" s="96" t="n">
         <f aca="false">G6-I6</f>
         <v>118426406.218</v>
       </c>
-      <c r="K6" s="95" t="n">
+      <c r="K6" s="97" t="n">
         <f aca="false">IFERROR(I6/G6,0)</f>
         <v>0.327006348146499</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="89" t="s">
+      <c r="A7" s="91" t="s">
         <v>190</v>
       </c>
-      <c r="B7" s="90" t="s">
+      <c r="B7" s="92" t="s">
         <v>191</v>
       </c>
-      <c r="C7" s="91" t="s">
+      <c r="C7" s="93" t="s">
         <v>382</v>
       </c>
-      <c r="D7" s="89" t="n">
+      <c r="D7" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="89" t="s">
+      <c r="E7" s="91" t="s">
         <v>384</v>
       </c>
-      <c r="F7" s="92" t="n">
+      <c r="F7" s="94" t="n">
         <v>46007</v>
       </c>
-      <c r="G7" s="93" t="n">
+      <c r="G7" s="95" t="n">
         <v>3390677291.57</v>
       </c>
-      <c r="H7" s="93" t="n">
+      <c r="H7" s="95" t="n">
         <f aca="false">+G7*1.044428</f>
         <v>3541318302.27987</v>
       </c>
-      <c r="I7" s="94" t="n">
+      <c r="I7" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!A:A,A7)</f>
         <v>3558187024</v>
       </c>
-      <c r="J7" s="94" t="n">
+      <c r="J7" s="96" t="n">
         <f aca="false">H7-I7</f>
         <v>-16868721.7201281</v>
       </c>
-      <c r="K7" s="95" t="n">
+      <c r="K7" s="97" t="n">
         <f aca="false">IFERROR(I7/H7,0)</f>
         <v>1.0047634017279</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="89" t="s">
+      <c r="A8" s="91" t="s">
         <v>153</v>
       </c>
-      <c r="B8" s="90" t="s">
+      <c r="B8" s="92" t="s">
         <v>155</v>
       </c>
-      <c r="C8" s="91" t="s">
+      <c r="C8" s="93" t="s">
         <v>382</v>
       </c>
-      <c r="D8" s="89" t="n">
+      <c r="D8" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="96" t="s">
+      <c r="E8" s="98" t="s">
         <v>385</v>
       </c>
-      <c r="F8" s="92" t="n">
+      <c r="F8" s="94" t="n">
         <v>46007</v>
       </c>
-      <c r="G8" s="93" t="n">
+      <c r="G8" s="95" t="n">
         <v>4837006176.45</v>
       </c>
-      <c r="H8" s="93" t="n">
+      <c r="H8" s="95" t="n">
         <f aca="false">+I8</f>
         <v>5105960136.19</v>
       </c>
-      <c r="I8" s="94" t="n">
+      <c r="I8" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!A:A,A8)</f>
         <v>5105960136.19</v>
       </c>
-      <c r="J8" s="94" t="n">
+      <c r="J8" s="96" t="n">
         <f aca="false">H8-I8</f>
         <v>0</v>
       </c>
-      <c r="K8" s="95" t="n">
+      <c r="K8" s="97" t="n">
         <f aca="false">IFERROR(I8/H8,0)</f>
         <v>1</v>
       </c>
@@ -41190,22 +41198,22 @@
   <dimension ref="A2:D9"/>
   <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="51" width="22.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="51" width="19.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="11.45"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="97" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="97" t="s">
+      <c r="A2" s="99" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="97" t="s">
+      <c r="C2" s="99" t="s">
         <v>386</v>
       </c>
-      <c r="D2" s="97" t="s">
+      <c r="D2" s="99" t="s">
         <v>387</v>
       </c>
     </row>
@@ -41213,13 +41221,13 @@
       <c r="A3" s="22" t="s">
         <v>267</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="51" t="s">
         <v>388</v>
       </c>
-      <c r="C3" s="98" t="n">
+      <c r="C3" s="100" t="n">
         <v>1759695739.95</v>
       </c>
-      <c r="D3" s="99" t="n">
+      <c r="D3" s="101" t="n">
         <v>44256</v>
       </c>
     </row>
@@ -41227,13 +41235,13 @@
       <c r="A4" s="22" t="s">
         <v>267</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="51" t="s">
         <v>389</v>
       </c>
-      <c r="C4" s="98" t="n">
+      <c r="C4" s="100" t="n">
         <v>351934615.48</v>
       </c>
-      <c r="D4" s="99" t="n">
+      <c r="D4" s="101" t="n">
         <v>46042</v>
       </c>
     </row>
@@ -41241,13 +41249,13 @@
       <c r="A5" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="51" t="s">
         <v>390</v>
       </c>
-      <c r="C5" s="98" t="n">
+      <c r="C5" s="100" t="n">
         <v>2337056186.58</v>
       </c>
-      <c r="D5" s="99" t="n">
+      <c r="D5" s="101" t="n">
         <v>45870</v>
       </c>
     </row>
@@ -41255,13 +41263,13 @@
       <c r="A6" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="51" t="s">
         <v>390</v>
       </c>
-      <c r="C6" s="98" t="n">
+      <c r="C6" s="100" t="n">
         <v>5000000000</v>
       </c>
-      <c r="D6" s="99" t="n">
+      <c r="D6" s="101" t="n">
         <v>46113</v>
       </c>
     </row>
@@ -41269,13 +41277,13 @@
       <c r="A7" s="22" t="s">
         <v>153</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="51" t="s">
         <v>391</v>
       </c>
-      <c r="C7" s="98" t="n">
+      <c r="C7" s="100" t="n">
         <v>30896493733.39</v>
       </c>
-      <c r="D7" s="99" t="n">
+      <c r="D7" s="101" t="n">
         <v>45870</v>
       </c>
     </row>
@@ -41283,13 +41291,13 @@
       <c r="A8" s="22" t="s">
         <v>190</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="51" t="s">
         <v>391</v>
       </c>
-      <c r="C8" s="98" t="n">
+      <c r="C8" s="100" t="n">
         <v>33906772915.32</v>
       </c>
-      <c r="D8" s="99" t="n">
+      <c r="D8" s="101" t="n">
         <v>45870</v>
       </c>
     </row>
@@ -41297,13 +41305,13 @@
       <c r="A9" s="22" t="s">
         <v>305</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="51" t="s">
         <v>390</v>
       </c>
-      <c r="C9" s="98" t="n">
+      <c r="C9" s="100" t="n">
         <v>1500000000</v>
       </c>
-      <c r="D9" s="99" t="n">
+      <c r="D9" s="101" t="n">
         <v>45839</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica 05/07/2026 05:56 (Buenos Aires)
</commit_message>
<xml_diff>
--- a/Master UOPs.xlsx
+++ b/Master UOPs.xlsx
@@ -2260,16 +2260,16 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="102">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2277,7 +2277,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2305,7 +2305,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2321,7 +2321,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2401,7 +2401,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2461,11 +2461,19 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2477,27 +2485,27 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="22" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2521,7 +2529,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="26" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2529,11 +2537,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="28" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="28" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="29" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="29" fillId="22" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2549,15 +2557,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="26" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="26" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="28" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="28" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="29" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="29" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2565,7 +2573,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2573,35 +2581,35 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="30" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="32" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="31" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="31" fillId="24" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="175" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2649,15 +2657,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3022,9 +3030,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>208440</xdr:colOff>
+      <xdr:colOff>208080</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>36360</xdr:rowOff>
+      <xdr:rowOff>36000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3039,7 +3047,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10472040" y="10696680"/>
-          <a:ext cx="4843800" cy="2045880"/>
+          <a:ext cx="4843440" cy="2045520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3061,9 +3069,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1493280</xdr:colOff>
+      <xdr:colOff>1492920</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>23400</xdr:rowOff>
+      <xdr:rowOff>23040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3078,7 +3086,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4453560" y="6731280"/>
-          <a:ext cx="6009840" cy="5998320"/>
+          <a:ext cx="6009480" cy="5997960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -39975,13 +39983,13 @@
       <c r="D562" s="14" t="s">
         <v>274</v>
       </c>
-      <c r="E562" s="14" t="n">
+      <c r="E562" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F562" s="14" t="s">
+      <c r="F562" s="50" t="s">
         <v>179</v>
       </c>
-      <c r="G562" s="14" t="s">
+      <c r="G562" s="50" t="s">
         <v>55</v>
       </c>
       <c r="H562" s="35" t="n">
@@ -40061,10 +40069,10 @@
       <c r="D563" s="14" t="s">
         <v>274</v>
       </c>
-      <c r="E563" s="14" t="n">
+      <c r="E563" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F563" s="14" t="s">
+      <c r="F563" s="50" t="s">
         <v>179</v>
       </c>
       <c r="G563" s="14" t="s">
@@ -40147,10 +40155,10 @@
       <c r="D564" s="14" t="s">
         <v>274</v>
       </c>
-      <c r="E564" s="14" t="n">
+      <c r="E564" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="F564" s="14" t="s">
+      <c r="F564" s="50" t="s">
         <v>179</v>
       </c>
       <c r="G564" s="14" t="s">
@@ -41600,1124 +41608,1124 @@
   <dimension ref="A1:K39"/>
   <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="18.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="22.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="51" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="51" width="18.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="51" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="51" width="18.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="51" width="12.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="51" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="51" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="51" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="51" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="51" width="22.73"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="52" t="s">
         <v>354</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="53" t="s">
         <v>355</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
     </row>
     <row r="3" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="4" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="54" t="s">
         <v>356</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="B4" s="55" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="54" t="s">
+      <c r="A5" s="56" t="s">
         <v>358</v>
       </c>
-      <c r="B5" s="55" t="n">
-        <v>0.243</v>
-      </c>
-      <c r="C5" s="56" t="s">
+      <c r="B5" s="57" t="n">
+        <v>0.252</v>
+      </c>
+      <c r="C5" s="58" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="54" t="s">
+      <c r="A6" s="56" t="s">
         <v>360</v>
       </c>
-      <c r="B6" s="57" t="n">
+      <c r="B6" s="59" t="n">
         <v>60</v>
       </c>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="58" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="60" t="s">
         <v>362</v>
       </c>
-      <c r="B7" s="59" t="n">
+      <c r="B7" s="61" t="n">
         <f aca="true">TODAY()</f>
-        <v>46206</v>
+        <v>46207</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="60" t="s">
+      <c r="A9" s="62" t="s">
         <v>363</v>
       </c>
-      <c r="B9" s="60" t="s">
+      <c r="B9" s="62" t="s">
         <v>364</v>
       </c>
-      <c r="C9" s="60" t="s">
+      <c r="C9" s="62" t="s">
         <v>365</v>
       </c>
-      <c r="D9" s="60" t="s">
+      <c r="D9" s="62" t="s">
         <v>366</v>
       </c>
-      <c r="E9" s="60" t="s">
+      <c r="E9" s="62" t="s">
         <v>367</v>
       </c>
-      <c r="F9" s="60" t="s">
+      <c r="F9" s="62" t="s">
         <v>368</v>
       </c>
-      <c r="G9" s="60" t="s">
+      <c r="G9" s="62" t="s">
         <v>369</v>
       </c>
-      <c r="H9" s="60" t="s">
+      <c r="H9" s="62" t="s">
         <v>370</v>
       </c>
-      <c r="I9" s="60" t="s">
+      <c r="I9" s="62" t="s">
         <v>371</v>
       </c>
-      <c r="J9" s="60" t="s">
+      <c r="J9" s="62" t="s">
         <v>372</v>
       </c>
-      <c r="K9" s="60" t="s">
+      <c r="K9" s="62" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="61" t="n">
+      <c r="A10" s="63" t="n">
         <v>1998</v>
       </c>
-      <c r="B10" s="62" t="n">
+      <c r="B10" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C10" s="63" t="n">
+      <c r="C10" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D10" s="61" t="n">
+      <c r="D10" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E10" s="62" t="n">
+      <c r="E10" s="64" t="n">
         <f aca="false">C10+D10</f>
         <v>46095</v>
       </c>
-      <c r="F10" s="64" t="str">
+      <c r="F10" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G10" s="61" t="n">
+      <c r="G10" s="63" t="n">
         <f aca="false">IF(F10="",MAX(0,$B$7-E10),MAX(0,F10-E10))</f>
-        <v>111</v>
-      </c>
-      <c r="H10" s="65" t="n">
+        <v>112</v>
+      </c>
+      <c r="H10" s="67" t="n">
         <v>50402510.51</v>
       </c>
-      <c r="I10" s="66" t="n">
+      <c r="I10" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J10" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J10" s="69" t="n">
         <f aca="false">H10*I10*(G10/365)</f>
-        <v>4184513.08488912</v>
-      </c>
-      <c r="K10" s="68" t="n">
+        <v>4361405.18341874</v>
+      </c>
+      <c r="K10" s="70" t="n">
         <f aca="false">H10+J10</f>
-        <v>54587023.5948891</v>
+        <v>54763915.6934187</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="69" t="n">
+      <c r="A11" s="71" t="n">
         <v>1999</v>
       </c>
-      <c r="B11" s="70" t="n">
+      <c r="B11" s="72" t="n">
         <v>46035</v>
       </c>
-      <c r="C11" s="71" t="n">
+      <c r="C11" s="73" t="n">
         <v>46035</v>
       </c>
-      <c r="D11" s="69" t="n">
+      <c r="D11" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E11" s="70" t="n">
+      <c r="E11" s="72" t="n">
         <f aca="false">C11+D11</f>
         <v>46095</v>
       </c>
-      <c r="F11" s="64" t="str">
+      <c r="F11" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G11" s="69" t="n">
+      <c r="G11" s="71" t="n">
         <f aca="false">IF(F11="",MAX(0,$B$7-E11),MAX(0,F11-E11))</f>
-        <v>111</v>
-      </c>
-      <c r="H11" s="72" t="n">
+        <v>112</v>
+      </c>
+      <c r="H11" s="74" t="n">
         <v>677271.96</v>
       </c>
-      <c r="I11" s="66" t="n">
+      <c r="I11" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J11" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J11" s="75" t="n">
         <f aca="false">H11*I11*(G11/365)</f>
-        <v>56228.4169969315</v>
-      </c>
-      <c r="K11" s="74" t="n">
+        <v>58605.3632455891</v>
+      </c>
+      <c r="K11" s="76" t="n">
         <f aca="false">H11+J11</f>
-        <v>733500.376996932</v>
+        <v>735877.323245589</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="61" t="n">
+      <c r="A12" s="63" t="n">
         <v>2000</v>
       </c>
-      <c r="B12" s="62" t="n">
+      <c r="B12" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C12" s="63" t="n">
+      <c r="C12" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D12" s="61" t="n">
+      <c r="D12" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E12" s="62" t="n">
+      <c r="E12" s="64" t="n">
         <f aca="false">C12+D12</f>
         <v>46095</v>
       </c>
-      <c r="F12" s="64" t="str">
+      <c r="F12" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G12" s="61" t="n">
+      <c r="G12" s="63" t="n">
         <f aca="false">IF(F12="",MAX(0,$B$7-E12),MAX(0,F12-E12))</f>
-        <v>111</v>
-      </c>
-      <c r="H12" s="65" t="n">
+        <v>112</v>
+      </c>
+      <c r="H12" s="67" t="n">
         <v>17699825.4</v>
       </c>
-      <c r="I12" s="66" t="n">
+      <c r="I12" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J12" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J12" s="69" t="n">
         <f aca="false">H12*I12*(G12/365)</f>
-        <v>1469473.44957863</v>
-      </c>
-      <c r="K12" s="68" t="n">
+        <v>1531592.56283178</v>
+      </c>
+      <c r="K12" s="70" t="n">
         <f aca="false">H12+J12</f>
-        <v>19169298.8495786</v>
+        <v>19231417.9628318</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="69" t="n">
+      <c r="A13" s="71" t="n">
         <v>2001</v>
       </c>
-      <c r="B13" s="70" t="n">
+      <c r="B13" s="72" t="n">
         <v>46035</v>
       </c>
-      <c r="C13" s="71" t="n">
+      <c r="C13" s="73" t="n">
         <v>46035</v>
       </c>
-      <c r="D13" s="69" t="n">
+      <c r="D13" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E13" s="70" t="n">
+      <c r="E13" s="72" t="n">
         <f aca="false">C13+D13</f>
         <v>46095</v>
       </c>
-      <c r="F13" s="64" t="str">
+      <c r="F13" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G13" s="69" t="n">
+      <c r="G13" s="71" t="n">
         <f aca="false">IF(F13="",MAX(0,$B$7-E13),MAX(0,F13-E13))</f>
-        <v>111</v>
-      </c>
-      <c r="H13" s="72" t="n">
+        <v>112</v>
+      </c>
+      <c r="H13" s="74" t="n">
         <v>1015907.94</v>
       </c>
-      <c r="I13" s="66" t="n">
+      <c r="I13" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J13" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J13" s="75" t="n">
         <f aca="false">H13*I13*(G13/365)</f>
-        <v>84342.6254953973</v>
-      </c>
-      <c r="K13" s="74" t="n">
+        <v>87908.0448683836</v>
+      </c>
+      <c r="K13" s="76" t="n">
         <f aca="false">H13+J13</f>
-        <v>1100250.5654954</v>
+        <v>1103815.98486838</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="61" t="n">
+      <c r="A14" s="63" t="n">
         <v>2002</v>
       </c>
-      <c r="B14" s="62" t="n">
+      <c r="B14" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C14" s="63" t="n">
+      <c r="C14" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D14" s="61" t="n">
+      <c r="D14" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E14" s="62" t="n">
+      <c r="E14" s="64" t="n">
         <f aca="false">C14+D14</f>
         <v>46095</v>
       </c>
-      <c r="F14" s="64" t="str">
+      <c r="F14" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G14" s="61" t="n">
+      <c r="G14" s="63" t="n">
         <f aca="false">IF(F14="",MAX(0,$B$7-E14),MAX(0,F14-E14))</f>
-        <v>111</v>
-      </c>
-      <c r="H14" s="65" t="n">
+        <v>112</v>
+      </c>
+      <c r="H14" s="67" t="n">
         <v>27253875.19</v>
       </c>
-      <c r="I14" s="66" t="n">
+      <c r="I14" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J14" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J14" s="69" t="n">
         <f aca="false">H14*I14*(G14/365)</f>
-        <v>2262668.98597964</v>
-      </c>
-      <c r="K14" s="68" t="n">
+        <v>2358318.88767386</v>
+      </c>
+      <c r="K14" s="70" t="n">
         <f aca="false">H14+J14</f>
-        <v>29516544.1759796</v>
+        <v>29612194.0776739</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="69" t="n">
+      <c r="A15" s="71" t="n">
         <v>2003</v>
       </c>
-      <c r="B15" s="70" t="n">
+      <c r="B15" s="72" t="n">
         <v>46035</v>
       </c>
-      <c r="C15" s="71" t="n">
+      <c r="C15" s="73" t="n">
         <v>46035</v>
       </c>
-      <c r="D15" s="69" t="n">
+      <c r="D15" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E15" s="70" t="n">
+      <c r="E15" s="72" t="n">
         <f aca="false">C15+D15</f>
         <v>46095</v>
       </c>
-      <c r="F15" s="64" t="str">
+      <c r="F15" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G15" s="69" t="n">
+      <c r="G15" s="71" t="n">
         <f aca="false">IF(F15="",MAX(0,$B$7-E15),MAX(0,F15-E15))</f>
-        <v>111</v>
-      </c>
-      <c r="H15" s="72" t="n">
+        <v>112</v>
+      </c>
+      <c r="H15" s="74" t="n">
         <v>1015907.94</v>
       </c>
-      <c r="I15" s="66" t="n">
+      <c r="I15" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J15" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J15" s="75" t="n">
         <f aca="false">H15*I15*(G15/365)</f>
-        <v>84342.6254953973</v>
-      </c>
-      <c r="K15" s="74" t="n">
+        <v>87908.0448683836</v>
+      </c>
+      <c r="K15" s="76" t="n">
         <f aca="false">H15+J15</f>
-        <v>1100250.5654954</v>
+        <v>1103815.98486838</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="61" t="n">
+      <c r="A16" s="63" t="n">
         <v>2004</v>
       </c>
-      <c r="B16" s="62" t="n">
+      <c r="B16" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C16" s="63" t="n">
+      <c r="C16" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D16" s="61" t="n">
+      <c r="D16" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E16" s="62" t="n">
+      <c r="E16" s="64" t="n">
         <f aca="false">C16+D16</f>
         <v>46095</v>
       </c>
-      <c r="F16" s="64" t="str">
+      <c r="F16" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G16" s="61" t="n">
+      <c r="G16" s="63" t="n">
         <f aca="false">IF(F16="",MAX(0,$B$7-E16),MAX(0,F16-E16))</f>
-        <v>111</v>
-      </c>
-      <c r="H16" s="65" t="n">
+        <v>112</v>
+      </c>
+      <c r="H16" s="67" t="n">
         <v>28627721.36</v>
       </c>
-      <c r="I16" s="66" t="n">
+      <c r="I16" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J16" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J16" s="69" t="n">
         <f aca="false">H16*I16*(G16/365)</f>
-        <v>2376728.32978652</v>
-      </c>
-      <c r="K16" s="68" t="n">
+        <v>2477199.86694312</v>
+      </c>
+      <c r="K16" s="70" t="n">
         <f aca="false">H16+J16</f>
-        <v>31004449.6897865</v>
+        <v>31104921.2269431</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="69" t="n">
+      <c r="A17" s="71" t="n">
         <v>2005</v>
       </c>
-      <c r="B17" s="70" t="n">
+      <c r="B17" s="72" t="n">
         <v>46035</v>
       </c>
-      <c r="C17" s="71" t="n">
+      <c r="C17" s="73" t="n">
         <v>46035</v>
       </c>
-      <c r="D17" s="69" t="n">
+      <c r="D17" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E17" s="70" t="n">
+      <c r="E17" s="72" t="n">
         <f aca="false">C17+D17</f>
         <v>46095</v>
       </c>
-      <c r="F17" s="64" t="str">
+      <c r="F17" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G17" s="69" t="n">
+      <c r="G17" s="71" t="n">
         <f aca="false">IF(F17="",MAX(0,$B$7-E17),MAX(0,F17-E17))</f>
-        <v>111</v>
-      </c>
-      <c r="H17" s="72" t="n">
+        <v>112</v>
+      </c>
+      <c r="H17" s="74" t="n">
         <v>238400.46</v>
       </c>
-      <c r="I17" s="66" t="n">
+      <c r="I17" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J17" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J17" s="75" t="n">
         <f aca="false">H17*I17*(G17/365)</f>
-        <v>19792.4633955617</v>
-      </c>
-      <c r="K17" s="74" t="n">
+        <v>20629.1510373699</v>
+      </c>
+      <c r="K17" s="76" t="n">
         <f aca="false">H17+J17</f>
-        <v>258192.923395562</v>
+        <v>259029.61103737</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="61" t="n">
+      <c r="A18" s="63" t="n">
         <v>2006</v>
       </c>
-      <c r="B18" s="62" t="n">
+      <c r="B18" s="64" t="n">
         <v>46035</v>
       </c>
-      <c r="C18" s="63" t="n">
+      <c r="C18" s="65" t="n">
         <v>46035</v>
       </c>
-      <c r="D18" s="61" t="n">
+      <c r="D18" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E18" s="62" t="n">
+      <c r="E18" s="64" t="n">
         <f aca="false">C18+D18</f>
         <v>46095</v>
       </c>
-      <c r="F18" s="64" t="str">
+      <c r="F18" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G18" s="61" t="n">
+      <c r="G18" s="63" t="n">
         <f aca="false">IF(F18="",MAX(0,$B$7-E18),MAX(0,F18-E18))</f>
-        <v>111</v>
-      </c>
-      <c r="H18" s="65" t="n">
+        <v>112</v>
+      </c>
+      <c r="H18" s="67" t="n">
         <v>6758414.64</v>
       </c>
-      <c r="I18" s="66" t="n">
+      <c r="I18" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J18" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J18" s="69" t="n">
         <f aca="false">H18*I18*(G18/365)</f>
-        <v>561096.544755945</v>
-      </c>
-      <c r="K18" s="68" t="n">
+        <v>584815.802711671</v>
+      </c>
+      <c r="K18" s="70" t="n">
         <f aca="false">H18+J18</f>
-        <v>7319511.18475595</v>
+        <v>7343230.44271167</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="69" t="n">
+      <c r="A19" s="71" t="n">
         <v>2008</v>
       </c>
-      <c r="B19" s="70" t="n">
+      <c r="B19" s="72" t="n">
         <v>46051</v>
       </c>
-      <c r="C19" s="71" t="n">
+      <c r="C19" s="73" t="n">
         <v>46051</v>
       </c>
-      <c r="D19" s="69" t="n">
+      <c r="D19" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E19" s="70" t="n">
+      <c r="E19" s="72" t="n">
         <f aca="false">C19+D19</f>
         <v>46111</v>
       </c>
-      <c r="F19" s="64" t="str">
+      <c r="F19" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G19" s="69" t="n">
+      <c r="G19" s="71" t="n">
         <f aca="false">IF(F19="",MAX(0,$B$7-E19),MAX(0,F19-E19))</f>
-        <v>95</v>
-      </c>
-      <c r="H19" s="72" t="n">
+        <v>96</v>
+      </c>
+      <c r="H19" s="74" t="n">
         <v>444448.23</v>
       </c>
-      <c r="I19" s="66" t="n">
+      <c r="I19" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J19" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J19" s="75" t="n">
         <f aca="false">H19*I19*(G19/365)</f>
-        <v>31580.1776576712</v>
-      </c>
-      <c r="K19" s="74" t="n">
+        <v>32964.6643357808</v>
+      </c>
+      <c r="K19" s="76" t="n">
         <f aca="false">H19+J19</f>
-        <v>476028.407657671</v>
+        <v>477412.894335781</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="61" t="n">
+      <c r="A20" s="63" t="n">
         <v>2010</v>
       </c>
-      <c r="B20" s="62" t="n">
+      <c r="B20" s="64" t="n">
         <v>46051</v>
       </c>
-      <c r="C20" s="63" t="n">
+      <c r="C20" s="65" t="n">
         <v>46051</v>
       </c>
-      <c r="D20" s="61" t="n">
+      <c r="D20" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E20" s="62" t="n">
+      <c r="E20" s="64" t="n">
         <f aca="false">C20+D20</f>
         <v>46111</v>
       </c>
-      <c r="F20" s="64" t="str">
+      <c r="F20" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G20" s="61" t="n">
+      <c r="G20" s="63" t="n">
         <f aca="false">IF(F20="",MAX(0,$B$7-E20),MAX(0,F20-E20))</f>
-        <v>95</v>
-      </c>
-      <c r="H20" s="65" t="n">
+        <v>96</v>
+      </c>
+      <c r="H20" s="67" t="n">
         <v>12832109.38</v>
       </c>
-      <c r="I20" s="66" t="n">
+      <c r="I20" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J20" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J20" s="69" t="n">
         <f aca="false">H20*I20*(G20/365)</f>
-        <v>911782.895261096</v>
-      </c>
-      <c r="K20" s="68" t="n">
+        <v>951755.794891397</v>
+      </c>
+      <c r="K20" s="70" t="n">
         <f aca="false">H20+J20</f>
-        <v>13743892.2752611</v>
+        <v>13783865.1748914</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="69" t="n">
+      <c r="A21" s="71" t="n">
         <v>2011</v>
       </c>
-      <c r="B21" s="70" t="n">
+      <c r="B21" s="72" t="n">
         <v>46056</v>
       </c>
-      <c r="C21" s="71" t="n">
+      <c r="C21" s="73" t="n">
         <v>46056</v>
       </c>
-      <c r="D21" s="69" t="n">
+      <c r="D21" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E21" s="70" t="n">
+      <c r="E21" s="72" t="n">
         <f aca="false">C21+D21</f>
         <v>46116</v>
       </c>
-      <c r="F21" s="64" t="str">
+      <c r="F21" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G21" s="69" t="n">
+      <c r="G21" s="71" t="n">
         <f aca="false">IF(F21="",MAX(0,$B$7-E21),MAX(0,F21-E21))</f>
-        <v>90</v>
-      </c>
-      <c r="H21" s="72" t="n">
+        <v>91</v>
+      </c>
+      <c r="H21" s="74" t="n">
         <v>184056.25</v>
       </c>
-      <c r="I21" s="66" t="n">
+      <c r="I21" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J21" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J21" s="75" t="n">
         <f aca="false">H21*I21*(G21/365)</f>
-        <v>12389.7590753425</v>
-      </c>
-      <c r="K21" s="74" t="n">
+        <v>12940.4150342466</v>
+      </c>
+      <c r="K21" s="76" t="n">
         <f aca="false">H21+J21</f>
-        <v>196446.009075342</v>
+        <v>196996.665034247</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="61" t="n">
+      <c r="A22" s="63" t="n">
         <v>2012</v>
       </c>
-      <c r="B22" s="62" t="n">
+      <c r="B22" s="64" t="n">
         <v>46056</v>
       </c>
-      <c r="C22" s="63" t="n">
+      <c r="C22" s="65" t="n">
         <v>46056</v>
       </c>
-      <c r="D22" s="61" t="n">
+      <c r="D22" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E22" s="62" t="n">
+      <c r="E22" s="64" t="n">
         <f aca="false">C22+D22</f>
         <v>46116</v>
       </c>
-      <c r="F22" s="64" t="str">
+      <c r="F22" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G22" s="61" t="n">
+      <c r="G22" s="63" t="n">
         <f aca="false">IF(F22="",MAX(0,$B$7-E22),MAX(0,F22-E22))</f>
-        <v>90</v>
-      </c>
-      <c r="H22" s="65" t="n">
+        <v>91</v>
+      </c>
+      <c r="H22" s="67" t="n">
         <v>5425916.78</v>
       </c>
-      <c r="I22" s="66" t="n">
+      <c r="I22" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J22" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J22" s="69" t="n">
         <f aca="false">H22*I22*(G22/365)</f>
-        <v>365245.959683836</v>
-      </c>
-      <c r="K22" s="68" t="n">
+        <v>381479.113447562</v>
+      </c>
+      <c r="K22" s="70" t="n">
         <f aca="false">H22+J22</f>
-        <v>5791162.73968384</v>
+        <v>5807395.89344756</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="69" t="n">
+      <c r="A23" s="71" t="n">
         <v>2013</v>
       </c>
-      <c r="B23" s="70" t="n">
+      <c r="B23" s="72" t="n">
         <v>46056</v>
       </c>
-      <c r="C23" s="71" t="n">
+      <c r="C23" s="73" t="n">
         <v>46056</v>
       </c>
-      <c r="D23" s="69" t="n">
+      <c r="D23" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E23" s="70" t="n">
+      <c r="E23" s="72" t="n">
         <f aca="false">C23+D23</f>
         <v>46116</v>
       </c>
-      <c r="F23" s="64" t="str">
+      <c r="F23" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G23" s="69" t="n">
+      <c r="G23" s="71" t="n">
         <f aca="false">IF(F23="",MAX(0,$B$7-E23),MAX(0,F23-E23))</f>
-        <v>90</v>
-      </c>
-      <c r="H23" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="66" t="n">
+        <v>91</v>
+      </c>
+      <c r="H23" s="74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J23" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J23" s="75" t="n">
         <f aca="false">H23*I23*(G23/365)</f>
         <v>0</v>
       </c>
-      <c r="K23" s="74" t="n">
+      <c r="K23" s="76" t="n">
         <f aca="false">H23+J23</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="61" t="n">
+      <c r="A24" s="63" t="n">
         <v>2014</v>
       </c>
-      <c r="B24" s="62" t="n">
+      <c r="B24" s="64" t="n">
         <v>46059</v>
       </c>
-      <c r="C24" s="63" t="n">
+      <c r="C24" s="65" t="n">
         <v>46059</v>
       </c>
-      <c r="D24" s="61" t="n">
+      <c r="D24" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E24" s="62" t="n">
+      <c r="E24" s="64" t="n">
         <f aca="false">C24+D24</f>
         <v>46119</v>
       </c>
-      <c r="F24" s="64" t="str">
+      <c r="F24" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G24" s="61" t="n">
+      <c r="G24" s="63" t="n">
         <f aca="false">IF(F24="",MAX(0,$B$7-E24),MAX(0,F24-E24))</f>
-        <v>87</v>
-      </c>
-      <c r="H24" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="66" t="n">
+        <v>88</v>
+      </c>
+      <c r="H24" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J24" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J24" s="69" t="n">
         <f aca="false">H24*I24*(G24/365)</f>
         <v>0</v>
       </c>
-      <c r="K24" s="68" t="n">
+      <c r="K24" s="70" t="n">
         <f aca="false">H24+J24</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="69" t="n">
+      <c r="A25" s="71" t="n">
         <v>2015</v>
       </c>
-      <c r="B25" s="70" t="n">
+      <c r="B25" s="72" t="n">
         <v>46098</v>
       </c>
-      <c r="C25" s="71" t="n">
+      <c r="C25" s="73" t="n">
         <v>46098</v>
       </c>
-      <c r="D25" s="69" t="n">
+      <c r="D25" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E25" s="70" t="n">
+      <c r="E25" s="72" t="n">
         <f aca="false">C25+D25</f>
         <v>46158</v>
       </c>
-      <c r="F25" s="64" t="str">
+      <c r="F25" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G25" s="69" t="n">
+      <c r="G25" s="71" t="n">
         <f aca="false">IF(F25="",MAX(0,$B$7-E25),MAX(0,F25-E25))</f>
-        <v>48</v>
-      </c>
-      <c r="H25" s="72" t="n">
+        <v>49</v>
+      </c>
+      <c r="H25" s="74" t="n">
         <v>203181.59</v>
       </c>
-      <c r="I25" s="66" t="n">
+      <c r="I25" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J25" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J25" s="75" t="n">
         <f aca="false">H25*I25*(G25/365)</f>
-        <v>7294.49741194521</v>
-      </c>
-      <c r="K25" s="74" t="n">
+        <v>7691.95400169863</v>
+      </c>
+      <c r="K25" s="76" t="n">
         <f aca="false">H25+J25</f>
-        <v>210476.087411945</v>
+        <v>210873.544001699</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="61" t="n">
+      <c r="A26" s="63" t="n">
         <v>2016</v>
       </c>
-      <c r="B26" s="62" t="n">
+      <c r="B26" s="64" t="n">
         <v>46098</v>
       </c>
-      <c r="C26" s="63" t="n">
+      <c r="C26" s="65" t="n">
         <v>46098</v>
       </c>
-      <c r="D26" s="61" t="n">
+      <c r="D26" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E26" s="62" t="n">
+      <c r="E26" s="64" t="n">
         <f aca="false">C26+D26</f>
         <v>46158</v>
       </c>
-      <c r="F26" s="64" t="str">
+      <c r="F26" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G26" s="61" t="n">
+      <c r="G26" s="63" t="n">
         <f aca="false">IF(F26="",MAX(0,$B$7-E26),MAX(0,F26-E26))</f>
-        <v>48</v>
-      </c>
-      <c r="H26" s="65" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="66" t="n">
+        <v>49</v>
+      </c>
+      <c r="H26" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J26" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J26" s="69" t="n">
         <f aca="false">H26*I26*(G26/365)</f>
         <v>0</v>
       </c>
-      <c r="K26" s="68" t="n">
+      <c r="K26" s="70" t="n">
         <f aca="false">H26+J26</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="69" t="n">
+      <c r="A27" s="71" t="n">
         <v>2017</v>
       </c>
-      <c r="B27" s="70" t="n">
+      <c r="B27" s="72" t="n">
         <v>46098</v>
       </c>
-      <c r="C27" s="71" t="n">
+      <c r="C27" s="73" t="n">
         <v>46098</v>
       </c>
-      <c r="D27" s="69" t="n">
+      <c r="D27" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E27" s="70" t="n">
+      <c r="E27" s="72" t="n">
         <f aca="false">C27+D27</f>
         <v>46158</v>
       </c>
-      <c r="F27" s="64" t="str">
+      <c r="F27" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G27" s="69" t="n">
+      <c r="G27" s="71" t="n">
         <f aca="false">IF(F27="",MAX(0,$B$7-E27),MAX(0,F27-E27))</f>
-        <v>48</v>
-      </c>
-      <c r="H27" s="72" t="n">
+        <v>49</v>
+      </c>
+      <c r="H27" s="74" t="n">
         <v>6266255.63</v>
       </c>
-      <c r="I27" s="66" t="n">
+      <c r="I27" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J27" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J27" s="75" t="n">
         <f aca="false">H27*I27*(G27/365)</f>
-        <v>224967.161028822</v>
-      </c>
-      <c r="K27" s="74" t="n">
+        <v>237224.987110521</v>
+      </c>
+      <c r="K27" s="76" t="n">
         <f aca="false">H27+J27</f>
-        <v>6491222.79102882</v>
+        <v>6503480.61711052</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="61" t="n">
+      <c r="A28" s="63" t="n">
         <v>2018</v>
       </c>
-      <c r="B28" s="62" t="n">
+      <c r="B28" s="64" t="n">
         <v>46122</v>
       </c>
-      <c r="C28" s="63" t="n">
+      <c r="C28" s="65" t="n">
         <v>46122</v>
       </c>
-      <c r="D28" s="61" t="n">
+      <c r="D28" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E28" s="62" t="n">
+      <c r="E28" s="64" t="n">
         <f aca="false">C28+D28</f>
         <v>46182</v>
       </c>
-      <c r="F28" s="64" t="str">
+      <c r="F28" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G28" s="61" t="n">
+      <c r="G28" s="63" t="n">
         <f aca="false">IF(F28="",MAX(0,$B$7-E28),MAX(0,F28-E28))</f>
-        <v>24</v>
-      </c>
-      <c r="H28" s="65" t="n">
+        <v>25</v>
+      </c>
+      <c r="H28" s="67" t="n">
         <v>633024.04</v>
       </c>
-      <c r="I28" s="66" t="n">
+      <c r="I28" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J28" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J28" s="69" t="n">
         <f aca="false">H28*I28*(G28/365)</f>
-        <v>11363.2150961096</v>
-      </c>
-      <c r="K28" s="68" t="n">
+        <v>12226.902690411</v>
+      </c>
+      <c r="K28" s="70" t="n">
         <f aca="false">H28+J28</f>
-        <v>644387.25509611</v>
+        <v>645250.942690411</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="69" t="n">
+      <c r="A29" s="71" t="n">
         <v>2019</v>
       </c>
-      <c r="B29" s="70" t="n">
+      <c r="B29" s="72" t="n">
         <v>46122</v>
       </c>
-      <c r="C29" s="71" t="n">
+      <c r="C29" s="73" t="n">
         <v>46122</v>
       </c>
-      <c r="D29" s="69" t="n">
+      <c r="D29" s="71" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E29" s="70" t="n">
+      <c r="E29" s="72" t="n">
         <f aca="false">C29+D29</f>
         <v>46182</v>
       </c>
-      <c r="F29" s="64" t="str">
+      <c r="F29" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G29" s="69" t="n">
+      <c r="G29" s="71" t="n">
         <f aca="false">IF(F29="",MAX(0,$B$7-E29),MAX(0,F29-E29))</f>
-        <v>24</v>
-      </c>
-      <c r="H29" s="72" t="n">
+        <v>25</v>
+      </c>
+      <c r="H29" s="74" t="n">
         <v>19702240.1</v>
       </c>
-      <c r="I29" s="75" t="n">
+      <c r="I29" s="77" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J29" s="73" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J29" s="75" t="n">
         <f aca="false">H29*I29*(G29/365)</f>
-        <v>353668.70448</v>
-      </c>
-      <c r="K29" s="74" t="n">
+        <v>380550.117</v>
+      </c>
+      <c r="K29" s="76" t="n">
         <f aca="false">H29+J29</f>
-        <v>20055908.80448</v>
+        <v>20082790.217</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="61" t="n">
+      <c r="A30" s="63" t="n">
         <v>2021</v>
       </c>
-      <c r="B30" s="62" t="n">
+      <c r="B30" s="64" t="n">
         <v>46122</v>
       </c>
-      <c r="C30" s="63" t="n">
+      <c r="C30" s="65" t="n">
         <v>46122</v>
       </c>
-      <c r="D30" s="61" t="n">
+      <c r="D30" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E30" s="62" t="n">
+      <c r="E30" s="64" t="n">
         <f aca="false">C30+D30</f>
         <v>46182</v>
       </c>
-      <c r="F30" s="64" t="str">
+      <c r="F30" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G30" s="61" t="n">
+      <c r="G30" s="63" t="n">
         <f aca="false">IF(F30="",MAX(0,$B$7-E30),MAX(0,F30-E30))</f>
-        <v>24</v>
-      </c>
-      <c r="H30" s="65" t="n">
+        <v>25</v>
+      </c>
+      <c r="H30" s="67" t="n">
         <v>95946.87</v>
       </c>
-      <c r="I30" s="66" t="n">
+      <c r="I30" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J30" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J30" s="69" t="n">
         <f aca="false">H30*I30*(G30/365)</f>
-        <v>1722.31203353425</v>
-      </c>
-      <c r="K30" s="68" t="n">
+        <v>1853.22036575342</v>
+      </c>
+      <c r="K30" s="70" t="n">
         <f aca="false">H30+J30</f>
-        <v>97669.1820335343</v>
+        <v>97800.0903657534</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="61" t="n">
+      <c r="A31" s="63" t="n">
         <v>2024</v>
       </c>
-      <c r="B31" s="62" t="n">
+      <c r="B31" s="64" t="n">
         <v>46142</v>
       </c>
-      <c r="C31" s="63" t="n">
+      <c r="C31" s="65" t="n">
         <v>46142</v>
       </c>
-      <c r="D31" s="61" t="n">
+      <c r="D31" s="63" t="n">
         <f aca="false">$B$6</f>
         <v>60</v>
       </c>
-      <c r="E31" s="62" t="n">
+      <c r="E31" s="64" t="n">
         <f aca="false">C31+D31</f>
         <v>46202</v>
       </c>
-      <c r="F31" s="64" t="str">
+      <c r="F31" s="66" t="str">
         <f aca="false">""</f>
         <v/>
       </c>
-      <c r="G31" s="61" t="n">
+      <c r="G31" s="63" t="n">
         <f aca="false">IF(F31="",MAX(0,$B$7-E31),MAX(0,F31-E31))</f>
-        <v>4</v>
-      </c>
-      <c r="H31" s="65" t="n">
+        <v>5</v>
+      </c>
+      <c r="H31" s="67" t="n">
         <v>131593300.43</v>
       </c>
-      <c r="I31" s="66" t="n">
+      <c r="I31" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.273</v>
-      </c>
-      <c r="J31" s="67" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J31" s="69" t="n">
         <f aca="false">H31*I31*(G31/365)</f>
-        <v>393698.312519343</v>
-      </c>
-      <c r="K31" s="68" t="n">
+        <v>508346.722209041</v>
+      </c>
+      <c r="K31" s="70" t="n">
         <f aca="false">H31+J31</f>
-        <v>131986998.742519</v>
+        <v>132101647.152209</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="76" t="s">
+      <c r="A32" s="78" t="s">
         <v>374</v>
       </c>
-      <c r="B32" s="76"/>
-      <c r="C32" s="76"/>
-      <c r="D32" s="76"/>
-      <c r="E32" s="76"/>
-      <c r="F32" s="76"/>
-      <c r="G32" s="77" t="n">
+      <c r="B32" s="78"/>
+      <c r="C32" s="78"/>
+      <c r="D32" s="78"/>
+      <c r="E32" s="78"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="79" t="n">
         <f aca="false">IF(COUNTA(F10:F31)&gt;0,AVERAGE(G10:G31),AVERAGE(G10:G31))</f>
-        <v>80.2727272727273</v>
-      </c>
-      <c r="H32" s="78" t="n">
+        <v>81.2727272727273</v>
+      </c>
+      <c r="H32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,H10:H31)</f>
         <v>311070314.7</v>
       </c>
-      <c r="I32" s="76"/>
-      <c r="J32" s="78" t="n">
+      <c r="I32" s="78"/>
+      <c r="J32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,J10:J31)</f>
-        <v>13412899.5206209</v>
-      </c>
-      <c r="K32" s="78" t="n">
+        <v>14095416.7986853</v>
+      </c>
+      <c r="K32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,K10:K31)</f>
-        <v>324483214.220621</v>
+        <v>325165731.498685</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="79" t="s">
+      <c r="A34" s="81" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="54" t="s">
+      <c r="A35" s="56" t="s">
         <v>376</v>
       </c>
-      <c r="B35" s="80" t="n">
+      <c r="B35" s="82" t="n">
         <f aca="false">H32</f>
         <v>311070314.7</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="54" t="s">
+      <c r="A36" s="56" t="s">
         <v>377</v>
       </c>
-      <c r="B36" s="80" t="n">
+      <c r="B36" s="82" t="n">
         <f aca="false">J32</f>
-        <v>13412899.5206209</v>
+        <v>14095416.7986853</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="81" t="s">
+      <c r="A37" s="83" t="s">
         <v>378</v>
       </c>
-      <c r="B37" s="82" t="n">
+      <c r="B37" s="84" t="n">
         <f aca="false">B35+B36</f>
-        <v>324483214.220621</v>
+        <v>325165731.498685</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="58" t="s">
+      <c r="A38" s="60" t="s">
         <v>379</v>
       </c>
-      <c r="B38" s="83" t="n">
+      <c r="B38" s="85" t="n">
         <f aca="false">COUNTIF(G10:G31,"&gt;"&amp;0)</f>
         <v>22</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="58" t="s">
+      <c r="A39" s="60" t="s">
         <v>380</v>
       </c>
-      <c r="B39" s="84" t="n">
+      <c r="B39" s="86" t="n">
         <f aca="false">G32</f>
-        <v>80.2727272727273</v>
+        <v>81.2727272727273</v>
       </c>
     </row>
   </sheetData>
@@ -42743,307 +42751,307 @@
   <dimension ref="A1:K8"/>
   <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="25.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="85" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="51" width="14.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="51" width="50.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="51" width="32.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="16.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="51" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="51" width="21.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="51" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="51" width="23.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="51" width="25.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="87" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="86" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="86" t="s">
+      <c r="A1" s="88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="86" t="s">
+      <c r="C1" s="88" t="s">
         <v>381</v>
       </c>
-      <c r="D1" s="86" t="s">
+      <c r="D1" s="88" t="s">
         <v>382</v>
       </c>
-      <c r="E1" s="86" t="s">
+      <c r="E1" s="88" t="s">
         <v>383</v>
       </c>
-      <c r="F1" s="86" t="s">
+      <c r="F1" s="88" t="s">
         <v>384</v>
       </c>
-      <c r="G1" s="87" t="s">
+      <c r="G1" s="89" t="s">
         <v>385</v>
       </c>
-      <c r="H1" s="87" t="s">
+      <c r="H1" s="89" t="s">
         <v>386</v>
       </c>
-      <c r="I1" s="87" t="s">
+      <c r="I1" s="89" t="s">
         <v>387</v>
       </c>
-      <c r="J1" s="87" t="s">
+      <c r="J1" s="89" t="s">
         <v>388</v>
       </c>
-      <c r="K1" s="88" t="s">
+      <c r="K1" s="90" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="89" t="s">
+      <c r="A2" s="91" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="90" t="s">
+      <c r="B2" s="92" t="s">
         <v>124</v>
       </c>
-      <c r="C2" s="91" t="s">
+      <c r="C2" s="93" t="s">
         <v>390</v>
       </c>
-      <c r="D2" s="89" t="n">
+      <c r="D2" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="89" t="s">
+      <c r="E2" s="91" t="s">
         <v>391</v>
       </c>
-      <c r="F2" s="92" t="n">
+      <c r="F2" s="94" t="n">
         <v>45938</v>
       </c>
-      <c r="G2" s="93" t="n">
+      <c r="G2" s="95" t="n">
         <v>21615296.4</v>
       </c>
-      <c r="H2" s="93"/>
-      <c r="I2" s="94" t="n">
+      <c r="H2" s="95"/>
+      <c r="I2" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!D:D,"Provision Tableros electricos")</f>
         <v>14902219.87</v>
       </c>
-      <c r="J2" s="94" t="n">
+      <c r="J2" s="96" t="n">
         <f aca="false">G2-I2</f>
         <v>6713076.53</v>
       </c>
-      <c r="K2" s="95" t="n">
+      <c r="K2" s="97" t="n">
         <f aca="false">IFERROR(I2/G2,0)</f>
         <v>0.689429355685356</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="89" t="s">
+      <c r="A3" s="91" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="90" t="s">
+      <c r="B3" s="92" t="s">
         <v>124</v>
       </c>
-      <c r="C3" s="91" t="s">
+      <c r="C3" s="93" t="s">
         <v>392</v>
       </c>
-      <c r="D3" s="89" t="n">
+      <c r="D3" s="91" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="89" t="s">
+      <c r="E3" s="91" t="s">
         <v>393</v>
       </c>
-      <c r="F3" s="92" t="n">
+      <c r="F3" s="94" t="n">
         <v>46078</v>
       </c>
-      <c r="G3" s="93" t="n">
+      <c r="G3" s="95" t="n">
         <v>48893832.04</v>
       </c>
-      <c r="H3" s="93"/>
-      <c r="I3" s="94" t="n">
+      <c r="H3" s="95"/>
+      <c r="I3" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!D:D,"Conexión y Cableado")</f>
         <v>41888536.4</v>
       </c>
-      <c r="J3" s="94" t="n">
+      <c r="J3" s="96" t="n">
         <f aca="false">G3-I3</f>
         <v>7005295.64</v>
       </c>
-      <c r="K3" s="95" t="n">
+      <c r="K3" s="97" t="n">
         <f aca="false">IFERROR(I3/G3,0)</f>
         <v>0.856724348497189</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="91" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="90" t="s">
+      <c r="B4" s="92" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="91" t="s">
+      <c r="C4" s="93" t="s">
         <v>394</v>
       </c>
-      <c r="D4" s="89" t="n">
+      <c r="D4" s="91" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="89" t="s">
+      <c r="E4" s="91" t="s">
         <v>395</v>
       </c>
-      <c r="F4" s="92" t="n">
+      <c r="F4" s="94" t="n">
         <v>45904</v>
       </c>
-      <c r="G4" s="93" t="n">
+      <c r="G4" s="95" t="n">
         <v>81685880</v>
       </c>
-      <c r="H4" s="93"/>
-      <c r="I4" s="94" t="n">
+      <c r="H4" s="95"/>
+      <c r="I4" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!D:D,"Manifold y Tableros")</f>
         <v>75806304.84</v>
       </c>
-      <c r="J4" s="94" t="n">
+      <c r="J4" s="96" t="n">
         <f aca="false">G4-I4</f>
         <v>5879575.16</v>
       </c>
-      <c r="K4" s="95" t="n">
+      <c r="K4" s="97" t="n">
         <f aca="false">IFERROR(I4/G4,0)</f>
         <v>0.928022136016653</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="89" t="s">
+      <c r="A5" s="91" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="90" t="s">
+      <c r="B5" s="92" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="91" t="s">
+      <c r="C5" s="93" t="s">
         <v>396</v>
       </c>
-      <c r="D5" s="89" t="n">
+      <c r="D5" s="91" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="89" t="s">
+      <c r="E5" s="91" t="s">
         <v>397</v>
       </c>
-      <c r="F5" s="92" t="n">
+      <c r="F5" s="94" t="n">
         <v>45916</v>
       </c>
-      <c r="G5" s="93" t="n">
+      <c r="G5" s="95" t="n">
         <v>12601653.25</v>
       </c>
-      <c r="H5" s="93"/>
-      <c r="I5" s="94" t="n">
+      <c r="H5" s="95"/>
+      <c r="I5" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!D:D,"Oficina Tecnica")</f>
         <v>0</v>
       </c>
-      <c r="J5" s="94" t="n">
+      <c r="J5" s="96" t="n">
         <f aca="false">G5-I5</f>
         <v>12601653.25</v>
       </c>
-      <c r="K5" s="95" t="n">
+      <c r="K5" s="97" t="n">
         <f aca="false">IFERROR(I5/G5,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="89" t="s">
+      <c r="A6" s="91" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="90" t="s">
+      <c r="B6" s="92" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="91" t="s">
+      <c r="C6" s="93" t="s">
         <v>398</v>
       </c>
-      <c r="D6" s="89" t="n">
+      <c r="D6" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="89" t="s">
+      <c r="E6" s="91" t="s">
         <v>399</v>
       </c>
-      <c r="F6" s="92" t="n">
+      <c r="F6" s="94" t="n">
         <v>44308</v>
       </c>
-      <c r="G6" s="93" t="n">
+      <c r="G6" s="95" t="n">
         <v>175969573.995</v>
       </c>
-      <c r="H6" s="93"/>
-      <c r="I6" s="94" t="n">
+      <c r="H6" s="95"/>
+      <c r="I6" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!A:A,A6)</f>
         <v>58113632.447</v>
       </c>
-      <c r="J6" s="94" t="n">
+      <c r="J6" s="96" t="n">
         <f aca="false">G6-I6</f>
         <v>117855941.548</v>
       </c>
-      <c r="K6" s="95" t="n">
+      <c r="K6" s="97" t="n">
         <f aca="false">IFERROR(I6/G6,0)</f>
         <v>0.330248185113247</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="89" t="s">
+      <c r="A7" s="91" t="s">
         <v>197</v>
       </c>
-      <c r="B7" s="90" t="s">
+      <c r="B7" s="92" t="s">
         <v>198</v>
       </c>
-      <c r="C7" s="91" t="s">
+      <c r="C7" s="93" t="s">
         <v>398</v>
       </c>
-      <c r="D7" s="89" t="n">
+      <c r="D7" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="89" t="s">
+      <c r="E7" s="91" t="s">
         <v>400</v>
       </c>
-      <c r="F7" s="92" t="n">
+      <c r="F7" s="94" t="n">
         <v>46007</v>
       </c>
-      <c r="G7" s="93" t="n">
+      <c r="G7" s="95" t="n">
         <v>3390677291.57</v>
       </c>
-      <c r="H7" s="93" t="n">
+      <c r="H7" s="95" t="n">
         <f aca="false">+G7*1.044428</f>
         <v>3541318302.27987</v>
       </c>
-      <c r="I7" s="94" t="n">
+      <c r="I7" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!A:A,A7)</f>
         <v>3541317286.68</v>
       </c>
-      <c r="J7" s="94" t="n">
+      <c r="J7" s="96" t="n">
         <f aca="false">H7-I7</f>
         <v>1015.59987211227</v>
       </c>
-      <c r="K7" s="95" t="n">
+      <c r="K7" s="97" t="n">
         <f aca="false">IFERROR(I7/H7,0)</f>
         <v>0.99999971321418</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="89" t="s">
+      <c r="A8" s="91" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="90" t="s">
+      <c r="B8" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="91" t="s">
+      <c r="C8" s="93" t="s">
         <v>398</v>
       </c>
-      <c r="D8" s="89" t="n">
+      <c r="D8" s="91" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="96" t="s">
+      <c r="E8" s="98" t="s">
         <v>401</v>
       </c>
-      <c r="F8" s="92" t="n">
+      <c r="F8" s="94" t="n">
         <v>46007</v>
       </c>
-      <c r="G8" s="93" t="n">
+      <c r="G8" s="95" t="n">
         <v>4837006176.45</v>
       </c>
-      <c r="H8" s="93" t="n">
+      <c r="H8" s="95" t="n">
         <f aca="false">+I8</f>
         <v>5105960136.19</v>
       </c>
-      <c r="I8" s="94" t="n">
+      <c r="I8" s="96" t="n">
         <f aca="false">SUMIFS(Master!I:I,Master!A:A,A8)</f>
         <v>5105960136.19</v>
       </c>
-      <c r="J8" s="94" t="n">
+      <c r="J8" s="96" t="n">
         <f aca="false">H8-I8</f>
         <v>0</v>
       </c>
-      <c r="K8" s="95" t="n">
+      <c r="K8" s="97" t="n">
         <f aca="false">IFERROR(I8/H8,0)</f>
         <v>1</v>
       </c>
@@ -43067,22 +43075,22 @@
   <dimension ref="A2:D9"/>
   <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="51" width="22.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="51" width="19.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="11.45"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="97" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="97" t="s">
+      <c r="A2" s="99" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="97" t="s">
+      <c r="C2" s="99" t="s">
         <v>402</v>
       </c>
-      <c r="D2" s="97" t="s">
+      <c r="D2" s="99" t="s">
         <v>403</v>
       </c>
     </row>
@@ -43090,13 +43098,13 @@
       <c r="A3" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="51" t="s">
         <v>404</v>
       </c>
-      <c r="C3" s="98" t="n">
+      <c r="C3" s="100" t="n">
         <v>1759695739.95</v>
       </c>
-      <c r="D3" s="99" t="n">
+      <c r="D3" s="101" t="n">
         <v>44256</v>
       </c>
     </row>
@@ -43104,13 +43112,13 @@
       <c r="A4" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="51" t="s">
         <v>405</v>
       </c>
-      <c r="C4" s="98" t="n">
+      <c r="C4" s="100" t="n">
         <v>351934615.48</v>
       </c>
-      <c r="D4" s="99" t="n">
+      <c r="D4" s="101" t="n">
         <v>46042</v>
       </c>
     </row>
@@ -43118,13 +43126,13 @@
       <c r="A5" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="51" t="s">
         <v>406</v>
       </c>
-      <c r="C5" s="98" t="n">
+      <c r="C5" s="100" t="n">
         <v>2337056186.58</v>
       </c>
-      <c r="D5" s="99" t="n">
+      <c r="D5" s="101" t="n">
         <v>45870</v>
       </c>
     </row>
@@ -43132,13 +43140,13 @@
       <c r="A6" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="51" t="s">
         <v>406</v>
       </c>
-      <c r="C6" s="98" t="n">
+      <c r="C6" s="100" t="n">
         <v>5000000000</v>
       </c>
-      <c r="D6" s="99" t="n">
+      <c r="D6" s="101" t="n">
         <v>46113</v>
       </c>
     </row>
@@ -43146,13 +43154,13 @@
       <c r="A7" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="51" t="s">
         <v>407</v>
       </c>
-      <c r="C7" s="98" t="n">
+      <c r="C7" s="100" t="n">
         <v>30896493733.39</v>
       </c>
-      <c r="D7" s="99" t="n">
+      <c r="D7" s="101" t="n">
         <v>45870</v>
       </c>
     </row>
@@ -43160,13 +43168,13 @@
       <c r="A8" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="51" t="s">
         <v>407</v>
       </c>
-      <c r="C8" s="98" t="n">
+      <c r="C8" s="100" t="n">
         <v>33906772915.32</v>
       </c>
-      <c r="D8" s="99" t="n">
+      <c r="D8" s="101" t="n">
         <v>45870</v>
       </c>
     </row>
@@ -43174,13 +43182,13 @@
       <c r="A9" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="51" t="s">
         <v>406</v>
       </c>
-      <c r="C9" s="98" t="n">
+      <c r="C9" s="100" t="n">
         <v>1500000000</v>
       </c>
-      <c r="D9" s="99" t="n">
+      <c r="D9" s="101" t="n">
         <v>45839</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica 10/07/2026 16:36 (Buenos Aires)
</commit_message>
<xml_diff>
--- a/Master UOPs.xlsx
+++ b/Master UOPs.xlsx
@@ -3030,9 +3030,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>208080</xdr:colOff>
+      <xdr:colOff>207720</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>36000</xdr:rowOff>
+      <xdr:rowOff>35640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3047,7 +3047,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10472040" y="10696680"/>
-          <a:ext cx="4843440" cy="2045520"/>
+          <a:ext cx="4843080" cy="2045160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3069,9 +3069,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1492920</xdr:colOff>
+      <xdr:colOff>1492560</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>23040</xdr:rowOff>
+      <xdr:rowOff>22680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3086,7 +3086,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4453560" y="6731280"/>
-          <a:ext cx="6009480" cy="5997960"/>
+          <a:ext cx="6009120" cy="5997600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -41665,7 +41665,7 @@
         <v>358</v>
       </c>
       <c r="B5" s="57" t="n">
-        <v>0.252</v>
+        <v>0.2557</v>
       </c>
       <c r="C5" s="58" t="s">
         <v>359</v>
@@ -41688,7 +41688,7 @@
       </c>
       <c r="B7" s="61" t="n">
         <f aca="true">TODAY()</f>
-        <v>46207</v>
+        <v>46213</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="9.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -41751,22 +41751,22 @@
       </c>
       <c r="G10" s="63" t="n">
         <f aca="false">IF(F10="",MAX(0,$B$7-E10),MAX(0,F10-E10))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H10" s="67" t="n">
         <v>50402510.51</v>
       </c>
       <c r="I10" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J10" s="69" t="n">
         <f aca="false">H10*I10*(G10/365)</f>
-        <v>4361405.18341874</v>
+        <v>4655341.57758747</v>
       </c>
       <c r="K10" s="70" t="n">
         <f aca="false">H10+J10</f>
-        <v>54763915.6934187</v>
+        <v>55057852.0875875</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -41793,22 +41793,22 @@
       </c>
       <c r="G11" s="71" t="n">
         <f aca="false">IF(F11="",MAX(0,$B$7-E11),MAX(0,F11-E11))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H11" s="74" t="n">
         <v>677271.96</v>
       </c>
       <c r="I11" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J11" s="75" t="n">
         <f aca="false">H11*I11*(G11/365)</f>
-        <v>58605.3632455891</v>
+        <v>62555.0648731397</v>
       </c>
       <c r="K11" s="76" t="n">
         <f aca="false">H11+J11</f>
-        <v>735877.323245589</v>
+        <v>739827.02487314</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -41835,22 +41835,22 @@
       </c>
       <c r="G12" s="63" t="n">
         <f aca="false">IF(F12="",MAX(0,$B$7-E12),MAX(0,F12-E12))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H12" s="67" t="n">
         <v>17699825.4</v>
       </c>
       <c r="I12" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J12" s="69" t="n">
         <f aca="false">H12*I12*(G12/365)</f>
-        <v>1531592.56283178</v>
+        <v>1634814.06515079</v>
       </c>
       <c r="K12" s="70" t="n">
         <f aca="false">H12+J12</f>
-        <v>19231417.9628318</v>
+        <v>19334639.4651508</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -41877,22 +41877,22 @@
       </c>
       <c r="G13" s="71" t="n">
         <f aca="false">IF(F13="",MAX(0,$B$7-E13),MAX(0,F13-E13))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H13" s="74" t="n">
         <v>1015907.94</v>
       </c>
       <c r="I13" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J13" s="75" t="n">
         <f aca="false">H13*I13*(G13/365)</f>
-        <v>87908.0448683836</v>
+        <v>93832.5973097096</v>
       </c>
       <c r="K13" s="76" t="n">
         <f aca="false">H13+J13</f>
-        <v>1103815.98486838</v>
+        <v>1109740.53730971</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -41919,22 +41919,22 @@
       </c>
       <c r="G14" s="63" t="n">
         <f aca="false">IF(F14="",MAX(0,$B$7-E14),MAX(0,F14-E14))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H14" s="67" t="n">
         <v>27253875.19</v>
       </c>
       <c r="I14" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J14" s="69" t="n">
         <f aca="false">H14*I14*(G14/365)</f>
-        <v>2358318.88767386</v>
+        <v>2517257.51432985</v>
       </c>
       <c r="K14" s="70" t="n">
         <f aca="false">H14+J14</f>
-        <v>29612194.0776739</v>
+        <v>29771132.7043299</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -41961,22 +41961,22 @@
       </c>
       <c r="G15" s="71" t="n">
         <f aca="false">IF(F15="",MAX(0,$B$7-E15),MAX(0,F15-E15))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H15" s="74" t="n">
         <v>1015907.94</v>
       </c>
       <c r="I15" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J15" s="75" t="n">
         <f aca="false">H15*I15*(G15/365)</f>
-        <v>87908.0448683836</v>
+        <v>93832.5973097096</v>
       </c>
       <c r="K15" s="76" t="n">
         <f aca="false">H15+J15</f>
-        <v>1103815.98486838</v>
+        <v>1109740.53730971</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42003,22 +42003,22 @@
       </c>
       <c r="G16" s="63" t="n">
         <f aca="false">IF(F16="",MAX(0,$B$7-E16),MAX(0,F16-E16))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H16" s="67" t="n">
         <v>28627721.36</v>
       </c>
       <c r="I16" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J16" s="69" t="n">
         <f aca="false">H16*I16*(G16/365)</f>
-        <v>2477199.86694312</v>
+        <v>2644150.46334558</v>
       </c>
       <c r="K16" s="70" t="n">
         <f aca="false">H16+J16</f>
-        <v>31104921.2269431</v>
+        <v>31271871.8233456</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42045,22 +42045,22 @@
       </c>
       <c r="G17" s="71" t="n">
         <f aca="false">IF(F17="",MAX(0,$B$7-E17),MAX(0,F17-E17))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H17" s="74" t="n">
         <v>238400.46</v>
       </c>
       <c r="I17" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J17" s="75" t="n">
         <f aca="false">H17*I17*(G17/365)</f>
-        <v>20629.1510373699</v>
+        <v>22019.4502679342</v>
       </c>
       <c r="K17" s="76" t="n">
         <f aca="false">H17+J17</f>
-        <v>259029.61103737</v>
+        <v>260419.910267934</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42087,22 +42087,22 @@
       </c>
       <c r="G18" s="63" t="n">
         <f aca="false">IF(F18="",MAX(0,$B$7-E18),MAX(0,F18-E18))</f>
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H18" s="67" t="n">
         <v>6758414.64</v>
       </c>
       <c r="I18" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J18" s="69" t="n">
         <f aca="false">H18*I18*(G18/365)</f>
-        <v>584815.802711671</v>
+        <v>624229.395595792</v>
       </c>
       <c r="K18" s="70" t="n">
         <f aca="false">H18+J18</f>
-        <v>7343230.44271167</v>
+        <v>7382644.03559579</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42129,22 +42129,22 @@
       </c>
       <c r="G19" s="71" t="n">
         <f aca="false">IF(F19="",MAX(0,$B$7-E19),MAX(0,F19-E19))</f>
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H19" s="74" t="n">
         <v>444448.23</v>
       </c>
       <c r="I19" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J19" s="75" t="n">
         <f aca="false">H19*I19*(G19/365)</f>
-        <v>32964.6643357808</v>
+        <v>35484.5031499233</v>
       </c>
       <c r="K19" s="76" t="n">
         <f aca="false">H19+J19</f>
-        <v>477412.894335781</v>
+        <v>479932.733149923</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42171,22 +42171,22 @@
       </c>
       <c r="G20" s="63" t="n">
         <f aca="false">IF(F20="",MAX(0,$B$7-E20),MAX(0,F20-E20))</f>
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H20" s="67" t="n">
         <v>12832109.38</v>
       </c>
       <c r="I20" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J20" s="69" t="n">
         <f aca="false">H20*I20*(G20/365)</f>
-        <v>951755.794891397</v>
+        <v>1024508.58160639</v>
       </c>
       <c r="K20" s="70" t="n">
         <f aca="false">H20+J20</f>
-        <v>13783865.1748914</v>
+        <v>13856617.9616064</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42213,22 +42213,22 @@
       </c>
       <c r="G21" s="71" t="n">
         <f aca="false">IF(F21="",MAX(0,$B$7-E21),MAX(0,F21-E21))</f>
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="H21" s="74" t="n">
         <v>184056.25</v>
       </c>
       <c r="I21" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J21" s="75" t="n">
         <f aca="false">H21*I21*(G21/365)</f>
-        <v>12940.4150342466</v>
+        <v>13974.6094537671</v>
       </c>
       <c r="K21" s="76" t="n">
         <f aca="false">H21+J21</f>
-        <v>196996.665034247</v>
+        <v>198030.859453767</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42255,22 +42255,22 @@
       </c>
       <c r="G22" s="63" t="n">
         <f aca="false">IF(F22="",MAX(0,$B$7-E22),MAX(0,F22-E22))</f>
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="H22" s="67" t="n">
         <v>5425916.78</v>
       </c>
       <c r="I22" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J22" s="69" t="n">
         <f aca="false">H22*I22*(G22/365)</f>
-        <v>381479.113447562</v>
+        <v>411966.819540992</v>
       </c>
       <c r="K22" s="70" t="n">
         <f aca="false">H22+J22</f>
-        <v>5807395.89344756</v>
+        <v>5837883.59954099</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42297,14 +42297,14 @@
       </c>
       <c r="G23" s="71" t="n">
         <f aca="false">IF(F23="",MAX(0,$B$7-E23),MAX(0,F23-E23))</f>
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="H23" s="74" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J23" s="75" t="n">
         <f aca="false">H23*I23*(G23/365)</f>
@@ -42339,14 +42339,14 @@
       </c>
       <c r="G24" s="63" t="n">
         <f aca="false">IF(F24="",MAX(0,$B$7-E24),MAX(0,F24-E24))</f>
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="H24" s="67" t="n">
         <v>0</v>
       </c>
       <c r="I24" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J24" s="69" t="n">
         <f aca="false">H24*I24*(G24/365)</f>
@@ -42381,22 +42381,22 @@
       </c>
       <c r="G25" s="71" t="n">
         <f aca="false">IF(F25="",MAX(0,$B$7-E25),MAX(0,F25-E25))</f>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="H25" s="74" t="n">
         <v>203181.59</v>
       </c>
       <c r="I25" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J25" s="75" t="n">
         <f aca="false">H25*I25*(G25/365)</f>
-        <v>7691.95400169863</v>
+        <v>8747.1066149726</v>
       </c>
       <c r="K25" s="76" t="n">
         <f aca="false">H25+J25</f>
-        <v>210873.544001699</v>
+        <v>211928.696614973</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42423,14 +42423,14 @@
       </c>
       <c r="G26" s="63" t="n">
         <f aca="false">IF(F26="",MAX(0,$B$7-E26),MAX(0,F26-E26))</f>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="H26" s="67" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J26" s="69" t="n">
         <f aca="false">H26*I26*(G26/365)</f>
@@ -42465,22 +42465,22 @@
       </c>
       <c r="G27" s="71" t="n">
         <f aca="false">IF(F27="",MAX(0,$B$7-E27),MAX(0,F27-E27))</f>
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="H27" s="74" t="n">
         <v>6266255.63</v>
       </c>
       <c r="I27" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J27" s="75" t="n">
         <f aca="false">H27*I27*(G27/365)</f>
-        <v>237224.987110521</v>
+        <v>269766.596827411</v>
       </c>
       <c r="K27" s="76" t="n">
         <f aca="false">H27+J27</f>
-        <v>6503480.61711052</v>
+        <v>6536022.22682741</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42507,22 +42507,22 @@
       </c>
       <c r="G28" s="63" t="n">
         <f aca="false">IF(F28="",MAX(0,$B$7-E28),MAX(0,F28-E28))</f>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="H28" s="67" t="n">
         <v>633024.04</v>
       </c>
       <c r="I28" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J28" s="69" t="n">
         <f aca="false">H28*I28*(G28/365)</f>
-        <v>12226.902690411</v>
+        <v>15360.284972789</v>
       </c>
       <c r="K28" s="70" t="n">
         <f aca="false">H28+J28</f>
-        <v>645250.942690411</v>
+        <v>648384.324972789</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42549,22 +42549,22 @@
       </c>
       <c r="G29" s="71" t="n">
         <f aca="false">IF(F29="",MAX(0,$B$7-E29),MAX(0,F29-E29))</f>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="H29" s="74" t="n">
         <v>19702240.1</v>
       </c>
       <c r="I29" s="77" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J29" s="75" t="n">
         <f aca="false">H29*I29*(G29/365)</f>
-        <v>380550.117</v>
+        <v>478073.506558</v>
       </c>
       <c r="K29" s="76" t="n">
         <f aca="false">H29+J29</f>
-        <v>20082790.217</v>
+        <v>20180313.606558</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42591,22 +42591,22 @@
       </c>
       <c r="G30" s="63" t="n">
         <f aca="false">IF(F30="",MAX(0,$B$7-E30),MAX(0,F30-E30))</f>
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="H30" s="67" t="n">
         <v>95946.87</v>
       </c>
       <c r="I30" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J30" s="69" t="n">
         <f aca="false">H30*I30*(G30/365)</f>
-        <v>1853.22036575342</v>
+        <v>2328.14422884658</v>
       </c>
       <c r="K30" s="70" t="n">
         <f aca="false">H30+J30</f>
-        <v>97800.0903657534</v>
+        <v>98275.0142288466</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42633,22 +42633,22 @@
       </c>
       <c r="G31" s="63" t="n">
         <f aca="false">IF(F31="",MAX(0,$B$7-E31),MAX(0,F31-E31))</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H31" s="67" t="n">
         <v>131593300.43</v>
       </c>
       <c r="I31" s="68" t="n">
         <f aca="false">$B$5+3%</f>
-        <v>0.282</v>
+        <v>0.2857</v>
       </c>
       <c r="J31" s="69" t="n">
         <f aca="false">H31*I31*(G31/365)</f>
-        <v>508346.722209041</v>
+        <v>1133036.34318181</v>
       </c>
       <c r="K31" s="70" t="n">
         <f aca="false">H31+J31</f>
-        <v>132101647.152209</v>
+        <v>132726336.773182</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42662,7 +42662,7 @@
       <c r="F32" s="78"/>
       <c r="G32" s="79" t="n">
         <f aca="false">IF(COUNTA(F10:F31)&gt;0,AVERAGE(G10:G31),AVERAGE(G10:G31))</f>
-        <v>81.2727272727273</v>
+        <v>87.2727272727273</v>
       </c>
       <c r="H32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,H10:H31)</f>
@@ -42671,11 +42671,11 @@
       <c r="I32" s="78"/>
       <c r="J32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,J10:J31)</f>
-        <v>14095416.7986853</v>
+        <v>15741279.2219049</v>
       </c>
       <c r="K32" s="80" t="n">
         <f aca="false">SUBTOTAL(109,K10:K31)</f>
-        <v>325165731.498685</v>
+        <v>326811593.921905</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42698,7 +42698,7 @@
       </c>
       <c r="B36" s="82" t="n">
         <f aca="false">J32</f>
-        <v>14095416.7986853</v>
+        <v>15741279.2219049</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42707,7 +42707,7 @@
       </c>
       <c r="B37" s="84" t="n">
         <f aca="false">B35+B36</f>
-        <v>325165731.498685</v>
+        <v>326811593.921905</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -42725,7 +42725,7 @@
       </c>
       <c r="B39" s="86" t="n">
         <f aca="false">G32</f>
-        <v>81.2727272727273</v>
+        <v>87.2727272727273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>